<commit_message>
Actualizacion automatica del mapa (2026-02-24 14:38:03)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R114"/>
+  <dimension ref="A1:R117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5155,22 +5155,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7621</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10/20/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Quito 3832</t>
+          <t>SAENZ AV. 1204</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>810404273</t>
+          <t>810416653</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5212,14 +5212,14 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.420412</v>
+        <v>-58.416237</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.616726</v>
+        <v>-34.65477</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>ALM-C</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5241,22 +5241,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7556</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SAENZ AV. 1204</t>
+          <t>SANCHEZ DE LORIA 1923</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5271,12 +5271,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>810416653</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>cambiar</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5298,10 +5298,10 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.416237</v>
+        <v>-58.411426</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.65477</v>
+        <v>-34.633266</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5315,7 +5315,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5327,22 +5327,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>7556</t>
+          <t>7579</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1923</t>
+          <t>AGUIRRE 508</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -5357,12 +5357,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>810421912</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5377,21 +5377,21 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L58" t="n">
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.411426</v>
+        <v>-58.435731</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.633266</v>
+        <v>-34.597659</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5401,7 +5401,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5413,22 +5413,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>7579</t>
+          <t>7755</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/24/2025</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>AGUIRRE 508</t>
+          <t>Munich 1715</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5443,7 +5443,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>810421912</t>
+          <t>810447258</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5463,31 +5463,31 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L59" t="n">
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.435731</v>
+        <v>-58.453119</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.597659</v>
+        <v>-34.55489</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>BLO-C</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5499,27 +5499,27 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>7620</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10/24/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>QUITO 3954</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5529,12 +5529,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>810447247</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -5553,17 +5553,17 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.422216</v>
+        <v>-58.4018</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.616828</v>
+        <v>-34.590471</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>ALM-C</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5585,22 +5585,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>7755</t>
+          <t>7631</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10/24/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Munich 1715</t>
+          <t>CALVO, CARLOS 3762</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5615,7 +5615,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>810447258</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5642,24 +5642,24 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.453119</v>
+        <v>-58.418542</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.55489</v>
+        <v>-34.624609</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>BLO-C</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5671,7 +5671,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>5749</t>
+          <t>7630</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5681,17 +5681,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
+          <t>INDEPENDENCIA AV. 3690</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Pendiente de Traspaso PROPIO</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5701,12 +5701,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>810451588</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5716,7 +5716,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -5725,17 +5725,17 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.4018</v>
+        <v>-58.417821</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.590471</v>
+        <v>-34.621158</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5757,7 +5757,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>7631</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5767,12 +5767,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CALVO, CARLOS 3762</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5787,12 +5787,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5814,14 +5814,14 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.418542</v>
+        <v>-58.430613</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.624609</v>
+        <v>-34.608805</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -5831,7 +5831,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5843,7 +5843,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>7630</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5853,12 +5853,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 3690</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>810451588</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -5900,24 +5900,24 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.417821</v>
+        <v>-58.50161</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.621158</v>
+        <v>-34.647648</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -5929,22 +5929,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>7643</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>ACEVEDO 524</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5959,12 +5959,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>810458896</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5986,14 +5986,14 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.430613</v>
+        <v>-58.439164</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.608805</v>
+        <v>-34.597069</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -6003,7 +6003,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6015,22 +6015,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7665</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>ARAOZ 2313</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6045,12 +6045,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada y cable cortado</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -6072,24 +6072,24 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.50161</v>
+        <v>-58.417634</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.647648</v>
+        <v>-34.587439</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6101,7 +6101,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>7643</t>
+          <t>7683</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ACEVEDO 524</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1684</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6131,12 +6131,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>810458896</t>
+          <t>01230516</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>colocar columna para pedir traspaso de nodo</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -6158,14 +6158,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.439164</v>
+        <v>-58.402647</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.597069</v>
+        <v>-34.591114</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6187,27 +6187,27 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>7665</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ARAOZ 2313</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -6217,12 +6217,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Picada y cable cortado</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6232,22 +6232,22 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L68" t="n">
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.417634</v>
+        <v>-58.436262</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.587439</v>
+        <v>-34.600478</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -6261,7 +6261,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6273,22 +6273,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>7683</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1684</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6303,12 +6303,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>01230516</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>colocar columna para pedir traspaso de nodo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6318,7 +6318,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -6330,24 +6330,24 @@
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.402647</v>
+        <v>-58.48121</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.591114</v>
+        <v>-34.61126</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6359,22 +6359,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>7619</t>
+          <t>7719</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>QUITO 4180</t>
+          <t>CIUDAD DE LA PAZ 180</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6389,12 +6389,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>810471618</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R400 para traspaso</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -6416,14 +6416,14 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.425596</v>
+        <v>-58.440031</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.617038</v>
+        <v>-34.575409</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>ALM-C</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6445,27 +6445,27 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S01150217</t>
+          <t>7732</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Vera 311</t>
+          <t>LINIERS VIRREY 1142</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pendiente de Traspaso PROPIO</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -6475,12 +6475,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>01230602</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Traspasar Fuente</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6490,26 +6490,26 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L71" t="n">
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.436262</v>
+        <v>-58.413563</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.600478</v>
+        <v>-34.624645</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6531,22 +6531,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>7744</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/31/2025</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>NECOCHEA 369</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6561,12 +6561,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>01233359</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R200 para rtaspaso de nodo</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6576,7 +6576,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -6588,24 +6588,24 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.48121</v>
+        <v>-58.364132</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.61126</v>
+        <v>-34.628423</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>CON-F</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6617,22 +6617,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>7719</t>
+          <t xml:space="preserve">7829 </t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ 180</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6647,12 +6647,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Colocar R400 para traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -6674,14 +6674,14 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.440031</v>
+        <v>-58.460356</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.575409</v>
+        <v>-34.630793</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6703,22 +6703,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>7732</t>
+          <t>7780</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>11/4/2025</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1142</t>
+          <t>INDEPENDENCIA AV. 1654</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6733,12 +6733,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>810573618</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Columna picada e inclinada</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6760,14 +6760,14 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.413563</v>
+        <v>-58.389676</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.624645</v>
+        <v>-34.618127</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -6777,7 +6777,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>CEN-?</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6789,22 +6789,22 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>7744</t>
+          <t>7810</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10/31/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>NECOCHEA 369</t>
+          <t>GUTENBERG 3212</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6819,12 +6819,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>01233359</t>
+          <t>810651343</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Colocar R200 para rtaspaso de nodo</t>
+          <t>Cambiar columna y ver que el vano quede separado del balcon esta inclinada hacia la casa</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6834,7 +6834,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -6846,56 +6846,56 @@
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.364132</v>
+        <v>-58.501325</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.628423</v>
+        <v>-34.594325</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>CON-F</t>
+          <t>PUE-Q</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PUE</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">7829 </t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6905,12 +6905,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6932,24 +6932,24 @@
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.460356</v>
+        <v>-58.510994</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.630793</v>
+        <v>-34.655027</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6961,22 +6961,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>7604</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>11/4/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 1654</t>
+          <t>SAN JUAN AV. 3741</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6991,12 +6991,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>810573618</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Columna picada e inclinada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7018,14 +7018,14 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.389676</v>
+        <v>-58.418108</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.618127</v>
+        <v>-34.62564</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>CEN-?</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7047,22 +7047,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>7810</t>
+          <t>7764</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>GUTENBERG 3212</t>
+          <t>2 DE ABRIL DE 1982 6510</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7077,17 +7077,17 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>810651343</t>
+          <t>01411184</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Cambiar columna y ver que el vano quede separado del balcon esta inclinada hacia la casa</t>
+          <t>Desmontar poste en desuso</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -7097,63 +7097,63 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L78" t="n">
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.501325</v>
+        <v>-58.490261</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.594325</v>
+        <v>-34.677337</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>PUE-Q</t>
+          <t>PAV-M</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PUE</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>6415</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>CAMPICHUELO 215</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pendiente de Traspaso PROPIO</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -7163,12 +7163,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>810712875</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7190,24 +7190,24 @@
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.510994</v>
+        <v>-58.433771</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.655027</v>
+        <v>-34.614668</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7219,7 +7219,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>7604</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7229,12 +7229,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 3741</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7249,12 +7249,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7276,14 +7276,14 @@
         <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.418108</v>
+        <v>-58.433855</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.62564</v>
+        <v>-34.614487</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7305,22 +7305,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>7764</t>
+          <t>7842</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2 DE ABRIL DE 1982 6510</t>
+          <t>FERRARI 410</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7335,17 +7335,17 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>01411184</t>
+          <t>810713039</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Desmontar poste en desuso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -7355,31 +7355,31 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L81" t="n">
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.490261</v>
+        <v>-58.441198</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.677337</v>
+        <v>-34.605341</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>PAV-M</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7391,22 +7391,22 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>6415</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 215</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7421,12 +7421,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>810712875</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>columna inclinada base corroida</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -7448,14 +7448,14 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>-58.433771</v>
+        <v>-58.439239</v>
       </c>
       <c r="N82" t="n">
-        <v>-34.614668</v>
+        <v>-34.6604</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -7465,7 +7465,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7477,22 +7477,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>S01140678</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7507,12 +7507,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810804375</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>columna inclinada corroida</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -7534,14 +7534,14 @@
         <v>1</v>
       </c>
       <c r="M83" t="n">
-        <v>-58.433855</v>
+        <v>-58.388529</v>
       </c>
       <c r="N83" t="n">
-        <v>-34.614487</v>
+        <v>-34.655949</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
@@ -7551,7 +7551,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>CON-I</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7563,22 +7563,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>7842</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>FERRARI 410</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7593,12 +7593,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>810713039</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -7620,14 +7620,14 @@
         <v>1</v>
       </c>
       <c r="M84" t="n">
-        <v>-58.441198</v>
+        <v>-58.491325</v>
       </c>
       <c r="N84" t="n">
-        <v>-34.605341</v>
+        <v>-34.647761</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -7649,22 +7649,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t xml:space="preserve">7869 </t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7679,12 +7679,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>columna inclinada base corroida</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -7706,14 +7706,14 @@
         <v>1</v>
       </c>
       <c r="M85" t="n">
-        <v>-58.439239</v>
+        <v>-58.469394</v>
       </c>
       <c r="N85" t="n">
-        <v>-34.6604</v>
+        <v>-34.626925</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
@@ -7723,7 +7723,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7735,22 +7735,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>S01140678</t>
+          <t>7892</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>12/1/2025</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
+          <t>Juncal 1642</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -7765,12 +7765,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>810804375</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>columna inclinada corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -7792,14 +7792,14 @@
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>-58.388529</v>
+        <v>-58.390974</v>
       </c>
       <c r="N86" t="n">
-        <v>-34.655949</v>
+        <v>-34.594177</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>CON-I</t>
+          <t>RET-N</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -7821,22 +7821,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t xml:space="preserve">7898 </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>12/4/2025</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t>BONIFACIO, JOSE 2319</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -7851,12 +7851,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>810984687</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -7878,24 +7878,24 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.491325</v>
+        <v>-58.459955</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.647761</v>
+        <v>-34.631973</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7907,22 +7907,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">7869 </t>
+          <t>S01204545</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>12/10/2025</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>Medina 420</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7937,12 +7937,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -7964,51 +7964,51 @@
         <v>1</v>
       </c>
       <c r="M88" t="n">
-        <v>-58.469394</v>
+        <v>-58.48802</v>
       </c>
       <c r="N88" t="n">
-        <v>-34.626925</v>
+        <v>-34.641075</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>7892</t>
+          <t>8024</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>12/15/2025</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Juncal 1642</t>
+          <t>Cafayate 5230</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>811198624</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -8050,14 +8050,14 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.390974</v>
+        <v>-58.465491</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.594177</v>
+        <v>-34.687203</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>RET-N</t>
+          <t>PAV-T</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8079,22 +8079,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">7898 </t>
+          <t>7927</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12/4/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>BONIFACIO, JOSE 2319</t>
+          <t>Pico 3481</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -8109,12 +8109,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>810984687</t>
+          <t>811198751</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -8129,31 +8129,31 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L90" t="n">
         <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>-58.459955</v>
+        <v>-58.484883</v>
       </c>
       <c r="N90" t="n">
-        <v>-34.631973</v>
+        <v>-34.54464</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>COG-Q</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8165,22 +8165,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>S01204545</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12/10/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Medina 420</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -8195,12 +8195,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -8222,51 +8222,51 @@
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>-58.48802</v>
+        <v>-58.463198</v>
       </c>
       <c r="N91" t="n">
-        <v>-34.641075</v>
+        <v>-34.62624</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>8024</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12/15/2025</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Cafayate 5230</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -8281,12 +8281,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>811198624</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -8308,51 +8308,51 @@
         <v>1</v>
       </c>
       <c r="M92" t="n">
-        <v>-58.465491</v>
+        <v>-58.471183</v>
       </c>
       <c r="N92" t="n">
-        <v>-34.687203</v>
+        <v>-34.638988</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>PAV-T</t>
+          <t>PCH-O</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>7927</t>
+          <t xml:space="preserve">7997 </t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Pico 3481</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -8367,12 +8367,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>811198751</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -8387,31 +8387,31 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L93" t="n">
         <v>1</v>
       </c>
       <c r="M93" t="n">
-        <v>-58.484883</v>
+        <v>-58.46357</v>
       </c>
       <c r="N93" t="n">
-        <v>-34.54464</v>
+        <v>-34.623187</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>COG-Q</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8423,22 +8423,22 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t xml:space="preserve">8001 </t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t>CASTRO, EMILIO AV. 7650</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -8453,12 +8453,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>811299445</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -8473,31 +8473,31 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L94" t="n">
         <v>1</v>
       </c>
       <c r="M94" t="n">
-        <v>-58.463198</v>
+        <v>-58.524273</v>
       </c>
       <c r="N94" t="n">
-        <v>-34.62624</v>
+        <v>-34.65615</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8509,22 +8509,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t xml:space="preserve">8061 </t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t xml:space="preserve">FOREST AV. 957 </t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -8539,12 +8539,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>811453824</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -8559,21 +8559,21 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L95" t="n">
         <v>1</v>
       </c>
       <c r="M95" t="n">
-        <v>-58.471183</v>
+        <v>-58.45732</v>
       </c>
       <c r="N95" t="n">
-        <v>-34.638988</v>
+        <v>-34.581366</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
@@ -8583,29 +8583,29 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>PCH-O</t>
+          <t>ATH-N</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">7997 </t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8625,7 +8625,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -8652,10 +8652,10 @@
         <v>1</v>
       </c>
       <c r="M96" t="n">
-        <v>-58.46357</v>
+        <v>-58.459547</v>
       </c>
       <c r="N96" t="n">
-        <v>-34.623187</v>
+        <v>-34.626309</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -8669,7 +8669,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8681,22 +8681,22 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">8001 </t>
+          <t>8083</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>1/13/2026</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>CASTRO, EMILIO AV. 7650</t>
+          <t>USPALLATA 3625</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>811299445</t>
+          <t>811454350</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -8731,31 +8731,31 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L97" t="n">
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>-58.524273</v>
+        <v>-58.414313</v>
       </c>
       <c r="N97" t="n">
-        <v>-34.65615</v>
+        <v>-34.641194</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>PAV-I</t>
+          <t>PPT-G</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8767,22 +8767,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">8061 </t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">FOREST AV. 957 </t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -8797,12 +8797,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>811453824</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -8817,31 +8817,31 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L98" t="n">
         <v>1</v>
       </c>
       <c r="M98" t="n">
-        <v>-58.45732</v>
+        <v>-58.465166</v>
       </c>
       <c r="N98" t="n">
-        <v>-34.581366</v>
+        <v>-34.670435</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>ATH-N</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -8853,22 +8853,22 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t xml:space="preserve">8145 </t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>GUAMINI 5049</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -8883,12 +8883,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811498019</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t xml:space="preserve">corroida </t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -8910,10 +8910,10 @@
         <v>1</v>
       </c>
       <c r="M99" t="n">
-        <v>-58.459547</v>
+        <v>-58.475365</v>
       </c>
       <c r="N99" t="n">
-        <v>-34.626309</v>
+        <v>-34.688865</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -8927,7 +8927,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PAV-S</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8939,17 +8939,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>8083</t>
+          <t>8203</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>1/13/2026</t>
+          <t>1/23/2026</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>USPALLATA 3625</t>
+          <t xml:space="preserve">TRAFUL 3812 </t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8969,12 +8969,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>811454350</t>
+          <t>811498075</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -8996,14 +8996,14 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>-58.414313</v>
+        <v>-58.414437</v>
       </c>
       <c r="N100" t="n">
-        <v>-34.641194</v>
+        <v>-34.651882</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
@@ -9013,7 +9013,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>PPT-G</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9025,17 +9025,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -9055,12 +9055,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -9082,14 +9082,14 @@
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>-58.465166</v>
+        <v>-58.438399</v>
       </c>
       <c r="N101" t="n">
-        <v>-34.670435</v>
+        <v>-34.663958</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
@@ -9099,7 +9099,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9111,17 +9111,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">8145 </t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>1/16/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>GUAMINI 5049</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -9141,12 +9141,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>811498019</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t xml:space="preserve">corroida </t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -9168,10 +9168,10 @@
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>-58.475365</v>
+        <v>-58.475565</v>
       </c>
       <c r="N102" t="n">
-        <v>-34.688865</v>
+        <v>-34.660488</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>PAV-S</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9197,22 +9197,22 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>8203</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>1/23/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRAFUL 3812 </t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>811498075</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -9254,14 +9254,14 @@
         <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>-58.414437</v>
+        <v>-58.460855</v>
       </c>
       <c r="N103" t="n">
-        <v>-34.651882</v>
+        <v>-34.631046</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
@@ -9271,7 +9271,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9283,17 +9283,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -9313,12 +9313,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -9340,14 +9340,14 @@
         <v>1</v>
       </c>
       <c r="M104" t="n">
-        <v>-58.438399</v>
+        <v>-58.479751</v>
       </c>
       <c r="N104" t="n">
-        <v>-34.663958</v>
+        <v>-34.677211</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9369,22 +9369,22 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -9399,12 +9399,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -9426,51 +9426,51 @@
         <v>1</v>
       </c>
       <c r="M105" t="n">
-        <v>-58.475565</v>
+        <v>-58.491573</v>
       </c>
       <c r="N105" t="n">
-        <v>-34.660488</v>
+        <v>-34.639215</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -9512,36 +9512,36 @@
         <v>1</v>
       </c>
       <c r="M106" t="n">
-        <v>-58.460855</v>
+        <v>-58.487715</v>
       </c>
       <c r="N106" t="n">
-        <v>-34.631046</v>
+        <v>-34.636671</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t xml:space="preserve">8245 </t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9551,12 +9551,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t xml:space="preserve">ZELADA 4401 </t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -9571,7 +9571,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811626837</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -9598,51 +9598,51 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.479751</v>
+        <v>-58.488539</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.677211</v>
+        <v>-34.640962</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -9657,12 +9657,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -9684,51 +9684,51 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.491573</v>
+        <v>-58.481162</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.639215</v>
+        <v>-34.665875</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>-747</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -9743,12 +9743,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -9770,51 +9770,47 @@
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.487715</v>
+        <v>-58.413945</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.636671</v>
+        <v>-34.582774</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">8245 </t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>1/29/2026</t>
-        </is>
-      </c>
+          <t>S01421388</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADA 4401 </t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -9829,12 +9825,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>811626837</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -9853,49 +9849,49 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.488539</v>
+        <v>-58.437739</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.640962</v>
+        <v>-34.638224</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>8302</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>2/10/2026</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>LEGUIZAMON, MARTINIANO 3983</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9915,12 +9911,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -9935,17 +9931,17 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L111" t="n">
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.481162</v>
+        <v>-58.479051</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.665875</v>
+        <v>-34.675657</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -9971,18 +9967,22 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>S01421388</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr"/>
+          <t>8303</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2/10/2026</t>
+        </is>
+      </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t>LEGUIZAMON, MARTINIANO 3951</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -10002,7 +10002,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -10021,13 +10021,13 @@
         </is>
       </c>
       <c r="L112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.437739</v>
+        <v>-58.479542</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.638224</v>
+        <v>-34.675295</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -10041,7 +10041,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10053,22 +10053,22 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>8302</t>
+          <t>-759</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2/10/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>LEGUIZAMON, MARTINIANO 3983</t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -10088,7 +10088,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -10103,17 +10103,17 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L113" t="n">
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.479051</v>
+        <v>-58.469878</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.675657</v>
+        <v>-34.626919</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -10127,7 +10127,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10139,86 +10139,344 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>8303</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2/10/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>LEGUIZAMON, MARTINIANO 3951</t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>inclinada corroida</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>1</v>
+      </c>
+      <c r="M114" t="n">
+        <v>-58.46026</v>
+      </c>
+      <c r="N114" t="n">
+        <v>-34.640706</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>PPT-N</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>8268</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2/23/2026</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>MONTREAL 5391</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E115" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
         <is>
           <t>Pendiente ADM</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr">
+      <c r="H115" t="inlineStr">
         <is>
           <t>inclinada</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
+      <c r="I115" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="J115" t="inlineStr">
         <is>
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr">
+      <c r="K115" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L114" t="n">
-        <v>1</v>
-      </c>
-      <c r="M114" t="n">
-        <v>-58.479542</v>
-      </c>
-      <c r="N114" t="n">
-        <v>-34.675295</v>
-      </c>
-      <c r="O114" t="inlineStr">
+      <c r="L115" t="n">
+        <v>1</v>
+      </c>
+      <c r="M115" t="n">
+        <v>-58.480708</v>
+      </c>
+      <c r="N115" t="n">
+        <v>-34.667639</v>
+      </c>
+      <c r="O115" t="inlineStr">
         <is>
           <t>Boedo</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr">
+      <c r="P115" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q114" t="inlineStr">
+      <c r="Q115" t="inlineStr">
         <is>
           <t>PAV-Q</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr">
+      <c r="R115" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>8244</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2/23/2026</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZELADA 4401 </t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>1</v>
+      </c>
+      <c r="M116" t="n">
+        <v>-58.488539</v>
+      </c>
+      <c r="N116" t="n">
+        <v>-34.640962</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>PCH-S</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>S00936659</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2/23/2026</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" t="n">
+        <v>-58.474151</v>
+      </c>
+      <c r="N117" t="n">
+        <v>-34.630046</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>NRA-R</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2NRA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-10 12:20:46)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,96 +413,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R94"/>
+  <dimension ref="A1:R99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Caso</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>F. De Reclamo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Direccion</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Comuna</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>OT</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tipo de tarea</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Tipo de Elemento</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Attachments</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Coordenada_X</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Coordenada_Y</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Operacion</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>PD</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>N2</t>
         </is>
@@ -5069,7 +5057,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">7829 </t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5843,7 +5831,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">7869 </t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6015,7 +6003,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">7898 </t>
+          <t>7898</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -6441,7 +6429,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">7997 </t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -7645,7 +7633,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">8245 </t>
+          <t>8245</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7817,7 +7805,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>-747</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7985,7 +7973,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>-759</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -8493,6 +8481,432 @@
         </is>
       </c>
       <c r="R94" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>S00176142</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>3/6/2026</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CULPINA 533</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
+        <v>1</v>
+      </c>
+      <c r="M95" t="n">
+        <v>-58.464205</v>
+      </c>
+      <c r="N95" t="n">
+        <v>-34.636221</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>8554</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>3/9/2026</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>OLIDEN 55</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>columna inclinada</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>1</v>
+      </c>
+      <c r="M96" t="n">
+        <v>-58.517269</v>
+      </c>
+      <c r="N96" t="n">
+        <v>-34.639879</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>PAV-B</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>-772</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>3/10/2026</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>LA PLATA AV. 2304</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Desplazar Columna</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L97" t="n">
+        <v>1</v>
+      </c>
+      <c r="M97" t="n">
+        <v>-58.423086</v>
+      </c>
+      <c r="N97" t="n">
+        <v>-34.641356</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>PPT-L</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>-773</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>3/9/2026</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>LA PLATA AV. 2244</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>desmonte</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Desmonte</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>1</v>
+      </c>
+      <c r="M98" t="n">
+        <v>-58.423288</v>
+      </c>
+      <c r="N98" t="n">
+        <v>-34.640581</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>PPT-L</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>-774</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>3/9/2026</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CASEROS AV. 4131</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>mover a 4111</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L99" t="n">
+        <v>1</v>
+      </c>
+      <c r="M99" t="n">
+        <v>-58.422741</v>
+      </c>
+      <c r="N99" t="n">
+        <v>-34.639999</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>PPT-L</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-11 15:32:40)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R72"/>
+  <dimension ref="A1:R74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1887,27 +1887,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>7260</t>
+          <t>5894</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9/10/2025</t>
+          <t>5/27/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vidal 1861</t>
+          <t>ALBARELLOS AV. 3100</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Transito</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1917,17 +1917,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>809642175</t>
+          <t>ICD30340076</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>QAP fotos del gcba tenia las incorrectas</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Tensor</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1937,21 +1937,21 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.458298</v>
+        <v>-58.512533</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.566511</v>
+        <v>-34.579243</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>COG-F</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1973,22 +1973,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6475</t>
+          <t>7260</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9/17/2025</t>
+          <t>9/10/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Av Amancio Alcorta 3570</t>
+          <t>Vidal 1861</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>809800213</t>
+          <t>809642175</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>aplomar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2023,31 +2023,31 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.409278</v>
+        <v>-58.458298</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.653566</v>
+        <v>-34.566511</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>COG-F</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6182</t>
+          <t>6475</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Los Patos 2702</t>
+          <t>Av Amancio Alcorta 3570</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2089,17 +2089,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>809818308</t>
+          <t>809800213</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
+          <t>aplomar</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2109,17 +2109,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.399262</v>
+        <v>-58.409278</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.639685</v>
+        <v>-34.653566</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PPT-K</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2145,22 +2145,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7373</t>
+          <t>6182</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10/2/2025</t>
+          <t>9/17/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SANTIAGO DEL ESTERO 1253</t>
+          <t>Los Patos 2702</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>810132493</t>
+          <t>809818308</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2202,10 +2202,10 @@
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.384406</v>
+        <v>-58.399262</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.622932</v>
+        <v>-34.639685</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>CON-M</t>
+          <t>PPT-K</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2231,22 +2231,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>7373</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/13/2025</t>
+          <t>10/2/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>SANTIAGO DEL ESTERO 1253</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>810333018</t>
+          <t>810132493</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2288,14 +2288,14 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.46138</v>
+        <v>-58.384406</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.629774</v>
+        <v>-34.622932</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>CON-M</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2317,17 +2317,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7516</t>
+          <t>7595</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/13/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ALVAREZ, CRISOSTOMO 3000</t>
+          <t>FALCON, RAMON L.,CNEL. 2353</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>810333018</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2374,10 +2374,10 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.458516</v>
+        <v>-58.46138</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.646422</v>
+        <v>-34.629774</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2403,7 +2403,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7735</t>
+          <t>7516</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2413,12 +2413,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GARCIA, MARTIN AV. 772</t>
+          <t>ALVAREZ, CRISOSTOMO 3000</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810371042</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2460,14 +2460,14 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.374086</v>
+        <v>-58.458516</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.633168</v>
+        <v>-34.646422</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2477,29 +2477,29 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CON-B</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>ARATO-25058.AF.1CON</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7735</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SAENZ AV. 1204</t>
+          <t>GARCIA, MARTIN AV. 772</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>810416653</t>
+          <t>810371042</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2546,10 +2546,10 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.416237</v>
+        <v>-58.374086</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.65477</v>
+        <v>-34.633168</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2563,34 +2563,34 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>CON-B</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.AF.1CON</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7556</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1923</t>
+          <t>SAENZ AV. 1204</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2605,12 +2605,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>810416653</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2632,10 +2632,10 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.411426</v>
+        <v>-58.416237</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.633266</v>
+        <v>-34.65477</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2661,22 +2661,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7579</t>
+          <t>7556</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AGUIRRE 508</t>
+          <t>SANCHEZ DE LORIA 1923</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2691,12 +2691,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>810421912</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>cambiar</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2711,21 +2711,21 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.435731</v>
+        <v>-58.411426</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.597659</v>
+        <v>-34.633266</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2747,22 +2747,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7631</t>
+          <t>7579</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CALVO, CARLOS 3762</t>
+          <t>AGUIRRE 508</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>810421912</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2797,21 +2797,21 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.418542</v>
+        <v>-58.435731</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.624609</v>
+        <v>-34.597659</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2833,7 +2833,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>7631</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2843,12 +2843,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>CALVO, CARLOS 3762</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2890,14 +2890,14 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.430613</v>
+        <v>-58.418542</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.608805</v>
+        <v>-34.624609</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2919,7 +2919,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2929,12 +2929,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2976,24 +2976,24 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.50161</v>
+        <v>-58.430613</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.647648</v>
+        <v>-34.608805</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3005,22 +3005,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7643</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ACEVEDO 524</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>810458896</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3062,24 +3062,24 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.439164</v>
+        <v>-58.50161</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.597069</v>
+        <v>-34.647648</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3091,7 +3091,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7665</t>
+          <t>7643</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3101,12 +3101,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ARAOZ 2313</t>
+          <t>ACEVEDO 524</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>810458896</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Picada y cable cortado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3148,10 +3148,10 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.417634</v>
+        <v>-58.439164</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.587439</v>
+        <v>-34.597069</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3165,7 +3165,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3177,22 +3177,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>7665</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>ARAOZ 2313</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3207,12 +3207,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada y cable cortado</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3234,24 +3234,24 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.48121</v>
+        <v>-58.417634</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.61126</v>
+        <v>-34.587439</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3263,7 +3263,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7719</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3273,12 +3273,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ 180</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Colocar R400 para traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3320,24 +3320,24 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.440031</v>
+        <v>-58.48121</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.575409</v>
+        <v>-34.61126</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3349,7 +3349,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7732</t>
+          <t>7719</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3359,12 +3359,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1142</t>
+          <t>CIUDAD DE LA PAZ 180</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R400 para traspaso</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3406,14 +3406,14 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.413563</v>
+        <v>-58.440031</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.624645</v>
+        <v>-34.575409</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3435,22 +3435,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7744</t>
+          <t>7732</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/31/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>NECOCHEA 369</t>
+          <t>LINIERS VIRREY 1142</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>01233359</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Colocar R200 para rtaspaso de nodo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3492,14 +3492,14 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.364132</v>
+        <v>-58.413563</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.628423</v>
+        <v>-34.624645</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>CON-F</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3521,22 +3521,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7829</t>
+          <t>7744</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>10/31/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>NECOCHEA 369</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3551,12 +3551,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>01233359</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R200 para rtaspaso de nodo</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3578,14 +3578,14 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.460356</v>
+        <v>-58.364132</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.630793</v>
+        <v>-34.628423</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>CON-F</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3607,22 +3607,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>11/4/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 1654</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>810573618</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Columna picada e inclinada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3664,14 +3664,14 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.389676</v>
+        <v>-58.460356</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.618127</v>
+        <v>-34.630793</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>CEN-?</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3693,22 +3693,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7604</t>
+          <t>7780</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/4/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 3741</t>
+          <t>INDEPENDENCIA AV. 1654</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>810573618</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Columna picada e inclinada</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3750,14 +3750,14 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.418108</v>
+        <v>-58.389676</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.62564</v>
+        <v>-34.618127</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>CEN-?</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3779,7 +3779,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>7604</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3789,12 +3789,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t>SAN JUAN AV. 3741</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3836,14 +3836,14 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.433855</v>
+        <v>-58.418108</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.614487</v>
+        <v>-34.62564</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3865,22 +3865,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7842</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FERRARI 410</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810713039</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3922,24 +3922,24 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.441198</v>
+        <v>-58.433855</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.605341</v>
+        <v>-34.614487</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3951,22 +3951,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t>7842</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t>FERRARI 410</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810713039</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>columna inclinada base corroida</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4008,24 +4008,24 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.439239</v>
+        <v>-58.441198</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.6604</v>
+        <v>-34.605341</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S01140678</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4047,12 +4047,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810804375</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>columna inclinada corroida</t>
+          <t>columna inclinada base corroida</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4094,10 +4094,10 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.388529</v>
+        <v>-58.439239</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.655949</v>
+        <v>-34.6604</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>CON-I</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4123,22 +4123,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t>S01140678</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>810804375</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>columna inclinada corroida</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4180,24 +4180,24 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.491325</v>
+        <v>-58.388529</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.647761</v>
+        <v>-34.655949</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>CON-I</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4209,7 +4209,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4219,12 +4219,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4266,24 +4266,24 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.469394</v>
+        <v>-58.491325</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.626925</v>
+        <v>-34.647761</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4295,22 +4295,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>7892</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Juncal 1642</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4325,12 +4325,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4340,7 +4340,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -4352,14 +4352,14 @@
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.390974</v>
+        <v>-58.469394</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.594177</v>
+        <v>-34.626925</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>RET-N</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4381,22 +4381,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7898</t>
+          <t>7892</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>12/4/2025</t>
+          <t>12/1/2025</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BONIFACIO, JOSE 2319</t>
+          <t>Juncal 1642</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>810984687</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -4438,14 +4438,14 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.459955</v>
+        <v>-58.390974</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.631973</v>
+        <v>-34.594177</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>RET-N</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4467,22 +4467,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S01204545</t>
+          <t>7898</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>12/10/2025</t>
+          <t>12/4/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Medina 420</t>
+          <t>BONIFACIO, JOSE 2319</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4497,12 +4497,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t>810984687</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4524,51 +4524,51 @@
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.48802</v>
+        <v>-58.459955</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.641075</v>
+        <v>-34.631973</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t>S01204545</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>12/10/2025</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t>Medina 420</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4583,12 +4583,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4610,51 +4610,51 @@
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.463198</v>
+        <v>-58.48802</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.62624</v>
+        <v>-34.641075</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4669,12 +4669,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4696,47 +4696,51 @@
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.471183</v>
+        <v>-58.463198</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.638988</v>
+        <v>-34.62624</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R50" t="inlineStr"/>
+          <t>NRA-E</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>7997</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4751,7 +4755,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4778,51 +4782,47 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.46357</v>
+        <v>-58.471183</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.623187</v>
+        <v>-34.638988</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>NRA-E</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>8061</t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>FOREST AV. 957</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4837,12 +4837,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811453824</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4857,31 +4857,31 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.45732</v>
+        <v>-58.46357</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.581366</v>
+        <v>-34.623187</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>ATH-N</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4893,22 +4893,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>8061</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>FOREST AV. 957</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4923,12 +4923,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811453824</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4943,31 +4943,31 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.459547</v>
+        <v>-58.45732</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.626309</v>
+        <v>-34.581366</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>ATH-N</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4979,22 +4979,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5036,10 +5036,10 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.465166</v>
+        <v>-58.459547</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.670435</v>
+        <v>-34.626309</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5065,17 +5065,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5095,12 +5095,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5122,14 +5122,14 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.438399</v>
+        <v>-58.465166</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.663958</v>
+        <v>-34.670435</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5151,7 +5151,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5181,12 +5181,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5208,14 +5208,14 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.475565</v>
+        <v>-58.438399</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.660488</v>
+        <v>-34.663958</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5237,22 +5237,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5294,10 +5294,10 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.460855</v>
+        <v>-58.475565</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.631046</v>
+        <v>-34.660488</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5323,22 +5323,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -5353,12 +5353,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5380,10 +5380,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.479751</v>
+        <v>-58.460855</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.677211</v>
+        <v>-34.631046</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5409,7 +5409,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5419,12 +5419,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5466,36 +5466,36 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.491573</v>
+        <v>-58.479751</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.639215</v>
+        <v>-34.677211</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5525,12 +5525,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5552,10 +5552,10 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.487715</v>
+        <v>-58.491573</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.636671</v>
+        <v>-34.639215</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5581,7 +5581,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>8245</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADA 4401 </t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811626837</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5638,10 +5638,10 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.488539</v>
+        <v>-58.487715</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.640962</v>
+        <v>-34.636671</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5667,22 +5667,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>8245</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t xml:space="preserve">ZELADA 4401 </t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5697,12 +5697,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>811626837</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5724,51 +5724,51 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.481162</v>
+        <v>-58.488539</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.665875</v>
+        <v>-34.640962</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>8490</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Ugarteche 2816</t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>corroida inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5810,14 +5810,14 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.413945</v>
+        <v>-58.481162</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.582774</v>
+        <v>-34.665875</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>AGU-M</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5839,7 +5839,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5849,12 +5849,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5896,14 +5896,14 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.437739</v>
+        <v>-58.413945</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.638224</v>
+        <v>-34.582774</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -5925,17 +5925,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -5955,12 +5955,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5982,10 +5982,10 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.469878</v>
+        <v>-58.437739</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.626919</v>
+        <v>-34.638224</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5999,7 +5999,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6011,22 +6011,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>900009468810</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t xml:space="preserve">CUENCA 3033 </t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6061,31 +6061,31 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L66" t="n">
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.46026</v>
+        <v>-58.494814</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.640706</v>
+        <v>-34.601905</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>DEV-B</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6097,7 +6097,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6107,12 +6107,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6154,10 +6154,10 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.480708</v>
+        <v>-58.469878</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.667639</v>
+        <v>-34.626919</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6183,22 +6183,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>8244</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADA 4401 </t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>812440296</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6240,36 +6240,36 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.488539</v>
+        <v>-58.46026</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.640962</v>
+        <v>-34.640706</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6279,12 +6279,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6299,7 +6299,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -6326,36 +6326,36 @@
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.474151</v>
+        <v>-58.480708</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.630046</v>
+        <v>-34.667639</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NRA-R</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>8244</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -6365,12 +6365,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t xml:space="preserve">ZELADA 4401 </t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440296</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>inclinada base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6400,58 +6400,58 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L70" t="n">
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.464382</v>
+        <v>-58.488539</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.683083</v>
+        <v>-34.640962</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6471,12 +6471,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6486,7 +6486,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -6498,109 +6498,281 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.464205</v>
+        <v>-58.474151</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.636221</v>
+        <v>-34.630046</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R71" t="inlineStr"/>
+          <t>NRA-R</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2NRA</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>S00552343</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2/23/2026</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>inclinada base corroida</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>1</v>
+      </c>
+      <c r="M72" t="n">
+        <v>-58.464382</v>
+      </c>
+      <c r="N72" t="n">
+        <v>-34.683083</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>S00176142</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>3/6/2026</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CULPINA 533</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>1</v>
+      </c>
+      <c r="M73" t="n">
+        <v>-58.464205</v>
+      </c>
+      <c r="N73" t="n">
+        <v>-34.636221</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>8554</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>3/9/2026</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>OLIDEN 55</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
         <is>
           <t>Pendiente ADM</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>columna inclinada</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="J74" t="inlineStr">
         <is>
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="K74" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="L72" t="n">
-        <v>1</v>
-      </c>
-      <c r="M72" t="n">
+      <c r="L74" t="n">
+        <v>1</v>
+      </c>
+      <c r="M74" t="n">
         <v>-58.517269</v>
       </c>
-      <c r="N72" t="n">
+      <c r="N74" t="n">
         <v>-34.639879</v>
       </c>
-      <c r="O72" t="inlineStr">
+      <c r="O74" t="inlineStr">
         <is>
           <t>Devoto</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr">
+      <c r="P74" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q72" t="inlineStr">
+      <c r="Q74" t="inlineStr">
         <is>
           <t>PAV-B</t>
         </is>
       </c>
-      <c r="R72" t="inlineStr">
+      <c r="R74" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-18 10:10:21)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1371,22 +1371,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6180</t>
+          <t>5839</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5/4/2025</t>
+          <t>5/19/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AZARA 15</t>
+          <t>AYACUCHO 267</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1401,12 +1401,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>805655333</t>
+          <t>806926385</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Picada entro tambien como reclamo 7611</t>
+          <t>Colocar columna y dar aviso para traspaso de nodo teco</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1428,14 +1428,14 @@
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>-58.372751</v>
+        <v>-58.395063</v>
       </c>
       <c r="N12" t="n">
-        <v>-34.631917</v>
+        <v>-34.606257</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1445,34 +1445,34 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>CON-B</t>
+          <t>CLI-B</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>ARATO-25058.AF.1CON</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5839</t>
+          <t>5935</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5/19/2025</t>
+          <t>5/27/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AYACUCHO 267</t>
+          <t>ALVAREZ THOMAS AV. 3305</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1487,51 +1487,51 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>806926385</t>
+          <t>807044131</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Colocar columna y dar aviso para traspaso de nodo teco</t>
+          <t>Columna inclinada</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L13" t="n">
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>-58.395063</v>
+        <v>-58.483927</v>
       </c>
       <c r="N13" t="n">
-        <v>-34.606257</v>
+        <v>-34.570689</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>CLI-B</t>
+          <t>PUE-E</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1543,22 +1543,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5935</t>
+          <t>5948</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>5/27/2025</t>
+          <t>6/2/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ALVAREZ THOMAS AV. 3305</t>
+          <t>MURGUIONDO 3990</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1573,17 +1573,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>807044131</t>
+          <t>807129347</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Columna inclinada</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1600,24 +1600,24 @@
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>-58.483927</v>
+        <v>-58.477944</v>
       </c>
       <c r="N14" t="n">
-        <v>-34.570689</v>
+        <v>-34.675149</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>PUE-E</t>
+          <t>PAV-V</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1629,22 +1629,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5948</t>
+          <t>6010</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6/2/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MURGUIONDO 3990</t>
+          <t>ESTADO DE PALESTINA 771</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1659,12 +1659,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>807129347</t>
+          <t>807215458</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>Picada y mal ubicada ver con Pedro</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1679,21 +1679,21 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>-58.477944</v>
+        <v>-58.425478</v>
       </c>
       <c r="N15" t="n">
-        <v>-34.675149</v>
+        <v>-34.601865</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>PAV-V</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1715,22 +1715,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6010</t>
+          <t>6075</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>6/9/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ESTADO DE PALESTINA 771</t>
+          <t>ALBERTI 191</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1745,12 +1745,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>807215458</t>
+          <t>810533286</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Picada y mal ubicada ver con Pedro</t>
+          <t>Desmontar PRFV 400</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1772,10 +1772,10 @@
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>-58.425478</v>
+        <v>-58.401624</v>
       </c>
       <c r="N16" t="n">
-        <v>-34.601865</v>
+        <v>-34.612001</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1801,22 +1801,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6075</t>
+          <t>7260</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>6/9/2025</t>
+          <t>9/10/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ALBERTI 191</t>
+          <t>Vidal 1861</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1831,12 +1831,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>810533286</t>
+          <t>809642175</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Desmontar PRFV 400</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1858,24 +1858,24 @@
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.401624</v>
+        <v>-58.458298</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.612001</v>
+        <v>-34.566511</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>COG-F</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1887,27 +1887,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5894</t>
+          <t>6475</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5/27/2025</t>
+          <t>9/17/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ALBARELLOS AV. 3100</t>
+          <t>Av Amancio Alcorta 3570</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pendiente de Transito</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1917,17 +1917,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>ICD30340076</t>
+          <t>809800213</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>QAP fotos del gcba tenia las incorrectas</t>
+          <t>aplomar</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Tensor</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1941,27 +1941,27 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.512533</v>
+        <v>-58.409278</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.579243</v>
+        <v>-34.653566</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1973,22 +1973,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>7260</t>
+          <t>6182</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9/10/2025</t>
+          <t>9/17/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Vidal 1861</t>
+          <t>Los Patos 2702</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2003,12 +2003,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>809642175</t>
+          <t>809818308</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2030,24 +2030,24 @@
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.458298</v>
+        <v>-58.399262</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.566511</v>
+        <v>-34.639685</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>COG-F</t>
+          <t>PPT-K</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2059,22 +2059,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6475</t>
+          <t>7373</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>9/17/2025</t>
+          <t>10/2/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Av Amancio Alcorta 3570</t>
+          <t>SANTIAGO DEL ESTERO 1253</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2089,17 +2089,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>809800213</t>
+          <t>810132493</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>aplomar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2109,17 +2109,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.409278</v>
+        <v>-58.384406</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.653566</v>
+        <v>-34.622932</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>CON-M</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2145,22 +2145,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6182</t>
+          <t>7595</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>9/17/2025</t>
+          <t>10/13/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Los Patos 2702</t>
+          <t>FALCON, RAMON L.,CNEL. 2353</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>809818308</t>
+          <t>810333018</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2202,14 +2202,14 @@
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.399262</v>
+        <v>-58.46138</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.639685</v>
+        <v>-34.629774</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PPT-K</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2231,22 +2231,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7373</t>
+          <t>7516</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/2/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SANTIAGO DEL ESTERO 1253</t>
+          <t>ALVAREZ, CRISOSTOMO 3000</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>810132493</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2288,14 +2288,14 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.384406</v>
+        <v>-58.458516</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.622932</v>
+        <v>-34.646422</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>CON-M</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2317,22 +2317,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>7735</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10/13/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>GARCIA, MARTIN AV. 772</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>810333018</t>
+          <t>810371042</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2374,14 +2374,14 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.46138</v>
+        <v>-58.374086</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.629774</v>
+        <v>-34.633168</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2391,34 +2391,34 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>CON-B</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.AF.1CON</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7516</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ALVAREZ, CRISOSTOMO 3000</t>
+          <t>SAENZ AV. 1204</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>810416653</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2460,14 +2460,14 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.458516</v>
+        <v>-58.416237</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.646422</v>
+        <v>-34.65477</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2489,22 +2489,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7735</t>
+          <t>7556</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GARCIA, MARTIN AV. 772</t>
+          <t>SANCHEZ DE LORIA 1923</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2519,12 +2519,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>810371042</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>cambiar</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2546,10 +2546,10 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.374086</v>
+        <v>-58.411426</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.633168</v>
+        <v>-34.633266</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2563,19 +2563,19 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>CON-B</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>ARATO-25058.AF.1CON</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7579</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2585,12 +2585,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SAENZ AV. 1204</t>
+          <t>AGUIRRE 508</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>810416653</t>
+          <t>810421912</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2625,21 +2625,21 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.416237</v>
+        <v>-58.435731</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.65477</v>
+        <v>-34.597659</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2661,17 +2661,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7556</t>
+          <t>7631</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1923</t>
+          <t>CALVO, CARLOS 3762</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2691,12 +2691,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2718,14 +2718,14 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.411426</v>
+        <v>-58.418542</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.633266</v>
+        <v>-34.624609</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2747,22 +2747,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7579</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AGUIRRE 508</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>810421912</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2797,21 +2797,21 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.435731</v>
+        <v>-58.430613</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.597659</v>
+        <v>-34.608805</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2833,7 +2833,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7631</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2843,12 +2843,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CALVO, CARLOS 3762</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2890,24 +2890,24 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.418542</v>
+        <v>-58.50161</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.624609</v>
+        <v>-34.647648</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2919,22 +2919,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>7643</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>ACEVEDO 524</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>810458896</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2976,14 +2976,14 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.430613</v>
+        <v>-58.439164</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.608805</v>
+        <v>-34.597069</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3005,22 +3005,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7665</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>ARAOZ 2313</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada y cable cortado</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3062,24 +3062,24 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.50161</v>
+        <v>-58.417634</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.647648</v>
+        <v>-34.587439</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3091,22 +3091,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7643</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ACEVEDO 524</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>810458896</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3148,24 +3148,24 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.439164</v>
+        <v>-58.48121</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.597069</v>
+        <v>-34.61126</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3177,17 +3177,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7665</t>
+          <t>7719</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ARAOZ 2313</t>
+          <t>CIUDAD DE LA PAZ 180</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3207,12 +3207,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Picada y cable cortado</t>
+          <t>Colocar R400 para traspaso</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.417634</v>
+        <v>-58.440031</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.587439</v>
+        <v>-34.575409</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3263,7 +3263,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>7732</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3273,12 +3273,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>LINIERS VIRREY 1142</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3293,7 +3293,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3320,24 +3320,24 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.48121</v>
+        <v>-58.413563</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.61126</v>
+        <v>-34.624645</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3349,22 +3349,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7719</t>
+          <t>7744</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/31/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ 180</t>
+          <t>NECOCHEA 369</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>01233359</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Colocar R400 para traspaso</t>
+          <t>Colocar R200 para rtaspaso de nodo</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3406,14 +3406,14 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.440031</v>
+        <v>-58.364132</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.575409</v>
+        <v>-34.628423</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>CON-F</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3435,22 +3435,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7732</t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1142</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3492,10 +3492,10 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.413563</v>
+        <v>-58.460356</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.624645</v>
+        <v>-34.630793</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3521,22 +3521,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7744</t>
+          <t>7780</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10/31/2025</t>
+          <t>11/4/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NECOCHEA 369</t>
+          <t>INDEPENDENCIA AV. 1654</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3551,12 +3551,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>01233359</t>
+          <t>810573618</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Colocar R200 para rtaspaso de nodo</t>
+          <t>Columna picada e inclinada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3578,10 +3578,10 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.364132</v>
+        <v>-58.389676</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.628423</v>
+        <v>-34.618127</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>CON-F</t>
+          <t>CEN-?</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3607,22 +3607,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7829</t>
+          <t>7604</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>SAN JUAN AV. 3741</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3664,10 +3664,10 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.460356</v>
+        <v>-58.418108</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.630793</v>
+        <v>-34.62564</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3693,22 +3693,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11/4/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 1654</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>810573618</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Columna picada e inclinada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3750,14 +3750,14 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.389676</v>
+        <v>-58.433855</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.618127</v>
+        <v>-34.614487</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>CEN-?</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3779,22 +3779,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7604</t>
+          <t>7842</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 3741</t>
+          <t>FERRARI 410</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>810713039</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3836,24 +3836,24 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.418108</v>
+        <v>-58.441198</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.62564</v>
+        <v>-34.605341</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3865,22 +3865,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>columna inclinada base corroida</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3922,14 +3922,14 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.433855</v>
+        <v>-58.439239</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.614487</v>
+        <v>-34.6604</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3951,22 +3951,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>7842</t>
+          <t>S01140678</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FERRARI 410</t>
+          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810713039</t>
+          <t>810804375</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>columna inclinada corroida</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4008,24 +4008,24 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.441198</v>
+        <v>-58.388529</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.605341</v>
+        <v>-34.655949</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>CON-I</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4037,22 +4037,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>columna inclinada base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4094,24 +4094,24 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.439239</v>
+        <v>-58.491325</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.6604</v>
+        <v>-34.647761</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4123,22 +4123,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S01140678</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>810804375</t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>columna inclinada corroida</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4180,14 +4180,14 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.388529</v>
+        <v>-58.469394</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.655949</v>
+        <v>-34.626925</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>CON-I</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4209,22 +4209,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t>7892</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>12/1/2025</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t>Juncal 1642</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -4266,24 +4266,24 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.491325</v>
+        <v>-58.390974</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.647761</v>
+        <v>-34.594177</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>RET-N</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4295,22 +4295,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>7961</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>12/2/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>CASTILLO 12</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4325,12 +4325,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>810984643</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4345,21 +4345,21 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.469394</v>
+        <v>-58.430396</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.626925</v>
+        <v>-34.599668</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4381,22 +4381,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7892</t>
+          <t>7898</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>12/4/2025</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Juncal 1642</t>
+          <t>BONIFACIO, JOSE 2319</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>810984687</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -4438,14 +4438,14 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.390974</v>
+        <v>-58.459955</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.594177</v>
+        <v>-34.631973</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>RET-N</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4467,22 +4467,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7961</t>
+          <t>S01204545</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>12/2/2025</t>
+          <t>12/10/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CASTILLO 12</t>
+          <t>Medina 420</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4497,12 +4497,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>810984643</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4517,53 +4517,53 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.430396</v>
+        <v>-58.48802</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.599668</v>
+        <v>-34.641075</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7898</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12/4/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BONIFACIO, JOSE 2319</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -4583,12 +4583,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>810984687</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4610,10 +4610,10 @@
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.459955</v>
+        <v>-58.463198</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.631973</v>
+        <v>-34.62624</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4639,22 +4639,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S01204545</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>12/10/2025</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Medina 420</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4669,12 +4669,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4696,10 +4696,10 @@
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.48802</v>
+        <v>-58.471183</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.641075</v>
+        <v>-34.638988</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -4713,29 +4713,25 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PCH-S</t>
-        </is>
-      </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>ARATO-25058.PO.2PCH</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4755,12 +4751,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4782,10 +4778,10 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.463198</v>
+        <v>-58.46357</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.62624</v>
+        <v>-34.623187</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -4811,22 +4807,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t>8061</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t>FOREST AV. 957</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4841,12 +4837,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>811453824</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4861,21 +4857,21 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.471183</v>
+        <v>-58.45732</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.638988</v>
+        <v>-34.581366</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -4885,25 +4881,29 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr"/>
+          <t>ATH-N</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>7997</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4950,10 +4950,10 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.46357</v>
+        <v>-58.459547</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.623187</v>
+        <v>-34.626309</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4967,7 +4967,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4979,22 +4979,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>8061</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>FOREST AV. 957</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>811453824</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5029,31 +5029,31 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.45732</v>
+        <v>-58.465166</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.581366</v>
+        <v>-34.670435</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>ATH-N</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5065,22 +5065,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5095,12 +5095,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5122,14 +5122,14 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.459547</v>
+        <v>-58.438399</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.626309</v>
+        <v>-34.663958</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5151,17 +5151,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5181,12 +5181,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5208,10 +5208,10 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.465166</v>
+        <v>-58.475565</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.670435</v>
+        <v>-34.660488</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5237,22 +5237,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5267,12 +5267,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5294,14 +5294,14 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.438399</v>
+        <v>-58.460855</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.663958</v>
+        <v>-34.631046</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5323,17 +5323,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5353,12 +5353,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5380,10 +5380,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.475565</v>
+        <v>-58.479751</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.660488</v>
+        <v>-34.677211</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5409,22 +5409,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5466,36 +5466,36 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.460855</v>
+        <v>-58.491573</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.631046</v>
+        <v>-34.639215</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5505,12 +5505,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -5525,12 +5525,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5552,36 +5552,36 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.479751</v>
+        <v>-58.487715</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.677211</v>
+        <v>-34.636671</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>8245</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t xml:space="preserve">ZELADA 4401 </t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811626837</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5638,10 +5638,10 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.491573</v>
+        <v>-58.488539</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.639215</v>
+        <v>-34.640962</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5667,22 +5667,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>8125</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/2/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5697,12 +5697,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811626981</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5724,51 +5724,51 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.487715</v>
+        <v>-58.423058</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.636671</v>
+        <v>-34.608916</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>ALM-E</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>8245</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADA 4401 </t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811626837</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5810,51 +5810,51 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.488539</v>
+        <v>-58.481162</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.640962</v>
+        <v>-34.665875</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>8125</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2/2/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811626981</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5896,14 +5896,14 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.423058</v>
+        <v>-58.413945</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.608916</v>
+        <v>-34.582774</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>ALM-E</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -5925,22 +5925,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5982,10 +5982,10 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.481162</v>
+        <v>-58.437739</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.665875</v>
+        <v>-34.638224</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5999,7 +5999,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6011,7 +6011,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>8490</t>
+          <t>900009468810</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -6021,12 +6021,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Ugarteche 2816</t>
+          <t xml:space="preserve">CUENCA 3033 </t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>corroida inclinada</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6061,31 +6061,31 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L66" t="n">
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.413945</v>
+        <v>-58.494814</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.582774</v>
+        <v>-34.601905</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>AGU-M</t>
+          <t>DEV-B</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6097,17 +6097,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6154,10 +6154,10 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.437739</v>
+        <v>-58.469878</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.638224</v>
+        <v>-34.626919</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6183,22 +6183,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>900009468810</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUENCA 3033 </t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6233,31 +6233,31 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L68" t="n">
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.494814</v>
+        <v>-58.46026</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.601905</v>
+        <v>-34.640706</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>DEV-B</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6269,7 +6269,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6279,12 +6279,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6299,12 +6299,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6326,10 +6326,10 @@
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.469878</v>
+        <v>-58.480708</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.626919</v>
+        <v>-34.667639</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -6343,7 +6343,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6355,22 +6355,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>8244</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t xml:space="preserve">ZELADA 4401 </t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>812440296</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6412,36 +6412,36 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.46026</v>
+        <v>-58.488539</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.640706</v>
+        <v>-34.640962</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -6451,12 +6451,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6498,36 +6498,36 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.480708</v>
+        <v>-58.474151</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.667639</v>
+        <v>-34.630046</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>NRA-R</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2NRA</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>8244</t>
+          <t>S00552343</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6537,12 +6537,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADA 4401 </t>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6557,12 +6557,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>812440296</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada base corroida</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6572,58 +6572,58 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L72" t="n">
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.488539</v>
+        <v>-58.464382</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.640962</v>
+        <v>-34.683083</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>S00176142</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t>CULPINA 533</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -6643,12 +6643,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -6670,51 +6670,47 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.474151</v>
+        <v>-58.464205</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.630046</v>
+        <v>-34.636221</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>NRA-R</t>
-        </is>
-      </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>ARATO-25058.PO.2NRA</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6734,7 +6730,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>inclinada base corroida</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6744,7 +6740,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -6756,24 +6752,24 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.464382</v>
+        <v>-58.517269</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.683083</v>
+        <v>-34.639879</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PAV-B</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6785,22 +6781,22 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>-772</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t>LA PLATA AV. 2304</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6820,7 +6816,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>Desplazar Columna</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6830,7 +6826,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -6842,10 +6838,10 @@
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.464205</v>
+        <v>-58.423086</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.636221</v>
+        <v>-34.641356</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6859,15 +6855,19 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr"/>
+          <t>PPT-L</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>-774</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -6877,12 +6877,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t>CASEROS AV. 4131</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>mover a 4111</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6917,31 +6917,31 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L76" t="n">
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.517269</v>
+        <v>-58.422741</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.639879</v>
+        <v>-34.639999</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PAV-B</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6953,17 +6953,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>8597</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>JUJUY AV 1717</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -6981,14 +6981,10 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7010,14 +7006,14 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.423086</v>
+        <v>-58.400922</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.641356</v>
+        <v>-34.630312</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -7027,96 +7023,10 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>PPT-F</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>-774</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>3/9/2026</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>CASEROS AV. 4131</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>mover a 4111</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L78" t="n">
-        <v>1</v>
-      </c>
-      <c r="M78" t="n">
-        <v>-58.422741</v>
-      </c>
-      <c r="N78" t="n">
-        <v>-34.639999</v>
-      </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q78" t="inlineStr">
-        <is>
-          <t>PPT-L</t>
-        </is>
-      </c>
-      <c r="R78" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-21 15:35:57)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R77"/>
+  <dimension ref="A1:R81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1801,22 +1801,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>7260</t>
+          <t>7038</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>9/10/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Vidal 1861</t>
+          <t>SARANDI 1011</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1831,12 +1831,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>809642175</t>
+          <t>809195660</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada entro tambien como caso 7209</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1858,24 +1858,24 @@
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.458298</v>
+        <v>-58.394543</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.566511</v>
+        <v>-34.620732</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>COG-F</t>
+          <t>CEN-C</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1887,22 +1887,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6475</t>
+          <t>7260</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9/17/2025</t>
+          <t>9/10/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Av Amancio Alcorta 3570</t>
+          <t>Vidal 1861</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1917,17 +1917,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>809800213</t>
+          <t>809642175</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>aplomar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1937,31 +1937,31 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.409278</v>
+        <v>-58.458298</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.653566</v>
+        <v>-34.566511</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>COG-F</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1973,7 +1973,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6182</t>
+          <t>6475</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Los Patos 2702</t>
+          <t>Av Amancio Alcorta 3570</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>809818308</t>
+          <t>809800213</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
+          <t>aplomar</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2023,17 +2023,17 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.399262</v>
+        <v>-58.409278</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.639685</v>
+        <v>-34.653566</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>PPT-K</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2059,22 +2059,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7373</t>
+          <t>6182</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10/2/2025</t>
+          <t>9/17/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SANTIAGO DEL ESTERO 1253</t>
+          <t>Los Patos 2702</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2089,12 +2089,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>810132493</t>
+          <t>809818308</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2116,10 +2116,10 @@
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.384406</v>
+        <v>-58.399262</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.622932</v>
+        <v>-34.639685</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>CON-M</t>
+          <t>PPT-K</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2145,22 +2145,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>7950</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10/13/2025</t>
+          <t>9/29/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>Fitz Roy 2476</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>810333018</t>
+          <t>810038995</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2202,14 +2202,14 @@
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.46138</v>
+        <v>-58.429159</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.629774</v>
+        <v>-34.577821</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>ATH-I</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2231,22 +2231,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7516</t>
+          <t>7372</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/2/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ALVAREZ, CRISOSTOMO 3000</t>
+          <t>DIAZ, CESAR, GRAL. 1657</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>ICD31468700</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R150 o R200</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2288,24 +2288,24 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.458516</v>
+        <v>-58.463851</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.646422</v>
+        <v>-34.606961</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2317,22 +2317,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7735</t>
+          <t>7373</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/2/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GARCIA, MARTIN AV. 772</t>
+          <t>SANTIAGO DEL ESTERO 1253</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>810371042</t>
+          <t>810132493</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2374,10 +2374,10 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.374086</v>
+        <v>-58.384406</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.633168</v>
+        <v>-34.622932</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2391,34 +2391,34 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CON-B</t>
+          <t>CON-M</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>ARATO-25058.AF.1CON</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7595</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/13/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SAENZ AV. 1204</t>
+          <t>FALCON, RAMON L.,CNEL. 2353</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810416653</t>
+          <t>810333018</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2460,14 +2460,14 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.416237</v>
+        <v>-58.46138</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.65477</v>
+        <v>-34.629774</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2489,22 +2489,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7556</t>
+          <t>7516</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1923</t>
+          <t>ALVAREZ, CRISOSTOMO 3000</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2519,12 +2519,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2546,14 +2546,14 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.411426</v>
+        <v>-58.458516</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.633266</v>
+        <v>-34.646422</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2575,22 +2575,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7579</t>
+          <t>7735</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AGUIRRE 508</t>
+          <t>GARCIA, MARTIN AV. 772</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>810421912</t>
+          <t>810371042</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2625,21 +2625,21 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.435731</v>
+        <v>-58.374086</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.597659</v>
+        <v>-34.633168</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2649,34 +2649,34 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>CON-B</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.AF.1CON</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7631</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CALVO, CARLOS 3762</t>
+          <t>SAENZ AV. 1204</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>810416653</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2718,14 +2718,14 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.418542</v>
+        <v>-58.416237</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.624609</v>
+        <v>-34.65477</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2747,22 +2747,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>7556</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>SANCHEZ DE LORIA 1923</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>cambiar</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2804,14 +2804,14 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.430613</v>
+        <v>-58.411426</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.608805</v>
+        <v>-34.633266</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2833,22 +2833,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7579</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>AGUIRRE 508</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>810421912</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2878,36 +2878,36 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.50161</v>
+        <v>-58.435731</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.647648</v>
+        <v>-34.597659</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2919,22 +2919,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7643</t>
+          <t>7631</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ACEVEDO 524</t>
+          <t>CALVO, CARLOS 3762</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>810458896</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2976,14 +2976,14 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.439164</v>
+        <v>-58.418542</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.597069</v>
+        <v>-34.624609</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3005,22 +3005,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7665</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ARAOZ 2313</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Picada y cable cortado</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3062,14 +3062,14 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.417634</v>
+        <v>-58.430613</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.587439</v>
+        <v>-34.608805</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3091,22 +3091,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3148,14 +3148,14 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.48121</v>
+        <v>-58.50161</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.61126</v>
+        <v>-34.647648</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3177,22 +3177,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7719</t>
+          <t>7643</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ 180</t>
+          <t>ACEVEDO 524</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3207,12 +3207,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>810458896</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Colocar R400 para traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.440031</v>
+        <v>-58.439164</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.575409</v>
+        <v>-34.597069</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3263,22 +3263,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7732</t>
+          <t>7665</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1142</t>
+          <t>ARAOZ 2313</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada y cable cortado</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3320,14 +3320,14 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.413563</v>
+        <v>-58.417634</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.624645</v>
+        <v>-34.587439</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3349,22 +3349,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7744</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/31/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NECOCHEA 369</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>01233359</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Colocar R200 para rtaspaso de nodo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3406,24 +3406,24 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.364132</v>
+        <v>-58.48121</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.628423</v>
+        <v>-34.61126</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>CON-F</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3435,22 +3435,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7829</t>
+          <t>7719</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>CIUDAD DE LA PAZ 180</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R400 para traspaso</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3492,14 +3492,14 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.460356</v>
+        <v>-58.440031</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.630793</v>
+        <v>-34.575409</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3521,22 +3521,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>7732</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>11/4/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 1654</t>
+          <t>LINIERS VIRREY 1142</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3551,12 +3551,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>810573618</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Columna picada e inclinada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3578,14 +3578,14 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.389676</v>
+        <v>-58.413563</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.618127</v>
+        <v>-34.624645</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>CEN-?</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3607,22 +3607,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7604</t>
+          <t>7744</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>10/31/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 3741</t>
+          <t>NECOCHEA 369</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>01233359</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R200 para rtaspaso de nodo</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3664,14 +3664,14 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.418108</v>
+        <v>-58.364132</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.62564</v>
+        <v>-34.628423</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>CON-F</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3693,22 +3693,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3750,14 +3750,14 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.433855</v>
+        <v>-58.460356</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.614487</v>
+        <v>-34.630793</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3779,22 +3779,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7842</t>
+          <t>7780</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/4/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FERRARI 410</t>
+          <t>INDEPENDENCIA AV. 1654</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810713039</t>
+          <t>810573618</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Columna picada e inclinada</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3836,24 +3836,24 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.441198</v>
+        <v>-58.389676</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.605341</v>
+        <v>-34.618127</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>CEN-?</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3865,22 +3865,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t>7604</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t>SAN JUAN AV. 3741</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>columna inclinada base corroida</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3922,14 +3922,14 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.439239</v>
+        <v>-58.418108</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.6604</v>
+        <v>-34.62564</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3951,22 +3951,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S01140678</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810804375</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>columna inclinada corroida</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4008,14 +4008,14 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.388529</v>
+        <v>-58.433855</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.655949</v>
+        <v>-34.614487</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>CON-I</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4037,22 +4037,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t>7842</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t>FERRARI 410</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>810713039</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4094,14 +4094,14 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.491325</v>
+        <v>-58.441198</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.647761</v>
+        <v>-34.605341</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4123,22 +4123,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>columna inclinada base corroida</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4180,14 +4180,14 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.469394</v>
+        <v>-58.439239</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.626925</v>
+        <v>-34.6604</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4209,22 +4209,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>7892</t>
+          <t>S01140678</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Juncal 1642</t>
+          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>810804375</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna inclinada corroida</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -4266,14 +4266,14 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.390974</v>
+        <v>-58.388529</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.594177</v>
+        <v>-34.655949</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>RET-N</t>
+          <t>CON-I</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4295,22 +4295,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>7961</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>12/2/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CASTILLO 12</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4325,12 +4325,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>810984643</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4345,31 +4345,31 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.430396</v>
+        <v>-58.491325</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.599668</v>
+        <v>-34.647761</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4381,17 +4381,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7898</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>12/4/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BONIFACIO, JOSE 2319</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4411,12 +4411,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>810984687</t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4438,10 +4438,10 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.459955</v>
+        <v>-58.469394</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.631973</v>
+        <v>-34.626925</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4467,22 +4467,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S01204545</t>
+          <t>7892</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>12/10/2025</t>
+          <t>12/1/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Medina 420</t>
+          <t>Juncal 1642</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4497,12 +4497,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4524,51 +4524,51 @@
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.48802</v>
+        <v>-58.390974</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.641075</v>
+        <v>-34.594177</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>RET-N</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t>7961</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>12/2/2025</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t>CASTILLO 12</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4583,12 +4583,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>810984643</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4603,21 +4603,21 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.463198</v>
+        <v>-58.430396</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.62624</v>
+        <v>-34.599668</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4639,22 +4639,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t>7898</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>12/4/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t>BONIFACIO, JOSE 2319</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4669,12 +4669,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>810984687</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4696,47 +4696,51 @@
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.471183</v>
+        <v>-58.459955</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.638988</v>
+        <v>-34.631973</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R50" t="inlineStr"/>
+          <t>PCH-F</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>7997</t>
+          <t>S01204545</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>12/10/2025</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>Medina 420</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4751,12 +4755,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4778,51 +4782,51 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.46357</v>
+        <v>-58.48802</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.623187</v>
+        <v>-34.641075</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>8061</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>FOREST AV. 957</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4837,12 +4841,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811453824</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4857,31 +4861,31 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.45732</v>
+        <v>-58.463198</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.581366</v>
+        <v>-34.62624</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>ATH-N</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4893,22 +4897,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>-705</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>12/22/2025</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>Larrea 370</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4923,12 +4927,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>02013924</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4938,7 +4942,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4950,14 +4954,14 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.459547</v>
+        <v>-58.402154</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.626309</v>
+        <v>-34.605295</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -4967,7 +4971,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4979,22 +4983,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -5009,12 +5013,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5036,51 +5040,47 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.465166</v>
+        <v>-58.471183</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.670435</v>
+        <v>-34.638988</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PAV-?</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5095,12 +5095,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5122,14 +5122,14 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.438399</v>
+        <v>-58.46357</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.663958</v>
+        <v>-34.623187</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5151,22 +5151,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8061</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>FOREST AV. 957</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5181,12 +5181,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811453824</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5201,31 +5201,31 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.475565</v>
+        <v>-58.45732</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.660488</v>
+        <v>-34.581366</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>ATH-N</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5237,17 +5237,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5294,10 +5294,10 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.460855</v>
+        <v>-58.459547</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.631046</v>
+        <v>-34.626309</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5323,17 +5323,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5380,10 +5380,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.479751</v>
+        <v>-58.465166</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.677211</v>
+        <v>-34.670435</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5409,22 +5409,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5466,51 +5466,51 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.491573</v>
+        <v>-58.438399</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.639215</v>
+        <v>-34.663958</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5552,51 +5552,51 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.487715</v>
+        <v>-58.475565</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.636671</v>
+        <v>-34.660488</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>8245</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADA 4401 </t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811626837</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5638,51 +5638,51 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.488539</v>
+        <v>-58.460855</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.640962</v>
+        <v>-34.631046</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>8125</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2/2/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811626981</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5724,14 +5724,14 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.423058</v>
+        <v>-58.479751</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.608916</v>
+        <v>-34.677211</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -5741,7 +5741,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>ALM-E</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5753,22 +5753,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5810,51 +5810,51 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.481162</v>
+        <v>-58.491573</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.665875</v>
+        <v>-34.639215</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>8490</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Ugarteche 2816</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>corroida inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5896,51 +5896,51 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.413945</v>
+        <v>-58.487715</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.582774</v>
+        <v>-34.636671</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>AGU-M</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>8125</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/2/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5955,12 +5955,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>811626981</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5982,14 +5982,14 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.437739</v>
+        <v>-58.423058</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.638224</v>
+        <v>-34.608916</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>ALM-E</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6011,22 +6011,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>900009468810</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUENCA 3033 </t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6061,31 +6061,31 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L66" t="n">
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.494814</v>
+        <v>-58.481162</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.601905</v>
+        <v>-34.665875</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>DEV-B</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6097,22 +6097,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6154,14 +6154,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.469878</v>
+        <v>-58.413945</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.626919</v>
+        <v>-34.582774</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6183,17 +6183,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6240,10 +6240,10 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.46026</v>
+        <v>-58.437739</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.640706</v>
+        <v>-34.638224</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6269,22 +6269,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>900009468810</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t xml:space="preserve">CUENCA 3033 </t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6299,12 +6299,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6319,31 +6319,31 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.480708</v>
+        <v>-58.494814</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.667639</v>
+        <v>-34.601905</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>DEV-B</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6355,7 +6355,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>8244</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -6365,12 +6365,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADA 4401 </t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>812440296</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6412,46 +6412,46 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.488539</v>
+        <v>-58.469878</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.640962</v>
+        <v>-34.626919</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6471,12 +6471,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6498,36 +6498,36 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.474151</v>
+        <v>-58.46026</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.630046</v>
+        <v>-34.640706</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>NRA-R</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -6557,12 +6557,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>inclinada base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6572,22 +6572,22 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L72" t="n">
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.464382</v>
+        <v>-58.480708</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.683083</v>
+        <v>-34.667639</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6613,17 +6613,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -6643,12 +6643,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -6670,47 +6670,51 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.464205</v>
+        <v>-58.474151</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.636221</v>
+        <v>-34.630046</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R73" t="inlineStr"/>
+          <t>NRA-R</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2NRA</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>S00552343</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6730,7 +6734,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>inclinada base corroida</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6740,7 +6744,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -6752,24 +6756,24 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.517269</v>
+        <v>-58.464382</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.639879</v>
+        <v>-34.683083</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PAV-B</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6781,22 +6785,22 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>S00176142</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>CULPINA 533</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6816,7 +6820,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6826,7 +6830,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -6838,10 +6842,10 @@
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.423086</v>
+        <v>-58.464205</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.641356</v>
+        <v>-34.636221</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6855,19 +6859,15 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PPT-L</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>-774</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -6877,12 +6877,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CASEROS AV. 4131</t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>mover a 4111</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6917,31 +6917,31 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L76" t="n">
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.422741</v>
+        <v>-58.517269</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.639999</v>
+        <v>-34.639879</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>PAV-B</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6953,82 +6953,418 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>-772</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>3/10/2026</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>LA PLATA AV. 2304</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Desplazar Columna</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" t="n">
+        <v>-58.423086</v>
+      </c>
+      <c r="N77" t="n">
+        <v>-34.641356</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>PPT-L</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>-774</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>3/9/2026</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>CASEROS AV. 4131</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>mover a 4111</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>1</v>
+      </c>
+      <c r="M78" t="n">
+        <v>-58.422741</v>
+      </c>
+      <c r="N78" t="n">
+        <v>-34.639999</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>PPT-L</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t>8597</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>3/13/2026</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>JUJUY AV 1717</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr">
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
         <is>
           <t>Cambiar Columna</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="J79" t="inlineStr">
         <is>
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
+      <c r="K79" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L77" t="n">
-        <v>1</v>
-      </c>
-      <c r="M77" t="n">
+      <c r="L79" t="n">
+        <v>1</v>
+      </c>
+      <c r="M79" t="n">
         <v>-58.400922</v>
       </c>
-      <c r="N77" t="n">
+      <c r="N79" t="n">
         <v>-34.630312</v>
       </c>
-      <c r="O77" t="inlineStr">
+      <c r="O79" t="inlineStr">
         <is>
           <t>San Telmo</t>
         </is>
       </c>
-      <c r="P77" t="inlineStr">
+      <c r="P79" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q77" t="inlineStr">
+      <c r="Q79" t="inlineStr">
         <is>
           <t>PPT-F</t>
         </is>
       </c>
-      <c r="R77" t="inlineStr">
+      <c r="R79" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7460 </t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>3/21/2026</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>TERRADA 2720</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>RIENDA A PIQUE CORTADA</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" t="n">
+        <v>-58.486103</v>
+      </c>
+      <c r="N80" t="n">
+        <v>-34.603895</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>NRA-P</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>00000609</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>3/21/2026</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ZELADA 4402</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>-58.48834</v>
+      </c>
+      <c r="N81" t="n">
+        <v>-34.641018</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>PCH-S</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-23 13:58:07)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R81"/>
+  <dimension ref="A1:R82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1801,27 +1801,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>7038</t>
+          <t>5894</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>5/27/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SARANDI 1011</t>
+          <t>ALBARELLOS AV. 3100</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Transito</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1831,17 +1831,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>809195660</t>
+          <t>ICD30340076</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Picada entro tambien como caso 7209</t>
+          <t>QAP fotos del gcba tenia las incorrectas</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Tensor</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1851,31 +1851,31 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.394543</v>
+        <v>-58.512533</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.620732</v>
+        <v>-34.579243</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>CEN-C</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1887,22 +1887,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>7260</t>
+          <t>7038</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9/10/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vidal 1861</t>
+          <t>SARANDI 1011</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1917,12 +1917,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>809642175</t>
+          <t>809195660</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada entro tambien como caso 7209</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1944,24 +1944,24 @@
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.458298</v>
+        <v>-58.394543</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.566511</v>
+        <v>-34.620732</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>COG-F</t>
+          <t>CEN-C</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1973,22 +1973,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6475</t>
+          <t>7260</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9/17/2025</t>
+          <t>9/10/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Av Amancio Alcorta 3570</t>
+          <t>Vidal 1861</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>809800213</t>
+          <t>809642175</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>aplomar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2023,31 +2023,31 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.409278</v>
+        <v>-58.458298</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.653566</v>
+        <v>-34.566511</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>COG-F</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6182</t>
+          <t>6475</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Los Patos 2702</t>
+          <t>Av Amancio Alcorta 3570</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2089,17 +2089,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>809818308</t>
+          <t>809800213</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
+          <t>aplomar</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2109,17 +2109,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.399262</v>
+        <v>-58.409278</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.639685</v>
+        <v>-34.653566</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PPT-K</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2145,22 +2145,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7950</t>
+          <t>6182</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>9/29/2025</t>
+          <t>9/17/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fitz Roy 2476</t>
+          <t>Los Patos 2702</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>810038995</t>
+          <t>809818308</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2202,14 +2202,14 @@
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.429159</v>
+        <v>-58.399262</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.577821</v>
+        <v>-34.639685</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>ATH-I</t>
+          <t>PPT-K</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2231,22 +2231,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7372</t>
+          <t>7950</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/2/2025</t>
+          <t>9/29/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DIAZ, CESAR, GRAL. 1657</t>
+          <t>Fitz Roy 2476</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ICD31468700</t>
+          <t>810038995</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Colocar R150 o R200</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2288,24 +2288,24 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.463851</v>
+        <v>-58.429159</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.606961</v>
+        <v>-34.577821</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>ATH-I</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2317,7 +2317,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7373</t>
+          <t>7372</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2327,12 +2327,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SANTIAGO DEL ESTERO 1253</t>
+          <t>DIAZ, CESAR, GRAL. 1657</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2347,12 +2347,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>810132493</t>
+          <t>ICD31468700</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R150 o R200</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2374,24 +2374,24 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.384406</v>
+        <v>-58.463851</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.622932</v>
+        <v>-34.606961</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CON-M</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2403,22 +2403,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>7373</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10/13/2025</t>
+          <t>10/2/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>SANTIAGO DEL ESTERO 1253</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810333018</t>
+          <t>810132493</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2460,14 +2460,14 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.46138</v>
+        <v>-58.384406</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.629774</v>
+        <v>-34.622932</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>CON-M</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2489,17 +2489,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7516</t>
+          <t>7595</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/13/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ALVAREZ, CRISOSTOMO 3000</t>
+          <t>FALCON, RAMON L.,CNEL. 2353</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>810333018</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2546,10 +2546,10 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.458516</v>
+        <v>-58.46138</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.646422</v>
+        <v>-34.629774</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2575,7 +2575,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7735</t>
+          <t>7516</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2585,12 +2585,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GARCIA, MARTIN AV. 772</t>
+          <t>ALVAREZ, CRISOSTOMO 3000</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>810371042</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2632,14 +2632,14 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.374086</v>
+        <v>-58.458516</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.633168</v>
+        <v>-34.646422</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2649,29 +2649,29 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CON-B</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>ARATO-25058.AF.1CON</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7735</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SAENZ AV. 1204</t>
+          <t>GARCIA, MARTIN AV. 772</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>810416653</t>
+          <t>810371042</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2718,10 +2718,10 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.416237</v>
+        <v>-58.374086</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.65477</v>
+        <v>-34.633168</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2735,34 +2735,34 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>CON-B</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.AF.1CON</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7556</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1923</t>
+          <t>SAENZ AV. 1204</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>810416653</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2804,10 +2804,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.411426</v>
+        <v>-58.416237</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.633266</v>
+        <v>-34.65477</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2833,22 +2833,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7579</t>
+          <t>7556</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AGUIRRE 508</t>
+          <t>SANCHEZ DE LORIA 1923</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>810421912</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>cambiar</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2883,21 +2883,21 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.435731</v>
+        <v>-58.411426</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.597659</v>
+        <v>-34.633266</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2919,22 +2919,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7631</t>
+          <t>7579</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CALVO, CARLOS 3762</t>
+          <t>AGUIRRE 508</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>810421912</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2969,21 +2969,21 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.418542</v>
+        <v>-58.435731</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.624609</v>
+        <v>-34.597659</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3005,7 +3005,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>7631</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3015,12 +3015,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>CALVO, CARLOS 3762</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3062,14 +3062,14 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.430613</v>
+        <v>-58.418542</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.608805</v>
+        <v>-34.624609</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3091,7 +3091,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3101,12 +3101,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3148,24 +3148,24 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.50161</v>
+        <v>-58.430613</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.647648</v>
+        <v>-34.608805</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3177,22 +3177,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7643</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ACEVEDO 524</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>810458896</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3234,24 +3234,24 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.439164</v>
+        <v>-58.50161</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.597069</v>
+        <v>-34.647648</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3263,7 +3263,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7665</t>
+          <t>7643</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3273,12 +3273,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ARAOZ 2313</t>
+          <t>ACEVEDO 524</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>810458896</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Picada y cable cortado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3320,10 +3320,10 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.417634</v>
+        <v>-58.439164</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.587439</v>
+        <v>-34.597069</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3349,22 +3349,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>7665</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>ARAOZ 2313</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada y cable cortado</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3406,24 +3406,24 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.48121</v>
+        <v>-58.417634</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.61126</v>
+        <v>-34.587439</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3435,7 +3435,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7719</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3445,12 +3445,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ 180</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Colocar R400 para traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3492,24 +3492,24 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.440031</v>
+        <v>-58.48121</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.575409</v>
+        <v>-34.61126</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3521,7 +3521,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7732</t>
+          <t>7719</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3531,12 +3531,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1142</t>
+          <t>CIUDAD DE LA PAZ 180</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3551,12 +3551,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R400 para traspaso</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3578,14 +3578,14 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.413563</v>
+        <v>-58.440031</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.624645</v>
+        <v>-34.575409</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3607,22 +3607,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7744</t>
+          <t>7732</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/31/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NECOCHEA 369</t>
+          <t>LINIERS VIRREY 1142</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>01233359</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Colocar R200 para rtaspaso de nodo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3664,14 +3664,14 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.364132</v>
+        <v>-58.413563</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.628423</v>
+        <v>-34.624645</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>CON-F</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3693,22 +3693,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7829</t>
+          <t>7744</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>10/31/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>NECOCHEA 369</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>01233359</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R200 para rtaspaso de nodo</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3750,14 +3750,14 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.460356</v>
+        <v>-58.364132</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.630793</v>
+        <v>-34.628423</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>CON-F</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3779,22 +3779,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/4/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 1654</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810573618</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Columna picada e inclinada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3836,14 +3836,14 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.389676</v>
+        <v>-58.460356</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.618127</v>
+        <v>-34.630793</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>CEN-?</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3865,22 +3865,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7604</t>
+          <t>7780</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/4/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 3741</t>
+          <t>INDEPENDENCIA AV. 1654</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>810573618</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Columna picada e inclinada</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3922,14 +3922,14 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.418108</v>
+        <v>-58.389676</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.62564</v>
+        <v>-34.618127</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>CEN-?</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3951,7 +3951,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>7604</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3961,12 +3961,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t>SAN JUAN AV. 3741</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4008,14 +4008,14 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.433855</v>
+        <v>-58.418108</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.614487</v>
+        <v>-34.62564</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4037,22 +4037,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7842</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FERRARI 410</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810713039</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4094,24 +4094,24 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.441198</v>
+        <v>-58.433855</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.605341</v>
+        <v>-34.614487</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4123,22 +4123,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t>7842</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t>FERRARI 410</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810713039</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>columna inclinada base corroida</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4180,24 +4180,24 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.439239</v>
+        <v>-58.441198</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.6604</v>
+        <v>-34.605341</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4209,7 +4209,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S01140678</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4219,12 +4219,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>810804375</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>columna inclinada corroida</t>
+          <t>columna inclinada base corroida</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4266,10 +4266,10 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.388529</v>
+        <v>-58.439239</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.655949</v>
+        <v>-34.6604</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>CON-I</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4295,22 +4295,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t>S01140678</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4325,12 +4325,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>810804375</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>columna inclinada corroida</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4352,24 +4352,24 @@
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.491325</v>
+        <v>-58.388529</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.647761</v>
+        <v>-34.655949</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>CON-I</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4381,7 +4381,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4391,12 +4391,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4411,12 +4411,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4438,24 +4438,24 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.469394</v>
+        <v>-58.491325</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.626925</v>
+        <v>-34.647761</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4467,22 +4467,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7892</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Juncal 1642</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4497,12 +4497,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4524,14 +4524,14 @@
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.390974</v>
+        <v>-58.469394</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.594177</v>
+        <v>-34.626925</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>RET-N</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4553,22 +4553,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7961</t>
+          <t>7892</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12/2/2025</t>
+          <t>12/1/2025</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CASTILLO 12</t>
+          <t>Juncal 1642</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>810984643</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4598,26 +4598,26 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.430396</v>
+        <v>-58.390974</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.599668</v>
+        <v>-34.594177</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>RET-N</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4639,22 +4639,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7898</t>
+          <t>7961</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>12/4/2025</t>
+          <t>12/2/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BONIFACIO, JOSE 2319</t>
+          <t>CASTILLO 12</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>810984687</t>
+          <t>810984643</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4689,21 +4689,21 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.459955</v>
+        <v>-58.430396</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.631973</v>
+        <v>-34.599668</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4725,22 +4725,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S01204545</t>
+          <t>7898</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>12/10/2025</t>
+          <t>12/4/2025</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Medina 420</t>
+          <t>BONIFACIO, JOSE 2319</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4755,12 +4755,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t>810984687</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4782,51 +4782,51 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.48802</v>
+        <v>-58.459955</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.641075</v>
+        <v>-34.631973</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t>S01204545</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>12/10/2025</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t>Medina 420</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4841,12 +4841,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4868,51 +4868,51 @@
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.463198</v>
+        <v>-58.48802</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.62624</v>
+        <v>-34.641075</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>-705</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>12/22/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Larrea 370</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4927,12 +4927,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>02013924</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4954,14 +4954,14 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.402154</v>
+        <v>-58.463198</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.605295</v>
+        <v>-34.62624</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>CLI-D</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4983,22 +4983,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t>-705</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>12/22/2025</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t>Larrea 370</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -5013,12 +5013,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>02013924</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -5040,47 +5040,51 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.471183</v>
+        <v>-58.402154</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.638988</v>
+        <v>-34.605295</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr"/>
+          <t>CLI-D</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>7997</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5095,7 +5099,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5122,51 +5126,47 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.46357</v>
+        <v>-58.471183</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.623187</v>
+        <v>-34.638988</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>NRA-E</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8061</t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>FOREST AV. 957</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5181,12 +5181,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811453824</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5201,31 +5201,31 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.45732</v>
+        <v>-58.46357</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.581366</v>
+        <v>-34.623187</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>ATH-N</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5237,22 +5237,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>8061</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>FOREST AV. 957</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5267,12 +5267,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811453824</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5287,31 +5287,31 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L57" t="n">
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.459547</v>
+        <v>-58.45732</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.626309</v>
+        <v>-34.581366</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>ATH-N</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5323,22 +5323,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -5353,12 +5353,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5380,10 +5380,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.465166</v>
+        <v>-58.459547</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.670435</v>
+        <v>-34.626309</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5409,17 +5409,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5466,14 +5466,14 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.438399</v>
+        <v>-58.465166</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.663958</v>
+        <v>-34.670435</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5495,7 +5495,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5525,12 +5525,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5552,14 +5552,14 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.475565</v>
+        <v>-58.438399</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.660488</v>
+        <v>-34.663958</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5581,22 +5581,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5638,10 +5638,10 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.460855</v>
+        <v>-58.475565</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.631046</v>
+        <v>-34.660488</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5667,22 +5667,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5697,12 +5697,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5724,10 +5724,10 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.479751</v>
+        <v>-58.460855</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.677211</v>
+        <v>-34.631046</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5753,7 +5753,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5763,12 +5763,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5810,36 +5810,36 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.491573</v>
+        <v>-58.479751</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.639215</v>
+        <v>-34.677211</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5849,7 +5849,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5896,10 +5896,10 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.487715</v>
+        <v>-58.491573</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.636671</v>
+        <v>-34.639215</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -5925,22 +5925,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8125</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2/2/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5955,12 +5955,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>811626981</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5982,51 +5982,51 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.423058</v>
+        <v>-58.487715</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.608916</v>
+        <v>-34.636671</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>ALM-E</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>8125</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>2/2/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>811626981</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6068,14 +6068,14 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.481162</v>
+        <v>-58.423058</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.665875</v>
+        <v>-34.608916</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>ALM-E</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6097,22 +6097,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>8490</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Ugarteche 2816</t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>corroida inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6154,14 +6154,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.413945</v>
+        <v>-58.481162</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.582774</v>
+        <v>-34.665875</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>AGU-M</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6183,7 +6183,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6240,14 +6240,14 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.437739</v>
+        <v>-58.413945</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.638224</v>
+        <v>-34.582774</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6269,7 +6269,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>900009468810</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6279,12 +6279,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUENCA 3033 </t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6299,12 +6299,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6319,31 +6319,31 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.494814</v>
+        <v>-58.437739</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.601905</v>
+        <v>-34.638224</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>DEV-B</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6355,22 +6355,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>900009468810</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t xml:space="preserve">CUENCA 3033 </t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6405,31 +6405,31 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L70" t="n">
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.469878</v>
+        <v>-58.494814</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.626919</v>
+        <v>-34.601905</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>DEV-B</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6441,17 +6441,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6471,12 +6471,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6498,10 +6498,10 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.46026</v>
+        <v>-58.469878</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.640706</v>
+        <v>-34.626919</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6527,22 +6527,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6557,12 +6557,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6584,10 +6584,10 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.480708</v>
+        <v>-58.46026</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.667639</v>
+        <v>-34.640706</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6613,7 +6613,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6623,12 +6623,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6643,7 +6643,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -6670,36 +6670,36 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.474151</v>
+        <v>-58.480708</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.630046</v>
+        <v>-34.667639</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>NRA-R</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6709,12 +6709,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6729,12 +6729,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>inclinada base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6744,63 +6744,63 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L74" t="n">
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.464382</v>
+        <v>-58.474151</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.683083</v>
+        <v>-34.630046</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>NRA-R</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2NRA</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>S00552343</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada base corroida</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6835,17 +6835,17 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L75" t="n">
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.464205</v>
+        <v>-58.464382</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.636221</v>
+        <v>-34.683083</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6859,30 +6859,34 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr"/>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>S00176142</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t>CULPINA 533</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6902,7 +6906,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6912,63 +6916,59 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L76" t="n">
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.517269</v>
+        <v>-58.464205</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.639879</v>
+        <v>-34.636221</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PAV-B</t>
-        </is>
-      </c>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7003,31 +7003,31 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L77" t="n">
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.423086</v>
+        <v>-58.517269</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.641356</v>
+        <v>-34.639879</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>PAV-B</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7039,22 +7039,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>-774</t>
+          <t>-772</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CASEROS AV. 4131</t>
+          <t>LA PLATA AV. 2304</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>mover a 4111</t>
+          <t>Desplazar Columna</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -7096,10 +7096,10 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.422741</v>
+        <v>-58.423086</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.639999</v>
+        <v>-34.641356</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -7125,22 +7125,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>8597</t>
+          <t>-774</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>3/13/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>JUJUY AV 1717</t>
+          <t>CASEROS AV. 4131</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7153,10 +7153,14 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>mover a 4111</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7178,14 +7182,14 @@
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.400922</v>
+        <v>-58.422741</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.630312</v>
+        <v>-34.639999</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -7195,7 +7199,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PPT-F</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7207,22 +7211,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">7460 </t>
+          <t>8597</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TERRADA 2720</t>
+          <t>JUJUY AV 1717</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7238,12 +7242,12 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>RIENDA A PIQUE CORTADA</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -7253,31 +7257,31 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.486103</v>
+        <v>-58.400922</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.603895</v>
+        <v>-34.630312</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>PPT-F</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7289,7 +7293,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>00000609</t>
+          <t xml:space="preserve">7460 </t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7299,12 +7303,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ZELADA 4402</t>
+          <t>TERRADA 2720</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7320,49 +7324,131 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
+          <t>RIENDA A PIQUE CORTADA</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" t="n">
+        <v>-58.486103</v>
+      </c>
+      <c r="N81" t="n">
+        <v>-34.603895</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>NRA-P</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>00000609</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>3/21/2026</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ZELADA 4402</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
           <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
+      <c r="I82" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="J82" t="inlineStr">
         <is>
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
+      <c r="K82" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L81" t="n">
-        <v>1</v>
-      </c>
-      <c r="M81" t="n">
+      <c r="L82" t="n">
+        <v>1</v>
+      </c>
+      <c r="M82" t="n">
         <v>-58.48834</v>
       </c>
-      <c r="N81" t="n">
+      <c r="N82" t="n">
         <v>-34.641018</v>
       </c>
-      <c r="O81" t="inlineStr">
+      <c r="O82" t="inlineStr">
         <is>
           <t>Devoto</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="P82" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q81" t="inlineStr">
+      <c r="Q82" t="inlineStr">
         <is>
           <t>PCH-S</t>
         </is>
       </c>
-      <c r="R81" t="inlineStr">
+      <c r="R82" t="inlineStr">
         <is>
           <t>ARATO-25058.PO.2PCH</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-25 10:26:19)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -1801,27 +1801,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5894</t>
+          <t>7038</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>5/27/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ALBARELLOS AV. 3100</t>
+          <t>SARANDI 1011</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pendiente de Transito</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1831,17 +1831,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ICD30340076</t>
+          <t>809195660</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>QAP fotos del gcba tenia las incorrectas</t>
+          <t>Picada entro tambien como caso 7209</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Tensor</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1851,31 +1851,31 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.512533</v>
+        <v>-58.394543</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.579243</v>
+        <v>-34.620732</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>CEN-C</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1887,22 +1887,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>7038</t>
+          <t>7260</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>9/10/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SARANDI 1011</t>
+          <t>Vidal 1861</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1917,12 +1917,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>809195660</t>
+          <t>809642175</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Picada entro tambien como caso 7209</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1944,24 +1944,24 @@
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.394543</v>
+        <v>-58.458298</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.620732</v>
+        <v>-34.566511</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>CEN-C</t>
+          <t>COG-F</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1973,22 +1973,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>7260</t>
+          <t>6475</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9/10/2025</t>
+          <t>9/17/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Vidal 1861</t>
+          <t>Av Amancio Alcorta 3570</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>809642175</t>
+          <t>809800213</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>aplomar</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2023,31 +2023,31 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.458298</v>
+        <v>-58.409278</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.566511</v>
+        <v>-34.653566</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>COG-F</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6475</t>
+          <t>6182</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Av Amancio Alcorta 3570</t>
+          <t>Los Patos 2702</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2089,17 +2089,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>809800213</t>
+          <t>809818308</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>aplomar</t>
+          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2109,17 +2109,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.409278</v>
+        <v>-58.399262</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.653566</v>
+        <v>-34.639685</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>PPT-K</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2145,22 +2145,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6182</t>
+          <t>7950</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>9/17/2025</t>
+          <t>9/29/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Los Patos 2702</t>
+          <t>Fitz Roy 2476</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>809818308</t>
+          <t>810038995</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Sacar PRFV del cantero, colocar en vereda y aplomar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2202,14 +2202,14 @@
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.399262</v>
+        <v>-58.429159</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.639685</v>
+        <v>-34.577821</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PPT-K</t>
+          <t>ATH-I</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2231,22 +2231,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7950</t>
+          <t>7372</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>9/29/2025</t>
+          <t>10/2/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fitz Roy 2476</t>
+          <t>DIAZ, CESAR, GRAL. 1657</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>810038995</t>
+          <t>ICD31468700</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R150 o R200</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2288,24 +2288,24 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.429159</v>
+        <v>-58.463851</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.577821</v>
+        <v>-34.606961</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>ATH-I</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2317,7 +2317,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7372</t>
+          <t>7373</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2327,12 +2327,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DIAZ, CESAR, GRAL. 1657</t>
+          <t>SANTIAGO DEL ESTERO 1253</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2347,12 +2347,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ICD31468700</t>
+          <t>810132493</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Colocar R150 o R200</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2374,24 +2374,24 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.463851</v>
+        <v>-58.384406</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.606961</v>
+        <v>-34.622932</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>CON-M</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2403,22 +2403,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7373</t>
+          <t>7595</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10/2/2025</t>
+          <t>10/13/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SANTIAGO DEL ESTERO 1253</t>
+          <t>FALCON, RAMON L.,CNEL. 2353</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810132493</t>
+          <t>810333018</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2460,14 +2460,14 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.384406</v>
+        <v>-58.46138</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.622932</v>
+        <v>-34.629774</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CON-M</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2489,17 +2489,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>7516</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/13/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>ALVAREZ, CRISOSTOMO 3000</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>810333018</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2546,10 +2546,10 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.46138</v>
+        <v>-58.458516</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.629774</v>
+        <v>-34.646422</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2575,7 +2575,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7516</t>
+          <t>7735</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2585,12 +2585,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ALVAREZ, CRISOSTOMO 3000</t>
+          <t>GARCIA, MARTIN AV. 772</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>810371042</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2632,14 +2632,14 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.458516</v>
+        <v>-58.374086</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.646422</v>
+        <v>-34.633168</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2649,29 +2649,29 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>CON-B</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.AF.1CON</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7735</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GARCIA, MARTIN AV. 772</t>
+          <t>SAENZ AV. 1204</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>810371042</t>
+          <t>810416653</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2718,10 +2718,10 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.374086</v>
+        <v>-58.416237</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.633168</v>
+        <v>-34.65477</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2735,34 +2735,34 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>CON-B</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>ARATO-25058.AF.1CON</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7556</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SAENZ AV. 1204</t>
+          <t>SANCHEZ DE LORIA 1923</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>810416653</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>cambiar</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2804,10 +2804,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.416237</v>
+        <v>-58.411426</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.65477</v>
+        <v>-34.633266</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2833,22 +2833,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7556</t>
+          <t>7579</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1923</t>
+          <t>AGUIRRE 508</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>810421912</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2883,21 +2883,21 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.411426</v>
+        <v>-58.435731</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.633266</v>
+        <v>-34.597659</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2919,22 +2919,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7579</t>
+          <t>7631</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AGUIRRE 508</t>
+          <t>CALVO, CARLOS 3762</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>810421912</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2969,21 +2969,21 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.435731</v>
+        <v>-58.418542</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.597659</v>
+        <v>-34.624609</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3005,7 +3005,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7631</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3015,12 +3015,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CALVO, CARLOS 3762</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3062,14 +3062,14 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.418542</v>
+        <v>-58.430613</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.624609</v>
+        <v>-34.608805</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3091,7 +3091,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3101,12 +3101,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3148,24 +3148,24 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.430613</v>
+        <v>-58.50161</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.608805</v>
+        <v>-34.647648</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3177,22 +3177,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7643</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>ACEVEDO 524</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>810458896</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3234,24 +3234,24 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.50161</v>
+        <v>-58.439164</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.647648</v>
+        <v>-34.597069</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3263,7 +3263,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7643</t>
+          <t>7665</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3273,12 +3273,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ACEVEDO 524</t>
+          <t>ARAOZ 2313</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>810458896</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada y cable cortado</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3320,10 +3320,10 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.439164</v>
+        <v>-58.417634</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.597069</v>
+        <v>-34.587439</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3349,22 +3349,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7665</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ARAOZ 2313</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Picada y cable cortado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3406,24 +3406,24 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.417634</v>
+        <v>-58.48121</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.587439</v>
+        <v>-34.61126</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3435,7 +3435,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>7719</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3445,12 +3445,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>CIUDAD DE LA PAZ 180</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R400 para traspaso</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3492,24 +3492,24 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.48121</v>
+        <v>-58.440031</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.61126</v>
+        <v>-34.575409</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3521,7 +3521,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7719</t>
+          <t>7732</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3531,12 +3531,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ 180</t>
+          <t>LINIERS VIRREY 1142</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3551,12 +3551,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Colocar R400 para traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3578,14 +3578,14 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.440031</v>
+        <v>-58.413563</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.575409</v>
+        <v>-34.624645</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3607,22 +3607,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7732</t>
+          <t>7744</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/31/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1142</t>
+          <t>NECOCHEA 369</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>01233359</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R200 para rtaspaso de nodo</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3664,14 +3664,14 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.413563</v>
+        <v>-58.364132</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.624645</v>
+        <v>-34.628423</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>CON-F</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3693,22 +3693,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7744</t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/31/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NECOCHEA 369</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>01233359</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Colocar R200 para rtaspaso de nodo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3750,14 +3750,14 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.364132</v>
+        <v>-58.460356</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.628423</v>
+        <v>-34.630793</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>CON-F</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3779,22 +3779,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7829</t>
+          <t>7780</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>11/4/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>INDEPENDENCIA AV. 1654</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>810573618</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Columna picada e inclinada</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3836,14 +3836,14 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.460356</v>
+        <v>-58.389676</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.630793</v>
+        <v>-34.618127</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>CEN-?</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3865,22 +3865,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>7604</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11/4/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 1654</t>
+          <t>SAN JUAN AV. 3741</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810573618</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Columna picada e inclinada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3922,14 +3922,14 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.389676</v>
+        <v>-58.418108</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.618127</v>
+        <v>-34.62564</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>CEN-?</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3951,7 +3951,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>7604</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3961,12 +3961,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 3741</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4008,14 +4008,14 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.418108</v>
+        <v>-58.433855</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.62564</v>
+        <v>-34.614487</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4037,22 +4037,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>7842</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t>FERRARI 410</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810713039</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4094,24 +4094,24 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.433855</v>
+        <v>-58.441198</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.614487</v>
+        <v>-34.605341</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4123,22 +4123,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>7842</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>FERRARI 410</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>810713039</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>columna inclinada base corroida</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4180,24 +4180,24 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.441198</v>
+        <v>-58.439239</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.605341</v>
+        <v>-34.6604</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4209,7 +4209,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t>S01140678</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4219,12 +4219,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810804375</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>columna inclinada base corroida</t>
+          <t>columna inclinada corroida</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4266,10 +4266,10 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.439239</v>
+        <v>-58.388529</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.6604</v>
+        <v>-34.655949</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>CON-I</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4295,22 +4295,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S01140678</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4325,12 +4325,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>810804375</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>columna inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4352,24 +4352,24 @@
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.388529</v>
+        <v>-58.491325</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.655949</v>
+        <v>-34.647761</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>CON-I</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4381,7 +4381,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4391,12 +4391,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4411,12 +4411,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4438,24 +4438,24 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.491325</v>
+        <v>-58.469394</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.647761</v>
+        <v>-34.626925</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4467,22 +4467,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>7892</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>12/1/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>Juncal 1642</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4497,12 +4497,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4524,14 +4524,14 @@
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.469394</v>
+        <v>-58.390974</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.626925</v>
+        <v>-34.594177</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>RET-N</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4553,22 +4553,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7892</t>
+          <t>7961</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>12/2/2025</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Juncal 1642</t>
+          <t>CASTILLO 12</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>810984643</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4598,26 +4598,26 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.390974</v>
+        <v>-58.430396</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.594177</v>
+        <v>-34.599668</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>RET-N</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4639,22 +4639,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7961</t>
+          <t>7898</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>12/2/2025</t>
+          <t>12/4/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CASTILLO 12</t>
+          <t>BONIFACIO, JOSE 2319</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>810984643</t>
+          <t>810984687</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4689,21 +4689,21 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.430396</v>
+        <v>-58.459955</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.599668</v>
+        <v>-34.631973</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4725,22 +4725,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>7898</t>
+          <t>S01204545</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>12/4/2025</t>
+          <t>12/10/2025</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>BONIFACIO, JOSE 2319</t>
+          <t>Medina 420</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4755,12 +4755,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>810984687</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4782,51 +4782,51 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.459955</v>
+        <v>-58.48802</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.631973</v>
+        <v>-34.641075</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S01204545</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>12/10/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Medina 420</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4841,12 +4841,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4868,51 +4868,51 @@
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.48802</v>
+        <v>-58.463198</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.641075</v>
+        <v>-34.62624</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t>-705</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>12/22/2025</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t>Larrea 370</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4927,12 +4927,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>02013924</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4954,14 +4954,14 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.463198</v>
+        <v>-58.402154</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.62624</v>
+        <v>-34.605295</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4983,22 +4983,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>-705</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>12/22/2025</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Larrea 370</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -5013,12 +5013,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>02013924</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -5040,51 +5040,47 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.402154</v>
+        <v>-58.471183</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.605295</v>
+        <v>-34.638988</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>CLI-D</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5099,7 +5095,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5126,47 +5122,51 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.471183</v>
+        <v>-58.46357</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.638988</v>
+        <v>-34.623187</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr"/>
+          <t>NRA-E</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7997</t>
+          <t>8061</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>FOREST AV. 957</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5181,12 +5181,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811453824</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5201,31 +5201,31 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.46357</v>
+        <v>-58.45732</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.623187</v>
+        <v>-34.581366</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>ATH-N</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5237,22 +5237,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>8061</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>FOREST AV. 957</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5267,12 +5267,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811453824</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5287,31 +5287,31 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L57" t="n">
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.45732</v>
+        <v>-58.459547</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.581366</v>
+        <v>-34.626309</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>ATH-N</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5323,22 +5323,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -5353,12 +5353,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5380,10 +5380,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.459547</v>
+        <v>-58.465166</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.626309</v>
+        <v>-34.670435</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5409,17 +5409,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5466,14 +5466,14 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.465166</v>
+        <v>-58.438399</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.670435</v>
+        <v>-34.663958</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5495,7 +5495,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5525,12 +5525,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5552,14 +5552,14 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.438399</v>
+        <v>-58.475565</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.663958</v>
+        <v>-34.660488</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5581,22 +5581,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5638,10 +5638,10 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.475565</v>
+        <v>-58.460855</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.660488</v>
+        <v>-34.631046</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5667,22 +5667,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5697,12 +5697,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5724,10 +5724,10 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.460855</v>
+        <v>-58.479751</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.631046</v>
+        <v>-34.677211</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5753,7 +5753,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5763,12 +5763,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5810,36 +5810,36 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.479751</v>
+        <v>-58.491573</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.677211</v>
+        <v>-34.639215</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5849,7 +5849,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5896,10 +5896,10 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.491573</v>
+        <v>-58.487715</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.639215</v>
+        <v>-34.636671</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -5925,22 +5925,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>8125</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/2/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5955,12 +5955,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811626981</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5982,51 +5982,51 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.487715</v>
+        <v>-58.423058</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.636671</v>
+        <v>-34.608916</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>ALM-E</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>8125</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2/2/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811626981</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6068,14 +6068,14 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.423058</v>
+        <v>-58.481162</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.608916</v>
+        <v>-34.665875</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>ALM-E</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6097,22 +6097,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6154,14 +6154,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.481162</v>
+        <v>-58.413945</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.665875</v>
+        <v>-34.582774</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6183,7 +6183,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>8490</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Ugarteche 2816</t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>corroida inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6240,14 +6240,14 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.413945</v>
+        <v>-58.437739</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.582774</v>
+        <v>-34.638224</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>AGU-M</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6269,7 +6269,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>900009468810</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6279,12 +6279,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t xml:space="preserve">CUENCA 3033 </t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6299,12 +6299,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6319,31 +6319,31 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.437739</v>
+        <v>-58.494814</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.638224</v>
+        <v>-34.601905</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>DEV-B</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6355,22 +6355,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>900009468810</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUENCA 3033 </t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6405,31 +6405,31 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L70" t="n">
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.494814</v>
+        <v>-58.469878</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.601905</v>
+        <v>-34.626919</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>DEV-B</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6441,17 +6441,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6471,12 +6471,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6498,10 +6498,10 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.469878</v>
+        <v>-58.46026</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.626919</v>
+        <v>-34.640706</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6527,22 +6527,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6557,12 +6557,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6584,10 +6584,10 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.46026</v>
+        <v>-58.480708</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.640706</v>
+        <v>-34.667639</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6613,7 +6613,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6623,12 +6623,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6643,7 +6643,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -6670,36 +6670,36 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.480708</v>
+        <v>-58.474151</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.667639</v>
+        <v>-34.630046</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>NRA-R</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2NRA</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>S00552343</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6709,12 +6709,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6729,12 +6729,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada base corroida</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6744,63 +6744,63 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L74" t="n">
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.474151</v>
+        <v>-58.464382</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.630046</v>
+        <v>-34.683083</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>NRA-R</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>S00176142</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>CULPINA 533</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>inclinada base corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6835,17 +6835,17 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L75" t="n">
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.464382</v>
+        <v>-58.464205</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.683083</v>
+        <v>-34.636221</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6859,34 +6859,30 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PAV-U</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6906,7 +6902,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6916,59 +6912,63 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L76" t="n">
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.464205</v>
+        <v>-58.517269</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.636221</v>
+        <v>-34.639879</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R76" t="inlineStr"/>
+          <t>PAV-B</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>-772</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t>LA PLATA AV. 2304</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>Desplazar Columna</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7003,31 +7003,31 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L77" t="n">
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.517269</v>
+        <v>-58.423086</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.639879</v>
+        <v>-34.641356</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>PAV-B</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7039,22 +7039,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>-774</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>CASEROS AV. 4131</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>mover a 4111</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -7096,10 +7096,10 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.423086</v>
+        <v>-58.422741</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.641356</v>
+        <v>-34.639999</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -7125,22 +7125,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>-774</t>
+          <t>8597</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CASEROS AV. 4131</t>
+          <t>JUJUY AV 1717</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7153,14 +7153,10 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>mover a 4111</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7182,14 +7178,14 @@
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.422741</v>
+        <v>-58.400922</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.639999</v>
+        <v>-34.630312</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -7199,7 +7195,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>PPT-F</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7211,22 +7207,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>8597</t>
+          <t xml:space="preserve">7460 </t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>3/13/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>JUJUY AV 1717</t>
+          <t>TERRADA 2720</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7242,12 +7238,12 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>RIENDA A PIQUE CORTADA</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -7257,31 +7253,31 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.400922</v>
+        <v>-58.486103</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.630312</v>
+        <v>-34.603895</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>PPT-F</t>
+          <t>NRA-P</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7293,7 +7289,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">7460 </t>
+          <t>00000609</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7303,12 +7299,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>TERRADA 2720</t>
+          <t>ZELADA 4402</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7324,12 +7320,12 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>RIENDA A PIQUE CORTADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -7339,21 +7335,21 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.486103</v>
+        <v>-58.48834</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.603895</v>
+        <v>-34.641018</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -7363,34 +7359,34 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>00000609</t>
+          <t>R0050</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/25/2026</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ZELADA 4402</t>
+          <t>IBERA 3244</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7428,14 +7424,14 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>-58.48834</v>
+        <v>-58.472542</v>
       </c>
       <c r="N82" t="n">
-        <v>-34.641018</v>
+        <v>-34.55798</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -7445,12 +7441,12 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-25 17:12:09)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R82"/>
+  <dimension ref="A1:R81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5151,22 +5151,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8061</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>FOREST AV. 957</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5181,12 +5181,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811453824</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5201,31 +5201,31 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.45732</v>
+        <v>-58.459547</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.581366</v>
+        <v>-34.626309</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>ATH-N</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5237,22 +5237,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5267,12 +5267,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5294,10 +5294,10 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.459547</v>
+        <v>-58.465166</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.626309</v>
+        <v>-34.670435</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5323,17 +5323,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5353,12 +5353,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5380,14 +5380,14 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.465166</v>
+        <v>-58.438399</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.670435</v>
+        <v>-34.663958</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5409,7 +5409,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5466,14 +5466,14 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.438399</v>
+        <v>-58.475565</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.663958</v>
+        <v>-34.660488</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5495,22 +5495,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5552,10 +5552,10 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.475565</v>
+        <v>-58.460855</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.660488</v>
+        <v>-34.631046</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5569,7 +5569,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5581,22 +5581,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5638,10 +5638,10 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.460855</v>
+        <v>-58.479751</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.631046</v>
+        <v>-34.677211</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5667,7 +5667,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5677,12 +5677,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5697,12 +5697,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5724,36 +5724,36 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.479751</v>
+        <v>-58.491573</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.677211</v>
+        <v>-34.639215</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5763,7 +5763,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5810,10 +5810,10 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.491573</v>
+        <v>-58.487715</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.639215</v>
+        <v>-34.636671</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -5839,22 +5839,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>8125</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/2/2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811626981</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5896,51 +5896,51 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.487715</v>
+        <v>-58.423058</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.636671</v>
+        <v>-34.608916</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>ALM-E</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8125</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2/2/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5955,12 +5955,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>811626981</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5982,14 +5982,14 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.423058</v>
+        <v>-58.481162</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.608916</v>
+        <v>-34.665875</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>ALM-E</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6011,22 +6011,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6068,14 +6068,14 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.481162</v>
+        <v>-58.413945</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.665875</v>
+        <v>-34.582774</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6097,7 +6097,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>8490</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6107,12 +6107,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Ugarteche 2816</t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>corroida inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6154,14 +6154,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.413945</v>
+        <v>-58.437739</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.582774</v>
+        <v>-34.638224</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>AGU-M</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6183,7 +6183,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>900009468810</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t xml:space="preserve">CUENCA 3033 </t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6233,31 +6233,31 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L68" t="n">
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.437739</v>
+        <v>-58.494814</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.638224</v>
+        <v>-34.601905</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>DEV-B</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6269,22 +6269,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>900009468810</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUENCA 3033 </t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6299,12 +6299,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6319,31 +6319,31 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.494814</v>
+        <v>-58.469878</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.601905</v>
+        <v>-34.626919</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>DEV-B</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6355,17 +6355,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6412,10 +6412,10 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.469878</v>
+        <v>-58.46026</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.626919</v>
+        <v>-34.640706</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6441,22 +6441,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6471,12 +6471,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6498,10 +6498,10 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.46026</v>
+        <v>-58.480708</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.640706</v>
+        <v>-34.667639</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6537,12 +6537,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6584,36 +6584,36 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.480708</v>
+        <v>-58.474151</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.667639</v>
+        <v>-34.630046</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>NRA-R</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2NRA</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>S00552343</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6623,12 +6623,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6643,12 +6643,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada base corroida</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6658,63 +6658,63 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L73" t="n">
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.474151</v>
+        <v>-58.464382</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.630046</v>
+        <v>-34.683083</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>NRA-R</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>S00176142</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>CULPINA 533</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>inclinada base corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6749,17 +6749,17 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L74" t="n">
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.464382</v>
+        <v>-58.464205</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.683083</v>
+        <v>-34.636221</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -6773,34 +6773,30 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PAV-U</t>
-        </is>
-      </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6820,7 +6816,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6830,59 +6826,63 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L75" t="n">
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.464205</v>
+        <v>-58.517269</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.636221</v>
+        <v>-34.639879</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr"/>
+          <t>PAV-B</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>-772</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t>LA PLATA AV. 2304</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>Desplazar Columna</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6917,31 +6917,31 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L76" t="n">
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.517269</v>
+        <v>-58.423086</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.639879</v>
+        <v>-34.641356</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PAV-B</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6953,22 +6953,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>-774</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>CASEROS AV. 4131</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>mover a 4111</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7010,10 +7010,10 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.423086</v>
+        <v>-58.422741</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.641356</v>
+        <v>-34.639999</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -7039,22 +7039,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>-774</t>
+          <t>8597</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CASEROS AV. 4131</t>
+          <t>JUJUY AV 1717</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7067,14 +7067,10 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
+      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>mover a 4111</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -7096,14 +7092,14 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.422741</v>
+        <v>-58.400922</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.639999</v>
+        <v>-34.630312</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -7113,7 +7109,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>PPT-F</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7125,22 +7121,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>8597</t>
+          <t xml:space="preserve">7460 </t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>3/13/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>JUJUY AV 1717</t>
+          <t>TERRADA 2720</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7156,12 +7152,12 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>RIENDA A PIQUE CORTADA</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -7171,31 +7167,31 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.400922</v>
+        <v>-58.486103</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.630312</v>
+        <v>-34.603895</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PPT-F</t>
+          <t>NRA-P</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7207,7 +7203,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">7460 </t>
+          <t>00000609</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7217,12 +7213,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TERRADA 2720</t>
+          <t>ZELADA 4402</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7238,12 +7234,12 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>RIENDA A PIQUE CORTADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -7253,21 +7249,21 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.486103</v>
+        <v>-58.48834</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.603895</v>
+        <v>-34.641018</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7277,34 +7273,34 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>00000609</t>
+          <t>R0050</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/25/2026</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ZELADA 4402</t>
+          <t>IBERA 3244</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7342,14 +7338,14 @@
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.48834</v>
+        <v>-58.472542</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.641018</v>
+        <v>-34.55798</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -7359,92 +7355,10 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
-        <is>
-          <t>ARATO-25058.PO.2PCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>R0050</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>3/25/2026</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>IBERA 3244</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L82" t="n">
-        <v>1</v>
-      </c>
-      <c r="M82" t="n">
-        <v>-58.472542</v>
-      </c>
-      <c r="N82" t="n">
-        <v>-34.55798</v>
-      </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>Saavedra</t>
-        </is>
-      </c>
-      <c r="P82" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q82" t="inlineStr">
-        <is>
-          <t>COG-L</t>
-        </is>
-      </c>
-      <c r="R82" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-27 12:53:19)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R81"/>
+  <dimension ref="A1:R82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7203,7 +7203,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>00000609</t>
+          <t>00201041</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7213,12 +7213,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ZELADA 4402</t>
+          <t>HABANA 4448</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7234,7 +7234,7 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DEMONTAR POSTE Y REEMPLAZAR POR COLUMNA</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7256,14 +7256,14 @@
         <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.48834</v>
+        <v>-58.518808</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.641018</v>
+        <v>-34.601236</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7273,34 +7273,34 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PUE-P</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>R0050</t>
+          <t>00000609</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>3/25/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>IBERA 3244</t>
+          <t>ZELADA 4402</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7338,27 +7338,109 @@
         <v>1</v>
       </c>
       <c r="M81" t="n">
+        <v>-58.48834</v>
+      </c>
+      <c r="N81" t="n">
+        <v>-34.641018</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>PCH-S</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>R0050</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>3/25/2026</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>IBERA 3244</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>1</v>
+      </c>
+      <c r="M82" t="n">
         <v>-58.472542</v>
       </c>
-      <c r="N81" t="n">
+      <c r="N82" t="n">
         <v>-34.55798</v>
       </c>
-      <c r="O81" t="inlineStr">
+      <c r="O82" t="inlineStr">
         <is>
           <t>Saavedra</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="P82" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q81" t="inlineStr">
+      <c r="Q82" t="inlineStr">
         <is>
           <t>COG-L</t>
         </is>
       </c>
-      <c r="R81" t="inlineStr">
+      <c r="R82" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-28 12:28:40)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R82"/>
+  <dimension ref="A1:R83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2403,27 +2403,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>7570</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10/13/2025</t>
+          <t>10/6/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2433,12 +2433,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810333018</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R150 o R200</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2460,10 +2460,10 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.46138</v>
+        <v>-58.465176</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.629774</v>
+        <v>-34.680979</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2489,17 +2489,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7516</t>
+          <t>7595</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/13/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ALVAREZ, CRISOSTOMO 3000</t>
+          <t>FALCON, RAMON L.,CNEL. 2353</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>810333018</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2546,10 +2546,10 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.458516</v>
+        <v>-58.46138</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.646422</v>
+        <v>-34.629774</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2575,7 +2575,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7735</t>
+          <t>7516</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2585,12 +2585,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GARCIA, MARTIN AV. 772</t>
+          <t>ALVAREZ, CRISOSTOMO 3000</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>810371042</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2632,14 +2632,14 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.374086</v>
+        <v>-58.458516</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.633168</v>
+        <v>-34.646422</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2649,29 +2649,29 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CON-B</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>ARATO-25058.AF.1CON</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7735</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SAENZ AV. 1204</t>
+          <t>GARCIA, MARTIN AV. 772</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>810416653</t>
+          <t>810371042</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2718,10 +2718,10 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.416237</v>
+        <v>-58.374086</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.65477</v>
+        <v>-34.633168</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2735,34 +2735,34 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>PPT-H</t>
+          <t>CON-B</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.AF.1CON</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7556</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SANCHEZ DE LORIA 1923</t>
+          <t>SAENZ AV. 1204</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>810416656</t>
+          <t>810416653</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2804,10 +2804,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.411426</v>
+        <v>-58.416237</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.633266</v>
+        <v>-34.65477</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>PPT-Q</t>
+          <t>PPT-H</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2833,22 +2833,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7579</t>
+          <t>7556</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10/22/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AGUIRRE 508</t>
+          <t>SANCHEZ DE LORIA 1923</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>810421912</t>
+          <t>810416656</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>cambiar</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2883,21 +2883,21 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.435731</v>
+        <v>-58.411426</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.597659</v>
+        <v>-34.633266</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PPT-Q</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2919,22 +2919,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7631</t>
+          <t>7579</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/22/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CALVO, CARLOS 3762</t>
+          <t>AGUIRRE 508</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>810451584</t>
+          <t>810421912</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2969,21 +2969,21 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.418542</v>
+        <v>-58.435731</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.624609</v>
+        <v>-34.597659</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3005,7 +3005,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>7631</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3015,12 +3015,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>CALVO, CARLOS 3762</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>810451584</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3062,14 +3062,14 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.430613</v>
+        <v>-58.418542</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.608805</v>
+        <v>-34.624609</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3091,7 +3091,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3101,12 +3101,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3148,24 +3148,24 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.50161</v>
+        <v>-58.430613</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.647648</v>
+        <v>-34.608805</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3177,22 +3177,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7643</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/28/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ACEVEDO 524</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>810458896</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3234,24 +3234,24 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.439164</v>
+        <v>-58.50161</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.597069</v>
+        <v>-34.647648</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3263,7 +3263,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7665</t>
+          <t>7643</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3273,12 +3273,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ARAOZ 2313</t>
+          <t>ACEVEDO 524</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>01450977</t>
+          <t>810458896</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Picada y cable cortado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3320,10 +3320,10 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.417634</v>
+        <v>-58.439164</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.587439</v>
+        <v>-34.597069</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>VCR-G</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3349,22 +3349,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>7665</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>ARAOZ 2313</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>01450977</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Picada y cable cortado</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3406,24 +3406,24 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.48121</v>
+        <v>-58.417634</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.61126</v>
+        <v>-34.587439</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>VCR-G</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3435,7 +3435,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7719</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3445,12 +3445,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ 180</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>01229656</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Colocar R400 para traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3492,24 +3492,24 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.440031</v>
+        <v>-58.48121</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.575409</v>
+        <v>-34.61126</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>COG-B</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3521,7 +3521,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7732</t>
+          <t>7719</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3531,12 +3531,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LINIERS VIRREY 1142</t>
+          <t>CIUDAD DE LA PAZ 180</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3551,12 +3551,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>810487035</t>
+          <t>01229656</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R400 para traspaso</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3578,14 +3578,14 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.413563</v>
+        <v>-58.440031</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.624645</v>
+        <v>-34.575409</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>CEN-P</t>
+          <t>COG-B</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3607,22 +3607,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7744</t>
+          <t>7732</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/31/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NECOCHEA 369</t>
+          <t>LINIERS VIRREY 1142</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>01233359</t>
+          <t>810487035</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Colocar R200 para rtaspaso de nodo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3664,14 +3664,14 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.364132</v>
+        <v>-58.413563</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.628423</v>
+        <v>-34.624645</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>CON-F</t>
+          <t>CEN-P</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3693,22 +3693,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7829</t>
+          <t>7744</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>10/31/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>NECOCHEA 369</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>01233359</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R200 para rtaspaso de nodo</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3750,14 +3750,14 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.460356</v>
+        <v>-58.364132</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.630793</v>
+        <v>-34.628423</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>CON-F</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3779,22 +3779,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/4/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 1654</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810573618</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Columna picada e inclinada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3836,14 +3836,14 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.389676</v>
+        <v>-58.460356</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.618127</v>
+        <v>-34.630793</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>CEN-?</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3865,22 +3865,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7604</t>
+          <t>7780</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/4/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 3741</t>
+          <t>INDEPENDENCIA AV. 1654</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3895,12 +3895,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810712796</t>
+          <t>810573618</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Columna picada e inclinada</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3922,14 +3922,14 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.418108</v>
+        <v>-58.389676</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.62564</v>
+        <v>-34.618127</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>ALM-A</t>
+          <t>CEN-?</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3951,7 +3951,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>7604</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3961,12 +3961,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t>SAN JUAN AV. 3741</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810712796</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4008,14 +4008,14 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.433855</v>
+        <v>-58.418108</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.614487</v>
+        <v>-34.62564</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-A</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4037,22 +4037,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7842</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FERRARI 410</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810713039</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4094,24 +4094,24 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.441198</v>
+        <v>-58.433855</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.605341</v>
+        <v>-34.614487</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4123,22 +4123,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t>7842</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t>FERRARI 410</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810713039</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>columna inclinada base corroida</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4180,24 +4180,24 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.439239</v>
+        <v>-58.441198</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.6604</v>
+        <v>-34.605341</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4209,7 +4209,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S01140678</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4219,12 +4219,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>810804375</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>columna inclinada corroida</t>
+          <t>columna inclinada base corroida</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4266,10 +4266,10 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.388529</v>
+        <v>-58.439239</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.655949</v>
+        <v>-34.6604</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>CON-I</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4295,22 +4295,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t>S01140678</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t xml:space="preserve"> VELEZ SARSFIELD AV. 1722</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4325,12 +4325,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>810804375</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>columna inclinada corroida</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4352,24 +4352,24 @@
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.491325</v>
+        <v>-58.388529</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.647761</v>
+        <v>-34.655949</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>CON-I</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4381,7 +4381,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4391,12 +4391,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4411,12 +4411,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4438,24 +4438,24 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.469394</v>
+        <v>-58.491325</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.626925</v>
+        <v>-34.647761</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4467,22 +4467,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7892</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>12/1/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Juncal 1642</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4497,12 +4497,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">01749376 </t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4524,14 +4524,14 @@
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.390974</v>
+        <v>-58.469394</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.594177</v>
+        <v>-34.626925</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>RET-N</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4553,22 +4553,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7961</t>
+          <t>7892</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12/2/2025</t>
+          <t>12/1/2025</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CASTILLO 12</t>
+          <t>Juncal 1642</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>810984643</t>
+          <t xml:space="preserve">01749376 </t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4598,26 +4598,26 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.430396</v>
+        <v>-58.390974</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.599668</v>
+        <v>-34.594177</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>RET-N</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4639,22 +4639,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7898</t>
+          <t>7961</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>12/4/2025</t>
+          <t>12/2/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BONIFACIO, JOSE 2319</t>
+          <t>CASTILLO 12</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>810984687</t>
+          <t>810984643</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4689,21 +4689,21 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.459955</v>
+        <v>-58.430396</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.631973</v>
+        <v>-34.599668</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4725,22 +4725,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S01204545</t>
+          <t>7898</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>12/10/2025</t>
+          <t>12/4/2025</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Medina 420</t>
+          <t>BONIFACIO, JOSE 2319</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4755,12 +4755,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t>810984687</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4782,51 +4782,51 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.48802</v>
+        <v>-58.459955</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.641075</v>
+        <v>-34.631973</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t>S01204545</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>12/10/2025</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t>Medina 420</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4841,12 +4841,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4868,51 +4868,51 @@
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.463198</v>
+        <v>-58.48802</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.62624</v>
+        <v>-34.641075</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>-705</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>12/22/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Larrea 370</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4927,12 +4927,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>02013924</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4954,14 +4954,14 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.402154</v>
+        <v>-58.463198</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.605295</v>
+        <v>-34.62624</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>CLI-D</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4983,22 +4983,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t>-705</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>12/22/2025</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t>Larrea 370</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -5013,12 +5013,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>02013924</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -5040,47 +5040,51 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.471183</v>
+        <v>-58.402154</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.638988</v>
+        <v>-34.605295</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr"/>
+          <t>CLI-D</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>7997</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5095,7 +5099,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5122,46 +5126,42 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.46357</v>
+        <v>-58.471183</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.623187</v>
+        <v>-34.638988</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>NRA-E</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5208,10 +5208,10 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.459547</v>
+        <v>-58.46357</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.626309</v>
+        <v>-34.623187</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5237,22 +5237,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5267,12 +5267,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5294,10 +5294,10 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.465166</v>
+        <v>-58.459547</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.670435</v>
+        <v>-34.626309</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5323,17 +5323,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5353,12 +5353,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>chocada</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5380,14 +5380,14 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.438399</v>
+        <v>-58.465166</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.663958</v>
+        <v>-34.670435</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5409,7 +5409,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>chocada</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5466,14 +5466,14 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.475565</v>
+        <v>-58.438399</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.660488</v>
+        <v>-34.663958</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5495,22 +5495,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5552,10 +5552,10 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.460855</v>
+        <v>-58.475565</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.631046</v>
+        <v>-34.660488</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5569,7 +5569,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5581,22 +5581,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5638,10 +5638,10 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.479751</v>
+        <v>-58.460855</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.677211</v>
+        <v>-34.631046</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5667,7 +5667,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S01447367</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5677,12 +5677,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>MOZART 216</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5697,12 +5697,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5724,36 +5724,36 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.491573</v>
+        <v>-58.479751</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.639215</v>
+        <v>-34.677211</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>S01447367</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5763,7 +5763,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>MOZART 216</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5810,10 +5810,10 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.487715</v>
+        <v>-58.491573</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.636671</v>
+        <v>-34.639215</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -5839,22 +5839,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>8125</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2/2/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>811626981</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5896,51 +5896,51 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.423058</v>
+        <v>-58.487715</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.608916</v>
+        <v>-34.636671</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>ALM-E</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>8125</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>2/2/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>ACUÑA DE FIGUEROA, FRANCISCO 180</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5955,12 +5955,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>811626981</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5982,14 +5982,14 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.481162</v>
+        <v>-58.423058</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.665875</v>
+        <v>-34.608916</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>ALM-E</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6011,22 +6011,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>8490</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Ugarteche 2816</t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>811627090</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>corroida inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6068,14 +6068,14 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.413945</v>
+        <v>-58.481162</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.582774</v>
+        <v>-34.665875</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>AGU-M</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6097,7 +6097,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>8490</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6107,12 +6107,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t>Ugarteche 2816</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>811627090</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>corroida inclinada</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6154,14 +6154,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.437739</v>
+        <v>-58.413945</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.638224</v>
+        <v>-34.582774</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>AGU-M</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6183,7 +6183,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>900009468810</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUENCA 3033 </t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>tensor roto</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6233,31 +6233,31 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L68" t="n">
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.494814</v>
+        <v>-58.437739</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.601905</v>
+        <v>-34.638224</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>DEV-B</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6269,22 +6269,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>900009468810</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t xml:space="preserve">CUENCA 3033 </t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6299,12 +6299,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>tensor roto</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6319,31 +6319,31 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.469878</v>
+        <v>-58.494814</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.626919</v>
+        <v>-34.601905</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>DEV-B</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6355,17 +6355,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6412,10 +6412,10 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.46026</v>
+        <v>-58.469878</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.640706</v>
+        <v>-34.626919</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6441,22 +6441,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6471,12 +6471,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6498,10 +6498,10 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.480708</v>
+        <v>-58.46026</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.667639</v>
+        <v>-34.640706</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6537,12 +6537,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6584,36 +6584,36 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.474151</v>
+        <v>-58.480708</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.630046</v>
+        <v>-34.667639</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>NRA-R</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6623,12 +6623,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6643,12 +6643,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>inclinada base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6658,63 +6658,63 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L73" t="n">
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.464382</v>
+        <v>-58.474151</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.683083</v>
+        <v>-34.630046</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>NRA-R</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2NRA</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>S00552343</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada base corroida</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6749,17 +6749,17 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L74" t="n">
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.464205</v>
+        <v>-58.464382</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.636221</v>
+        <v>-34.683083</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -6773,30 +6773,34 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R74" t="inlineStr"/>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>S00176142</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t>CULPINA 533</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6816,7 +6820,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>columna inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6826,63 +6830,59 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L75" t="n">
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.517269</v>
+        <v>-58.464205</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.639879</v>
+        <v>-34.636221</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PAV-B</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>columna inclinada</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6917,31 +6917,31 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L76" t="n">
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.423086</v>
+        <v>-58.517269</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.641356</v>
+        <v>-34.639879</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>PAV-B</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6953,22 +6953,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>-774</t>
+          <t>-772</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CASEROS AV. 4131</t>
+          <t>LA PLATA AV. 2304</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>mover a 4111</t>
+          <t>Desplazar Columna</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7010,10 +7010,10 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.422741</v>
+        <v>-58.423086</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.639999</v>
+        <v>-34.641356</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -7039,22 +7039,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>8597</t>
+          <t>-774</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3/13/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>JUJUY AV 1717</t>
+          <t>CASEROS AV. 4131</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7067,10 +7067,14 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>mover a 4111</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -7092,14 +7096,14 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.400922</v>
+        <v>-58.422741</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.630312</v>
+        <v>-34.639999</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -7109,7 +7113,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>PPT-F</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7121,22 +7125,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">7460 </t>
+          <t>8597</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>TERRADA 2720</t>
+          <t>JUJUY AV 1717</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7152,12 +7156,12 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>RIENDA A PIQUE CORTADA</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -7167,31 +7171,31 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.486103</v>
+        <v>-58.400922</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.603895</v>
+        <v>-34.630312</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>PPT-F</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7203,7 +7207,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>00201041</t>
+          <t xml:space="preserve">7460 </t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7213,7 +7217,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>HABANA 4448</t>
+          <t>TERRADA 2720</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7234,12 +7238,12 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>DEMONTAR POSTE Y REEMPLAZAR POR COLUMNA</t>
+          <t>RIENDA A PIQUE CORTADA</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -7249,17 +7253,17 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.518808</v>
+        <v>-58.486103</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.601236</v>
+        <v>-34.603895</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -7273,7 +7277,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>NRA-P</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7285,7 +7289,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>00000609</t>
+          <t>00201041</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7295,12 +7299,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ZELADA 4402</t>
+          <t>HABANA 4448</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7316,7 +7320,7 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DEMONTAR POSTE Y REEMPLAZAR POR COLUMNA</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -7338,14 +7342,14 @@
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.48834</v>
+        <v>-58.518808</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.641018</v>
+        <v>-34.601236</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -7355,34 +7359,34 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PUE-P</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>R0050</t>
+          <t>00000609</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>3/25/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>IBERA 3244</t>
+          <t>ZELADA 4402</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7420,27 +7424,109 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
+        <v>-58.48834</v>
+      </c>
+      <c r="N82" t="n">
+        <v>-34.641018</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>PCH-S</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>R0050</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>3/25/2026</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>IBERA 3244</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>1</v>
+      </c>
+      <c r="M83" t="n">
         <v>-58.472542</v>
       </c>
-      <c r="N82" t="n">
+      <c r="N83" t="n">
         <v>-34.55798</v>
       </c>
-      <c r="O82" t="inlineStr">
+      <c r="O83" t="inlineStr">
         <is>
           <t>Saavedra</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr">
+      <c r="P83" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q82" t="inlineStr">
+      <c r="Q83" t="inlineStr">
         <is>
           <t>COG-L</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr">
+      <c r="R83" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-27 14:49:38)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -1449,22 +1449,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>807044223</t>
+          <t>807044233</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5/22/2025</t>
+          <t>5/29/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cucha Cucha 2918</t>
+          <t>Martin Grandoli 5761</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1479,17 +1479,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>807044223</t>
+          <t xml:space="preserve">ICD30261461 </t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Aplomar</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1499,53 +1499,53 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L13" t="n">
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>-58.469783</v>
+        <v>-58.487144</v>
       </c>
       <c r="N13" t="n">
-        <v>-34.599214</v>
+        <v>-34.669078</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NRA-F</t>
+          <t>PAV-L</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.1NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>807044233</t>
+          <t>5948</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>5/29/2025</t>
+          <t>6/2/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Martin Grandoli 5761</t>
+          <t>MURGUIONDO 3990</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1565,17 +1565,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICD30261461 </t>
+          <t>807129347</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1585,17 +1585,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>-58.487144</v>
+        <v>-58.477944</v>
       </c>
       <c r="N14" t="n">
-        <v>-34.669078</v>
+        <v>-34.675149</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>PAV-L</t>
+          <t>PAV-V</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1621,22 +1621,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5948</t>
+          <t>-506</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6/2/2025</t>
+          <t>7/11/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MURGUIONDO 3990</t>
+          <t>Espinosa 591</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1651,12 +1651,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>807129347</t>
+          <t>808150511</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1666,22 +1666,22 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>-58.477944</v>
+        <v>-58.449</v>
       </c>
       <c r="N15" t="n">
-        <v>-34.675149</v>
+        <v>-34.616077</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>PAV-V</t>
+          <t>NRA-B</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1707,22 +1707,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>-506</t>
+          <t>-539</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7/11/2025</t>
+          <t>7/31/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Espinosa 591</t>
+          <t>Tejedor 1097</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>808150511</t>
+          <t>808615951</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1752,22 +1752,22 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L16" t="n">
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>-58.449</v>
+        <v>-58.440748</v>
       </c>
       <c r="N16" t="n">
-        <v>-34.616077</v>
+        <v>-34.63245</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NRA-B</t>
+          <t>PPT-P</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1793,7 +1793,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>-539</t>
+          <t>-540</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tejedor 1097</t>
+          <t>Tejedor 1071</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>808615951</t>
+          <t>808615948</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1843,17 +1843,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L17" t="n">
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.440748</v>
+        <v>-58.44037</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.63245</v>
+        <v>-34.632249</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>-540</t>
+          <t>6556</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7/31/2025</t>
+          <t>8/4/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tejedor 1071</t>
+          <t>2 DE ABRIL DE 1982 6982</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1909,17 +1909,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>808615948</t>
+          <t>03534653</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>DESMONTAR POSTE Y TRASPASAR  RED</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1929,17 +1929,17 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.44037</v>
+        <v>-58.494864</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.632249</v>
+        <v>-34.678826</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>PPT-P</t>
+          <t>PAV-M</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1965,22 +1965,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6556</t>
+          <t>5625</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>8/4/2025</t>
+          <t>8/20/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2 DE ABRIL DE 1982 6982</t>
+          <t>ACOYTE AV. 184</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1995,17 +1995,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>03534653</t>
+          <t>809065913</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y TRASPASAR  RED</t>
+          <t>Inclinada ver cambio</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2015,21 +2015,21 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.494864</v>
+        <v>-58.437583</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.678826</v>
+        <v>-34.616231</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>PAV-M</t>
+          <t>ALM-H</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2051,17 +2051,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5625</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>8/20/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ACOYTE AV. 184</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2081,12 +2081,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>809065913</t>
+          <t>ICD30508311</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Inclinada ver cambio</t>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2108,14 +2108,14 @@
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.437583</v>
+        <v>-58.435017</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.616231</v>
+        <v>-34.622044</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ALM-H</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2137,17 +2137,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2167,12 +2167,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>ICD30593982</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2194,10 +2194,10 @@
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.435017</v>
+        <v>-58.443232</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.622044</v>
+        <v>-34.620007</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2223,17 +2223,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>7102</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>8/30/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>AMBERES 995</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pendiente de Traspaso PROPIO</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2253,12 +2253,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>809309598</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2268,22 +2268,22 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.443232</v>
+        <v>-58.453382</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.620007</v>
+        <v>-34.612707</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>NRA-I</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2309,17 +2309,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7102</t>
+          <t>-586</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>8/30/2025</t>
+          <t>9/8/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMBERES 995</t>
+          <t>Franklin 666</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2339,17 +2339,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>809309598</t>
+          <t>ICD30709119</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspasar redes a la columna de telecentro y desmontar la picada</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2366,14 +2366,14 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.453382</v>
+        <v>-58.441362</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.612707</v>
+        <v>-34.607784</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NRA-I</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2395,17 +2395,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>-586</t>
+          <t>-601</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>9/8/2025</t>
+          <t>9/18/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Franklin 666</t>
+          <t>Pedro Goyena 1216</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2425,17 +2425,17 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ICD30709119</t>
+          <t>809837504</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Traspasar redes a la columna de telecentro y desmontar la picada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2452,14 +2452,14 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.441362</v>
+        <v>-58.444685</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.607784</v>
+        <v>-34.62711</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>PCH-D</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2481,22 +2481,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>-601</t>
+          <t>-611</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>9/18/2025</t>
+          <t>9/24/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pedro Goyena 1216</t>
+          <t>Lafuente 2606</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2511,12 +2511,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>809837504</t>
+          <t>809972807</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2538,14 +2538,14 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.444685</v>
+        <v>-58.444724</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.62711</v>
+        <v>-34.657961</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PCH-D</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2567,22 +2567,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>-611</t>
+          <t>7325</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>9/24/2025</t>
+          <t>9/26/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lafuente 2606</t>
+          <t>SALAS 596</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2597,12 +2597,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>809972807</t>
+          <t>810015422</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Cambio terminal</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2617,21 +2617,21 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.444724</v>
+        <v>-58.434543</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.657961</v>
+        <v>-34.632772</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2653,22 +2653,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7325</t>
+          <t>-626</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>9/26/2025</t>
+          <t>10/1/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SALAS 596</t>
+          <t>Soldado de la Frontera 5371</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2683,12 +2683,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>810015422</t>
+          <t>ICD31463420</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Cambio terminal</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2698,22 +2698,22 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.434543</v>
+        <v>-58.462371</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.632772</v>
+        <v>-34.687152</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2727,7 +2727,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>PAV-T</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2739,17 +2739,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>-626</t>
+          <t>7570</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/1/2025</t>
+          <t>10/6/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Soldado de la Frontera 5371</t>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>ICD31463420</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2796,10 +2796,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.462371</v>
+        <v>-58.465176</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.687152</v>
+        <v>-34.680979</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>PAV-T</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2825,17 +2825,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>7451</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>10/8/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>CORVALAN 3698</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pendiente de Traspaso PROPIO</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>810259135</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2870,22 +2870,22 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.465176</v>
+        <v>-58.46777</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.680979</v>
+        <v>-34.671445</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2899,7 +2899,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2911,17 +2911,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7451</t>
+          <t>943</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/8/2025</t>
+          <t>10/13/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CORVALAN 3698</t>
+          <t>BARCA CABO DE HORNOS 6899</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>810259135</t>
+          <t>810333113</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2968,10 +2968,10 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.46777</v>
+        <v>-58.491592</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.671445</v>
+        <v>-34.679774</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PAV-M</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2997,22 +2997,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>943</t>
+          <t>7516</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10/13/2025</t>
+          <t>10/15/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BARCA CABO DE HORNOS 6899</t>
+          <t>ALVAREZ, CRISOSTOMO 3000</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>810333113</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3047,17 +3047,17 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.491592</v>
+        <v>-58.458516</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.679774</v>
+        <v>-34.646422</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PAV-M</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3083,22 +3083,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7516</t>
+          <t>7624</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10/15/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ALVAREZ, CRISOSTOMO 3000</t>
+          <t>DIAZ VELEZ AV. 4516</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3113,12 +3113,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3140,14 +3140,14 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.458516</v>
+        <v>-58.430613</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.646422</v>
+        <v>-34.608805</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3169,22 +3169,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7624</t>
+          <t>-663</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>DIAZ VELEZ AV. 4516</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2693</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3199,12 +3199,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>01230744</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Picada con nodo teco</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3226,14 +3226,14 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.430613</v>
+        <v>-58.465679</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.608805</v>
+        <v>-34.63241</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3255,17 +3255,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>-663</t>
+          <t>8830</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>11/2/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2693</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2331</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3285,12 +3285,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>01230744</t>
+          <t>810526265</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Picada con nodo teco</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3300,7 +3300,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3312,10 +3312,10 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.465679</v>
+        <v>-58.460681</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.63241</v>
+        <v>-34.63089</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3341,7 +3341,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>8830</t>
+          <t>7829</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2331</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>810526265</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3398,10 +3398,10 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.460681</v>
+        <v>-58.460356</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.63089</v>
+        <v>-34.630793</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3427,22 +3427,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7829</t>
+          <t>7824</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11/2/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2309</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 1311</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>810712730</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3484,10 +3484,10 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.460356</v>
+        <v>-58.446763</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.630793</v>
+        <v>-34.624743</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PCH-I</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3513,7 +3513,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7824</t>
+          <t>7746</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 1311</t>
+          <t>CAMPICHUELO 229</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>810712730</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3570,14 +3570,14 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.446763</v>
+        <v>-58.433855</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.624743</v>
+        <v>-34.614487</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PCH-I</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3599,17 +3599,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7746</t>
+          <t>-672</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>11/13/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CAMPICHUELO 229</t>
+          <t>Federico Garcia Lorca 255</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>810734112</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Cambiar</t>
+          <t>Cambiar pasante</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3656,10 +3656,10 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.433855</v>
+        <v>-58.445239</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.614487</v>
+        <v>-34.618751</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>NRA-A</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3685,22 +3685,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>-672</t>
+          <t>S00073051</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11/13/2025</t>
+          <t>11/18/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Federico Garcia Lorca 255</t>
+          <t>Franklin 2427</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>810734112</t>
+          <t>TLC</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Cambiar pasante</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3739,17 +3739,17 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.445239</v>
+        <v>-58.468107</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.618751</v>
+        <v>-34.618068</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>NRA-A</t>
+          <t>NRA-D</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3771,22 +3771,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S00073051</t>
+          <t>S00958024</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/18/2025</t>
+          <t>11/19/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Franklin 2427</t>
+          <t>SAN PEDRITO 3010</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3801,12 +3801,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>TLC</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3825,17 +3825,17 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.468107</v>
+        <v>-58.439239</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.618068</v>
+        <v>-34.6604</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>NRA-D</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3857,22 +3857,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S00958024</t>
+          <t>7869</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11/19/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SAN PEDRITO 3010</t>
+          <t>BOGOTA 2770</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3887,12 +3887,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base picada</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3914,14 +3914,14 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.439239</v>
+        <v>-58.469394</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.6604</v>
+        <v>-34.626925</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3943,17 +3943,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>7869</t>
+          <t>-686</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>11/27/2025</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>BOGOTA 2770</t>
+          <t>Pumacahua 292</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3973,12 +3973,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>810862736</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>base picada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4000,10 +4000,10 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.469394</v>
+        <v>-58.453749</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.626925</v>
+        <v>-34.629882</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -4017,7 +4017,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PCH-A</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4029,17 +4029,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>-686</t>
+          <t>-703</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/27/2025</t>
+          <t>12/16/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Pumacahua 292</t>
+          <t>Calcena 211</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4059,12 +4059,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>810862736</t>
+          <t>811198653</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4086,10 +4086,10 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.453749</v>
+        <v>-58.456353</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.629882</v>
+        <v>-34.623684</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>PCH-A</t>
+          <t>NRA-C</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4115,17 +4115,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>-703</t>
+          <t>7929</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>12/16/2025</t>
+          <t>12/19/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Calcena 211</t>
+          <t>Riglos 957</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4145,12 +4145,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>811198653</t>
+          <t>811198753</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4172,10 +4172,10 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.456353</v>
+        <v>-58.435265</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.623684</v>
+        <v>-34.630164</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -4189,7 +4189,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>NRA-C</t>
+          <t>PPT-P</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4201,7 +4201,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>7929</t>
+          <t>7957</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Riglos 957</t>
+          <t>BACACAY 2357</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4231,12 +4231,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>811198753</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4258,10 +4258,10 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.435265</v>
+        <v>-58.463198</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.630164</v>
+        <v>-34.62624</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -4275,7 +4275,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>PPT-P</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4287,22 +4287,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>7957</t>
+          <t>7971</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>12/19/2025</t>
+          <t>12/23/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BACACAY 2357</t>
+          <t xml:space="preserve">GAONA AV. 1360 </t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4317,12 +4317,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>811238719</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4344,10 +4344,10 @@
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>-58.463198</v>
+        <v>-58.448401</v>
       </c>
       <c r="N46" t="n">
-        <v>-34.62624</v>
+        <v>-34.608681</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>NRA-B</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4373,7 +4373,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7971</t>
+          <t>6343</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAONA AV. 1360 </t>
+          <t>ESPINOSA 1099</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4403,12 +4403,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>811238719</t>
+          <t>811238674</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4423,17 +4423,17 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.448401</v>
+        <v>-58.452139</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.608681</v>
+        <v>-34.610772</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>NRA-B</t>
+          <t>NRA-H</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4459,17 +4459,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>6343</t>
+          <t>7995</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>12/23/2025</t>
+          <t>1/2/2026</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ESPINOSA 1099</t>
+          <t>ARANGUREN, JUAN F., DR. 462</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -4489,12 +4489,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>811238674</t>
+          <t>811299459</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4509,21 +4509,21 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.452139</v>
+        <v>-58.437431</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.610772</v>
+        <v>-34.612405</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NRA-H</t>
+          <t>ALM-I</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4545,7 +4545,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7995</t>
+          <t>7997</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4555,12 +4555,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 462</t>
+          <t>CARACAS 554</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>811299459</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4602,14 +4602,14 @@
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.437431</v>
+        <v>-58.46357</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.612405</v>
+        <v>-34.623187</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>ALM-I</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4631,17 +4631,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7997</t>
+          <t>S00982176</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CARACAS 554</t>
+          <t>GRANADEROS 110</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4688,10 +4688,10 @@
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.46357</v>
+        <v>-58.459547</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.623187</v>
+        <v>-34.626309</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4717,22 +4717,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S00982176</t>
+          <t>8123</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1/9/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>GRANADEROS 110</t>
+          <t>ACOYTE 908</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>811454448</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4774,14 +4774,14 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.459547</v>
+        <v>-58.440177</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.626309</v>
+        <v>-34.607612</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4803,7 +4803,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>8123</t>
+          <t>8127</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4813,12 +4813,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ACOYTE 908</t>
+          <t>ESCALADA AV. 3100</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4833,12 +4833,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811454448</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4860,14 +4860,14 @@
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.440177</v>
+        <v>-58.465166</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.607612</v>
+        <v>-34.670435</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4889,22 +4889,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>8127</t>
+          <t>8150</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1/14/2026</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ESCALADA AV. 3100</t>
+          <t>SAN JOSE DE CALASANZ 266</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4919,12 +4919,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>811497993</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4946,10 +4946,10 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.465166</v>
+        <v>-58.437998</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.670435</v>
+        <v>-34.62221</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PCH-K</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4975,22 +4975,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>8150</t>
+          <t>8211</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1/16/2026</t>
+          <t>1/26/2026</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SAN JOSE DE CALASANZ 266</t>
+          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -5005,12 +5005,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>811497993</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5032,14 +5032,14 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.437998</v>
+        <v>-58.438399</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.62221</v>
+        <v>-34.663958</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PCH-K</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5061,7 +5061,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>8211</t>
+          <t>8223</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RABANAL, FRANCISCO, INTENDENTE AV. 3085</t>
+          <t xml:space="preserve"> ESCALADA AV. 2421</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5118,14 +5118,14 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.438399</v>
+        <v>-58.475565</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.663958</v>
+        <v>-34.660488</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-P</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5147,22 +5147,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>-739</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>1/27/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESCALADA AV. 2421</t>
+          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5177,12 +5177,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5204,10 +5204,10 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.475565</v>
+        <v>-58.460855</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.660488</v>
+        <v>-34.631046</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PAV-P</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5233,22 +5233,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>-739</t>
+          <t>S01281615</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1/27/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ALBERDI, JUAN BAUTISTA AV. 2352</t>
+          <t>RUCCI, JOSE IGNACIO 4011</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5263,12 +5263,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5290,10 +5290,10 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.460855</v>
+        <v>-58.479751</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.631046</v>
+        <v>-34.677211</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5319,17 +5319,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S01281615</t>
+          <t>8270</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/3/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RUCCI, JOSE IGNACIO 4011</t>
+          <t>CASCO, HORACIO, DR. 5287</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5376,10 +5376,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.479751</v>
+        <v>-58.481162</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.677211</v>
+        <v>-34.665875</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5405,7 +5405,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>8270</t>
+          <t>8274</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5415,12 +5415,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CASCO, HORACIO, DR. 5287</t>
+          <t>RIGLOS 553</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5435,12 +5435,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -5462,10 +5462,10 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.481162</v>
+        <v>-58.436277</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.665875</v>
+        <v>-34.625202</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PCH-B</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5491,22 +5491,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>8274</t>
+          <t>S01421388</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2/3/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>RIGLOS 553</t>
+          <t>MITRE, EMILIO 1602</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -5548,10 +5548,10 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.436277</v>
+        <v>-58.437739</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.625202</v>
+        <v>-34.638224</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5565,7 +5565,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PCH-B</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5577,22 +5577,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S01421388</t>
+          <t>8121</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MITRE, EMILIO 1602</t>
+          <t>FRANKLIN 572</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5607,12 +5607,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>811627115</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5634,14 +5634,14 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.437739</v>
+        <v>-58.439651</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.638224</v>
+        <v>-34.607769</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PPT-S</t>
+          <t>ALM-O</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5663,17 +5663,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>8121</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/10/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FRANKLIN 572</t>
+          <t>ARENGREEN 1584</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -5693,12 +5693,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>811627115</t>
+          <t>812440072</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5713,21 +5713,21 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L62" t="n">
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.439651</v>
+        <v>-58.453265</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.607769</v>
+        <v>-34.615073</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>ALM-O</t>
+          <t>NRA-I</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5749,17 +5749,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>S00073317</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2/10/2026</t>
+          <t>2/11/2026</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ARENGREEN 1584</t>
+          <t xml:space="preserve"> ESPINOSA 82</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>812440072</t>
+          <t>812440077</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5799,17 +5799,17 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L63" t="n">
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.453265</v>
+        <v>-58.446397</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.615073</v>
+        <v>-34.621499</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>NRA-I</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5835,17 +5835,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S00073317</t>
+          <t>-752</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2/11/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ESPINOSA 82</t>
+          <t>RIVADAVIA AV. 5691</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>812440077</t>
+          <t>812440563</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5892,10 +5892,10 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.446397</v>
+        <v>-58.445685</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.621499</v>
+        <v>-34.622144</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -5921,7 +5921,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>-752</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5931,12 +5931,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 5691</t>
+          <t>TERRADA 402</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>812440563</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5978,10 +5978,10 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.445685</v>
+        <v>-58.469878</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.622144</v>
+        <v>-34.626919</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6007,17 +6007,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>S00086082</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>2/5/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>TERRADA 402</t>
+          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -6037,12 +6037,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6064,10 +6064,10 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.469878</v>
+        <v>-58.46026</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.626919</v>
+        <v>-34.640706</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -6081,7 +6081,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6093,22 +6093,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S00086082</t>
+          <t>8268</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2/5/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PRIMERA JUNTA 2899</t>
+          <t>MONTREAL 5391</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6123,12 +6123,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>inclinada corroida</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6150,10 +6150,10 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.46026</v>
+        <v>-58.480708</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.640706</v>
+        <v>-34.667639</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6179,7 +6179,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>8268</t>
+          <t>S00936659</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6189,12 +6189,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>MONTREAL 5391</t>
+          <t>FLORES, VENANCIO, GRAL. 3197</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6209,12 +6209,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6236,46 +6236,46 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.480708</v>
+        <v>-58.474151</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.667639</v>
+        <v>-34.630046</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>NRA-R</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2NRA</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>S00936659</t>
+          <t>S00115187</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/2/2026</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 3197</t>
+          <t>ESTADO PLURINACIONAL DE BOLIVIA 324</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6295,7 +6295,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>812503658</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -6322,51 +6322,51 @@
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.474151</v>
+        <v>-58.46673</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.630046</v>
+        <v>-34.627032</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NRA-R</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2NRA</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S00115187</t>
+          <t>S00552343</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>3/2/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ESTADO PLURINACIONAL DE BOLIVIA 324</t>
+          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6381,12 +6381,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>812503658</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6396,22 +6396,22 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L70" t="n">
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.46673</v>
+        <v>-58.464382</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.627032</v>
+        <v>-34.683083</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6437,22 +6437,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>S00176142</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/6/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>CULPINA 533</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6487,17 +6487,17 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L71" t="n">
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.464382</v>
+        <v>-58.464205</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.683083</v>
+        <v>-34.636221</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6511,34 +6511,30 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PAV-U</t>
-        </is>
-      </c>
-      <c r="R71" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>S00176142</t>
+          <t>8427</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>3/5/2026</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CULPINA 533</t>
+          <t xml:space="preserve">ESPINOSA 98 </t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6558,7 +6554,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base quebrada</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6568,7 +6564,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -6580,10 +6576,10 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.464205</v>
+        <v>-58.446457</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.636221</v>
+        <v>-34.621398</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -6597,30 +6593,34 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R72" t="inlineStr"/>
+          <t>PCH-G</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>8427</t>
+          <t>8424</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>3/5/2026</t>
+          <t>3/19/2026</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESPINOSA 98 </t>
+          <t>BONIFACIO JOSE 2319</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6635,12 +6635,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>812879799</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>base quebrada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6662,10 +6662,10 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.446457</v>
+        <v>-58.459955</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.621398</v>
+        <v>-34.631973</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6691,7 +6691,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>8424</t>
+          <t>8422</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6701,12 +6701,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BONIFACIO JOSE 2319</t>
+          <t>RIVADAVIA AV 5764</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6721,12 +6721,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>812879799</t>
+          <t>812879872</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6748,10 +6748,10 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.459955</v>
+        <v>-58.446644</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.631973</v>
+        <v>-34.622863</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -6765,7 +6765,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PCH-I</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6777,7 +6777,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>8422</t>
+          <t>00191122</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -6787,12 +6787,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV 5764</t>
+          <t>SAN PEDRITO AV 384</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>812879872</t>
+          <t>812879887</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -6834,10 +6834,10 @@
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.446644</v>
+        <v>-58.467504</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.622863</v>
+        <v>-34.635231</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6851,7 +6851,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PCH-I</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -6863,17 +6863,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>00191122</t>
+          <t xml:space="preserve">8642   </t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3/19/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SAN PEDRITO AV 384</t>
+          <t>CALCENA 347</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -6893,17 +6893,17 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>812879887</t>
+          <t>812879950</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>DESMONTAR COLUMNA Y MIGRAR RED A COLUMNA ALEDAÑA</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -6920,10 +6920,10 @@
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.467504</v>
+        <v>-58.457348</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.635231</v>
+        <v>-34.622249</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -6937,7 +6937,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>NRA-C</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6949,17 +6949,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">8642   </t>
+          <t>8795</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CALCENA 347</t>
+          <t>TERRERO 1390</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -6979,17 +6979,17 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>812879950</t>
+          <t>813046644</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA Y MIGRAR RED A COLUMNA ALEDAÑA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -7006,24 +7006,24 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.457348</v>
+        <v>-58.463605</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.622249</v>
+        <v>-34.612257</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>NRA-C</t>
+          <t>NRA-J</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7035,7 +7035,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>8795</t>
+          <t>8835</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7045,12 +7045,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>TERRERO 1390</t>
+          <t>GOLETA JULIET 6074</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>813046644</t>
+          <t>813046882</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -7092,24 +7092,24 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.463605</v>
+        <v>-58.465488</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.612257</v>
+        <v>-34.689546</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>NRA-J</t>
+          <t>PAV-T</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7121,7 +7121,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>8835</t>
+          <t>8845</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>GOLETA JULIET 6074</t>
+          <t>FERNANDEZ DE LA CRUZ 3999</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>813046882</t>
+          <t>813046942</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -7178,10 +7178,10 @@
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.465488</v>
+        <v>-58.454481</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.689546</v>
+        <v>-34.668745</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -7195,7 +7195,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PAV-T</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7207,7 +7207,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>8845</t>
+          <t>8862</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>FERNANDEZ DE LA CRUZ 3999</t>
+          <t>RIVERA FRUCTUOSO GENERAL 3396</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7237,12 +7237,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>813046942</t>
+          <t>813047032</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>NORMALIZAR POSTE APARENTEMENTE CAIDO</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7264,14 +7264,14 @@
         <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.454481</v>
+        <v>-58.444177</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.668745</v>
+        <v>-34.663998</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7293,7 +7293,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>8862</t>
+          <t>S00358190</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7303,12 +7303,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>RIVERA FRUCTUOSO GENERAL 3396</t>
+          <t>BACACAY 2261</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7323,12 +7323,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>813047032</t>
+          <t>813047548</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>NORMALIZAR POSTE APARENTEMENTE CAIDO</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -7350,14 +7350,14 @@
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.444177</v>
+        <v>-58.461722</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.663998</v>
+        <v>-34.625768</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7379,7 +7379,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>S00358190</t>
+          <t>8844</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -7389,12 +7389,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>BACACAY 2261</t>
+          <t>MARTINEZ CASTRO 2950</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7409,12 +7409,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>813047548</t>
+          <t>813047562</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE Y EN LO POSIBLE MIGRAR RED A COLUMNA</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -7436,10 +7436,10 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>-58.461722</v>
+        <v>-58.450186</v>
       </c>
       <c r="N82" t="n">
-        <v>-34.625768</v>
+        <v>-34.66107</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
@@ -7453,7 +7453,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7465,17 +7465,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>8844</t>
+          <t>AM00001</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>MARTINEZ CASTRO 2950</t>
+          <t>ARAUJO 2416</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7495,12 +7495,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>813047562</t>
+          <t>813304908</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y EN LO POSIBLE MIGRAR RED A COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -7522,24 +7522,24 @@
         <v>1</v>
       </c>
       <c r="M83" t="n">
-        <v>-58.450186</v>
+        <v>-58.481107</v>
       </c>
       <c r="N83" t="n">
-        <v>-34.66107</v>
+        <v>-34.659759</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-O</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7551,7 +7551,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>AM00001</t>
+          <t>8896</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7561,12 +7561,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ARAUJO 2416</t>
+          <t>QUIRNO 751</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>813304908</t>
+          <t>813304933</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -7608,51 +7608,47 @@
         <v>1</v>
       </c>
       <c r="M84" t="n">
-        <v>-58.481107</v>
+        <v>-58.46666</v>
       </c>
       <c r="N84" t="n">
-        <v>-34.659759</v>
+        <v>-34.640548</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>PAV-O</t>
-        </is>
-      </c>
-      <c r="R84" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>8896</t>
+          <t>8945</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>QUIRNO 751</t>
+          <t>DELLEPIANE, LUIS, TTE. GRAL. 5060</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7667,7 +7663,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>813304933</t>
+          <t>813350646</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -7694,10 +7690,10 @@
         <v>1</v>
       </c>
       <c r="M85" t="n">
-        <v>-58.46666</v>
+        <v>-58.474433</v>
       </c>
       <c r="N85" t="n">
-        <v>-34.640548</v>
+        <v>-34.668469</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -7711,15 +7707,19 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R85" t="inlineStr"/>
+          <t>PAV-V</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>8945</t>
+          <t>3450</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7729,12 +7729,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>DELLEPIANE, LUIS, TTE. GRAL. 5060</t>
+          <t>LAFERRERE, GREGORIO DE 3450</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>813350646</t>
+          <t>813350697</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -7776,10 +7776,10 @@
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>-58.474433</v>
+        <v>-58.467522</v>
       </c>
       <c r="N86" t="n">
-        <v>-34.668469</v>
+        <v>-34.642167</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -7793,19 +7793,15 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>PAV-V</t>
-        </is>
-      </c>
-      <c r="R86" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>3450</t>
+          <t>S00378456</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7815,7 +7811,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LAFERRERE, GREGORIO DE 3450</t>
+          <t>FRAY CAYETANO RODRIGUEZ 99</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7835,7 +7831,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>813350697</t>
+          <t>813352500</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7862,10 +7858,10 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.467522</v>
+        <v>-58.463098</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.642167</v>
+        <v>-34.627733</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -7879,10 +7875,14 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R87" t="inlineStr"/>
+          <t>PCH-H</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-28 08:42:01)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R114"/>
+  <dimension ref="A1:R115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9867,7 +9867,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">10149 </t>
+          <t xml:space="preserve">10097 </t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9877,12 +9877,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ECHEANDIA 3500</t>
+          <t>DESCALZI, NICOLAS 5404</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -9898,12 +9898,12 @@
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -9911,29 +9911,33 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L112" t="n">
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.465906</v>
+        <v>-58.463809</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.648743</v>
+        <v>-34.68275</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -9945,22 +9949,22 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>4512</t>
+          <t xml:space="preserve">10149 </t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 4512</t>
+          <t>ECHEANDIA 3500</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -9973,19 +9977,15 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>813649670</t>
-        </is>
-      </c>
+      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
-          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -9993,33 +9993,29 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K113" t="inlineStr"/>
       <c r="L113" t="n">
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.429509</v>
+        <v>-58.465906</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.615307</v>
+        <v>-34.648743</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10031,80 +10027,166 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
+          <t>4512</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>5/26/2026</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>RIVADAVIA AV. 4512</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>813649670</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>1</v>
+      </c>
+      <c r="M114" t="n">
+        <v>-58.429509</v>
+      </c>
+      <c r="N114" t="n">
+        <v>-34.615307</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>ALM-J</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
           <t>5027</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>5/26/2026</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C115" t="inlineStr">
         <is>
           <t>RIVADAVIA AV. 5012</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="D115" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr">
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
         <is>
           <t>DESPLAZAR COLUMNA TRAMBUS</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
+      <c r="I115" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="J115" t="inlineStr">
         <is>
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr">
+      <c r="K115" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L114" t="n">
-        <v>1</v>
-      </c>
-      <c r="M114" t="n">
+      <c r="L115" t="n">
+        <v>1</v>
+      </c>
+      <c r="M115" t="n">
         <v>-58.436804</v>
       </c>
-      <c r="N114" t="n">
+      <c r="N115" t="n">
         <v>-34.618542</v>
       </c>
-      <c r="O114" t="inlineStr">
+      <c r="O115" t="inlineStr">
         <is>
           <t>Boedo</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q114" t="inlineStr">
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
         <is>
           <t>ALM-F</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr">
+      <c r="R115" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 11:47:44)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R115"/>
+  <dimension ref="A1:R113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6549,7 +6549,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107591</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6605,7 +6605,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>8424</t>
+          <t>8422</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6615,12 +6615,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>BONIFACIO JOSE 2319</t>
+          <t>RIVADAVIA AV 5764</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6635,12 +6635,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>812879799</t>
+          <t>812879872</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6662,10 +6662,10 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.459955</v>
+        <v>-58.446644</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.631973</v>
+        <v>-34.622863</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PCH-I</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6691,7 +6691,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>8422</t>
+          <t>00191122</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6701,12 +6701,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV 5764</t>
+          <t>SAN PEDRITO AV 384</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>812879872</t>
+          <t>812879887</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6748,10 +6748,10 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.446644</v>
+        <v>-58.467504</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.622863</v>
+        <v>-34.635231</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -6765,7 +6765,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PCH-I</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6777,17 +6777,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>00191122</t>
+          <t xml:space="preserve">8642   </t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>3/19/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SAN PEDRITO AV 384</t>
+          <t>CALCENA 347</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -6807,17 +6807,17 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>812879887</t>
+          <t>812879950</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>DESMONTAR COLUMNA Y MIGRAR RED A COLUMNA ALEDAÑA</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -6834,10 +6834,10 @@
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.467504</v>
+        <v>-58.457348</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.635231</v>
+        <v>-34.622249</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6851,7 +6851,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>NRA-C</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -6863,17 +6863,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">8642   </t>
+          <t>8795</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CALCENA 347</t>
+          <t>TERRERO 1390</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -6893,17 +6893,17 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>812879950</t>
+          <t>813046644</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA Y MIGRAR RED A COLUMNA ALEDAÑA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -6920,24 +6920,24 @@
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.457348</v>
+        <v>-58.463605</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.622249</v>
+        <v>-34.612257</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>NRA-C</t>
+          <t>NRA-J</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6949,7 +6949,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>8795</t>
+          <t>8835</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>TERRERO 1390</t>
+          <t>GOLETA JULIET 6074</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6979,7 +6979,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>813046644</t>
+          <t>813046882</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -7006,24 +7006,24 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.463605</v>
+        <v>-58.465488</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.612257</v>
+        <v>-34.689546</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>NRA-J</t>
+          <t>PAV-T</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7035,7 +7035,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>8835</t>
+          <t>8845</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>GOLETA JULIET 6074</t>
+          <t>FERNANDEZ DE LA CRUZ 3999</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>813046882</t>
+          <t>813046942</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -7092,10 +7092,10 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.465488</v>
+        <v>-58.454481</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.689546</v>
+        <v>-34.668745</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>PAV-T</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7121,7 +7121,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>8845</t>
+          <t>8862</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>FERNANDEZ DE LA CRUZ 3999</t>
+          <t>RIVERA FRUCTUOSO GENERAL 3396</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7151,12 +7151,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>813046942</t>
+          <t>813047032</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>NORMALIZAR POSTE APARENTEMENTE CAIDO</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7178,14 +7178,14 @@
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.454481</v>
+        <v>-58.444177</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.668745</v>
+        <v>-34.663998</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7207,7 +7207,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>8862</t>
+          <t>S00358190</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>RIVERA FRUCTUOSO GENERAL 3396</t>
+          <t>BACACAY 2261</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7237,12 +7237,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>813047032</t>
+          <t>813047548</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>NORMALIZAR POSTE APARENTEMENTE CAIDO</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7264,14 +7264,14 @@
         <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.444177</v>
+        <v>-58.461722</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.663998</v>
+        <v>-34.625768</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7293,7 +7293,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>S00358190</t>
+          <t>8844</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7303,12 +7303,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>BACACAY 2261</t>
+          <t>MARTINEZ CASTRO 2950</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7323,12 +7323,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>813047548</t>
+          <t>813047562</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE Y EN LO POSIBLE MIGRAR RED A COLUMNA</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -7350,10 +7350,10 @@
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.461722</v>
+        <v>-58.450186</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.625768</v>
+        <v>-34.66107</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
@@ -7367,7 +7367,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7379,17 +7379,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>8844</t>
+          <t>AM00001</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>MARTINEZ CASTRO 2950</t>
+          <t>ARAUJO 2416</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7409,12 +7409,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>813047562</t>
+          <t>813304908</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y EN LO POSIBLE MIGRAR RED A COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -7436,24 +7436,24 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>-58.450186</v>
+        <v>-58.481107</v>
       </c>
       <c r="N82" t="n">
-        <v>-34.66107</v>
+        <v>-34.659759</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PAV-O</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7465,7 +7465,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>AM00001</t>
+          <t>8896</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -7475,12 +7475,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ARAUJO 2416</t>
+          <t>QUIRNO 751</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7495,7 +7495,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>813304908</t>
+          <t>813304933</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -7522,51 +7522,47 @@
         <v>1</v>
       </c>
       <c r="M83" t="n">
-        <v>-58.481107</v>
+        <v>-58.46666</v>
       </c>
       <c r="N83" t="n">
-        <v>-34.659759</v>
+        <v>-34.640548</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>PAV-O</t>
-        </is>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>8896</t>
+          <t>8945</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>QUIRNO 751</t>
+          <t>DELLEPIANE, LUIS, TTE. GRAL. 5060</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7581,7 +7577,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>813304933</t>
+          <t>813350646</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -7608,10 +7604,10 @@
         <v>1</v>
       </c>
       <c r="M84" t="n">
-        <v>-58.46666</v>
+        <v>-58.474433</v>
       </c>
       <c r="N84" t="n">
-        <v>-34.640548</v>
+        <v>-34.668469</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -7625,15 +7621,19 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R84" t="inlineStr"/>
+          <t>PAV-V</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>8945</t>
+          <t>3450</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7643,12 +7643,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>DELLEPIANE, LUIS, TTE. GRAL. 5060</t>
+          <t>LAFERRERE, GREGORIO DE 3450</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>813350646</t>
+          <t>813350697</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -7690,10 +7690,10 @@
         <v>1</v>
       </c>
       <c r="M85" t="n">
-        <v>-58.474433</v>
+        <v>-58.467522</v>
       </c>
       <c r="N85" t="n">
-        <v>-34.668469</v>
+        <v>-34.642167</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -7707,19 +7707,15 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>PAV-V</t>
-        </is>
-      </c>
-      <c r="R85" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>3450</t>
+          <t>S00378456</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7729,7 +7725,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>LAFERRERE, GREGORIO DE 3450</t>
+          <t>FRAY CAYETANO RODRIGUEZ 99</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7749,7 +7745,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>813350697</t>
+          <t>813352500</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -7776,10 +7772,10 @@
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>-58.467522</v>
+        <v>-58.463098</v>
       </c>
       <c r="N86" t="n">
-        <v>-34.642167</v>
+        <v>-34.627733</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -7793,15 +7789,19 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R86" t="inlineStr"/>
+          <t>PCH-H</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>S00378456</t>
+          <t>S00334047</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7811,12 +7811,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>FRAY CAYETANO RODRIGUEZ 99</t>
+          <t>SAN JOSE DE CALASANZ 755</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>813352500</t>
+          <t>813352503</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7858,10 +7858,10 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.463098</v>
+        <v>-58.437351</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.627733</v>
+        <v>-34.627956</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -7875,7 +7875,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PCH-C</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7887,22 +7887,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>S00334047</t>
+          <t>S00472131</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>4/29/2026</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SAN JOSE DE CALASANZ 755</t>
+          <t>LAFUENTE 3014</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7917,7 +7917,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>813352503</t>
+          <t>813353227</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -7944,14 +7944,14 @@
         <v>1</v>
       </c>
       <c r="M88" t="n">
-        <v>-58.437351</v>
+        <v>-58.440449</v>
       </c>
       <c r="N88" t="n">
-        <v>-34.627956</v>
+        <v>-34.661351</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>PCH-C</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -7973,22 +7973,22 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>S00472131</t>
+          <t>S00305777</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>4/29/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>LAFUENTE 3014</t>
+          <t>FALCON, RAMON L.,CNEL. 2353</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>813353227</t>
+          <t>813631421</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -8030,14 +8030,14 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.440449</v>
+        <v>-58.46138</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.661351</v>
+        <v>-34.629774</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -8047,7 +8047,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8059,17 +8059,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>S00305777</t>
+          <t>S00061238</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>TERRADA 440</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8089,7 +8089,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>813631421</t>
+          <t>814108554</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -8116,10 +8116,10 @@
         <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>-58.46138</v>
+        <v>-58.469993</v>
       </c>
       <c r="N90" t="n">
-        <v>-34.629774</v>
+        <v>-34.626657</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -8133,7 +8133,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8145,7 +8145,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>S00061238</t>
+          <t>S00434076</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>TERRADA 440</t>
+          <t>SENILLOSA 1113</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8173,7 +8173,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>814108577</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8198,10 +8202,10 @@
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>-58.469993</v>
+        <v>-58.427622</v>
       </c>
       <c r="N91" t="n">
-        <v>-34.626657</v>
+        <v>-34.629853</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -8215,7 +8219,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PPT-P</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -8227,7 +8231,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>S00434076</t>
+          <t>S00430171</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -8237,7 +8241,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SENILLOSA 1113</t>
+          <t>VARELA AV. 760</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8255,7 +8259,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>814108580</t>
+        </is>
+      </c>
       <c r="H92" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8280,10 +8288,10 @@
         <v>1</v>
       </c>
       <c r="M92" t="n">
-        <v>-58.427622</v>
+        <v>-58.4599</v>
       </c>
       <c r="N92" t="n">
-        <v>-34.629853</v>
+        <v>-34.638193</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -8297,7 +8305,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>PPT-P</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8309,7 +8317,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>S00430171</t>
+          <t>S00363093</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -8319,7 +8327,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>VARELA AV. 760</t>
+          <t>BACACAY 665</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8337,7 +8345,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>814108583</t>
+        </is>
+      </c>
       <c r="H93" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8362,14 +8374,14 @@
         <v>1</v>
       </c>
       <c r="M93" t="n">
-        <v>-58.4599</v>
+        <v>-58.439489</v>
       </c>
       <c r="N93" t="n">
-        <v>-34.638193</v>
+        <v>-34.616916</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
@@ -8379,7 +8391,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8391,7 +8403,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>S00363093</t>
+          <t>S00457605</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -8401,7 +8413,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>BACACAY 665</t>
+          <t>FALCON, RAMON L.,CNEL. 2363</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8419,7 +8431,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>814108590</t>
+        </is>
+      </c>
       <c r="H94" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8444,14 +8460,14 @@
         <v>1</v>
       </c>
       <c r="M94" t="n">
-        <v>-58.439489</v>
+        <v>-58.46164</v>
       </c>
       <c r="N94" t="n">
-        <v>-34.616916</v>
+        <v>-34.629853</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
@@ -8461,7 +8477,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8473,7 +8489,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>S00457605</t>
+          <t>S00459651</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -8483,7 +8499,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2363</t>
+          <t>CULPINA 89</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8501,7 +8517,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>814108592</t>
+        </is>
+      </c>
       <c r="H95" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8526,10 +8546,10 @@
         <v>1</v>
       </c>
       <c r="M95" t="n">
-        <v>-58.46164</v>
+        <v>-58.466433</v>
       </c>
       <c r="N95" t="n">
-        <v>-34.629853</v>
+        <v>-34.631185</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -8543,7 +8563,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -8555,7 +8575,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>S00459651</t>
+          <t xml:space="preserve">8557 </t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -8565,12 +8585,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>CULPINA 89</t>
+          <t>JANER, ANA MARIA 3424</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -8586,12 +8606,12 @@
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE MADERA</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -8608,10 +8628,10 @@
         <v>1</v>
       </c>
       <c r="M96" t="n">
-        <v>-58.466433</v>
+        <v>-58.450189</v>
       </c>
       <c r="N96" t="n">
-        <v>-34.631185</v>
+        <v>-34.659997</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -8625,7 +8645,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8637,7 +8657,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">8557 </t>
+          <t xml:space="preserve">900009974510 </t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -8647,12 +8667,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>JANER, ANA MARIA 3424</t>
+          <t>FALCON, RAMON L.,CNEL. 2819</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -8668,12 +8688,12 @@
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE MADERA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -8690,10 +8710,10 @@
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>-58.450189</v>
+        <v>-58.467888</v>
       </c>
       <c r="N97" t="n">
-        <v>-34.659997</v>
+        <v>-34.631753</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -8707,7 +8727,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8719,7 +8739,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">9208 </t>
+          <t xml:space="preserve">9206 </t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -8729,7 +8749,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2819</t>
+          <t>BONORINO, ESTEBAN, CNEL. AV. 2945</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8750,12 +8770,12 @@
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t xml:space="preserve">DESMONTAR POSTE </t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -8772,14 +8792,14 @@
         <v>1</v>
       </c>
       <c r="M98" t="n">
-        <v>-58.467888</v>
+        <v>-58.431721</v>
       </c>
       <c r="N98" t="n">
-        <v>-34.631753</v>
+        <v>-34.655142</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -8789,7 +8809,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PPT-J</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -8801,7 +8821,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009974510 </t>
+          <t xml:space="preserve">9209 </t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8811,7 +8831,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2819</t>
+          <t>ARANGUREN, JUAN F., DR. 2429</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8854,10 +8874,10 @@
         <v>1</v>
       </c>
       <c r="M99" t="n">
-        <v>-58.467888</v>
+        <v>-58.465714</v>
       </c>
       <c r="N99" t="n">
-        <v>-34.631753</v>
+        <v>-34.62319</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -8871,7 +8891,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8883,7 +8903,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">9206 </t>
+          <t xml:space="preserve">9921 </t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8893,7 +8913,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>BONORINO, ESTEBAN, CNEL. AV. 2945</t>
+          <t>AVELLANEDA AV. 1881</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8914,12 +8934,12 @@
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t xml:space="preserve">DESMONTAR POSTE </t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -8936,14 +8956,14 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>-58.431721</v>
+        <v>-58.457457</v>
       </c>
       <c r="N100" t="n">
-        <v>-34.655142</v>
+        <v>-34.621606</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
@@ -8953,7 +8973,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>PPT-J</t>
+          <t>NRA-C</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -8965,17 +8985,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">9209 </t>
+          <t>S00535834</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 2429</t>
+          <t>FALCON, RAMON L.,CNEL. 2355</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8993,7 +9013,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>814107932</t>
+        </is>
+      </c>
       <c r="H101" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9018,10 +9042,10 @@
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>-58.465714</v>
+        <v>-58.461432</v>
       </c>
       <c r="N101" t="n">
-        <v>-34.62319</v>
+        <v>-34.62979</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -9035,7 +9059,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9047,17 +9071,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">9921 </t>
+          <t>S00535884</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>AVELLANEDA AV. 1881</t>
+          <t>FALCON, RAMON L.,CNEL. 2327</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -9075,7 +9099,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>814107988</t>
+        </is>
+      </c>
       <c r="H102" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9100,10 +9128,10 @@
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>-58.457457</v>
+        <v>-58.46114</v>
       </c>
       <c r="N102" t="n">
-        <v>-34.621606</v>
+        <v>-34.629702</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -9117,7 +9145,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>NRA-C</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9129,7 +9157,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>S00535834</t>
+          <t xml:space="preserve">8884 </t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -9139,7 +9167,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2355</t>
+          <t>PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -9157,7 +9185,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>814108016</t>
+        </is>
+      </c>
       <c r="H103" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9182,10 +9214,10 @@
         <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>-58.461432</v>
+        <v>-58.46026</v>
       </c>
       <c r="N103" t="n">
-        <v>-34.62979</v>
+        <v>-34.640706</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -9199,7 +9231,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9211,7 +9243,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>S00535884</t>
+          <t xml:space="preserve">8889 </t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -9221,12 +9253,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2327</t>
+          <t>ARAOZ ALFARO, GREGORIO, DR 270</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -9239,7 +9271,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>814108018</t>
+        </is>
+      </c>
       <c r="H104" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9264,14 +9300,14 @@
         <v>1</v>
       </c>
       <c r="M104" t="n">
-        <v>-58.46114</v>
+        <v>-58.434739</v>
       </c>
       <c r="N104" t="n">
-        <v>-34.629702</v>
+        <v>-34.615027</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
@@ -9281,7 +9317,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>ALM-H</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9293,7 +9329,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">8884 </t>
+          <t xml:space="preserve">8908 </t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -9303,12 +9339,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>PRIMERA JUNTA 2899</t>
+          <t>RIGLOS 549</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -9334,7 +9370,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -9346,10 +9382,10 @@
         <v>1</v>
       </c>
       <c r="M105" t="n">
-        <v>-58.46026</v>
+        <v>-58.436278</v>
       </c>
       <c r="N105" t="n">
-        <v>-34.640706</v>
+        <v>-34.625163</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -9363,7 +9399,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PCH-B</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9375,7 +9411,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">8889 </t>
+          <t xml:space="preserve">8934 </t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -9385,12 +9421,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ARAOZ ALFARO, GREGORIO, DR 270</t>
+          <t>GRANADEROS 482</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -9403,7 +9439,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>814108021</t>
+        </is>
+      </c>
       <c r="H106" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9428,14 +9468,14 @@
         <v>1</v>
       </c>
       <c r="M106" t="n">
-        <v>-58.434739</v>
+        <v>-58.461709</v>
       </c>
       <c r="N106" t="n">
-        <v>-34.615027</v>
+        <v>-34.62211</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
@@ -9445,7 +9485,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>ALM-H</t>
+          <t>NRA-D</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9457,7 +9497,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">8908 </t>
+          <t xml:space="preserve">8993 </t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9467,7 +9507,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>RIGLOS 549</t>
+          <t>BERTRES 339</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9485,7 +9525,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>814108059</t>
+        </is>
+      </c>
       <c r="H107" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9498,7 +9542,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -9510,10 +9554,10 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.436278</v>
+        <v>-58.439032</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.625163</v>
+        <v>-34.622296</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -9527,7 +9571,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>PCH-B</t>
+          <t>PCH-K</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9539,7 +9583,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">8934 </t>
+          <t>S01401412</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9549,7 +9593,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>GRANADEROS 482</t>
+          <t>LAFUENTE 299</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9570,12 +9614,12 @@
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -9592,10 +9636,10 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.461709</v>
+        <v>-58.46677</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.62211</v>
+        <v>-34.633968</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -9609,7 +9653,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>NRA-D</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -9621,7 +9665,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">8993 </t>
+          <t xml:space="preserve">10096 </t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9631,12 +9675,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>BERTRES 339</t>
+          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -9662,7 +9706,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -9674,10 +9718,10 @@
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.439032</v>
+        <v>-58.460409</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.622296</v>
+        <v>-34.684521</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -9691,7 +9735,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>PCH-K</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -9703,7 +9747,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>S01401412</t>
+          <t xml:space="preserve">10097 </t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9713,12 +9757,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>LAFUENTE 299</t>
+          <t>DESCALZI, NICOLAS 5404</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -9734,7 +9778,7 @@
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -9756,10 +9800,10 @@
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.46677</v>
+        <v>-58.463809</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.633968</v>
+        <v>-34.68275</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -9773,7 +9817,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9785,7 +9829,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">10096 </t>
+          <t xml:space="preserve">10149 </t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9795,12 +9839,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
+          <t>ECHEANDIA 3500</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -9816,46 +9860,42 @@
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
-        </is>
-      </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr"/>
       <c r="L111" t="n">
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.460409</v>
+        <v>-58.465906</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.684521</v>
+        <v>-34.648743</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -9867,22 +9907,22 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">10097 </t>
+          <t>4512</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>DESCALZI, NICOLAS 5404</t>
+          <t>RIVADAVIA AV. 4512</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -9895,15 +9935,19 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>813649670</t>
+        </is>
+      </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -9920,10 +9964,10 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.463809</v>
+        <v>-58.429509</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.68275</v>
+        <v>-34.615307</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -9937,7 +9981,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -9949,22 +9993,22 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">10149 </t>
+          <t>5027</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ECHEANDIA 3500</t>
+          <t>RIVADAVIA AV. 5012</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -9977,15 +10021,19 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>814107858</t>
+        </is>
+      </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -9993,200 +10041,36 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L113" t="n">
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.465906</v>
+        <v>-58.436804</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.648743</v>
+        <v>-34.618542</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>4512</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>5/26/2026</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>RIVADAVIA AV. 4512</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>813649670</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K114" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L114" t="n">
-        <v>1</v>
-      </c>
-      <c r="M114" t="n">
-        <v>-58.429509</v>
-      </c>
-      <c r="N114" t="n">
-        <v>-34.615307</v>
-      </c>
-      <c r="O114" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P114" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q114" t="inlineStr">
-        <is>
-          <t>ALM-J</t>
-        </is>
-      </c>
-      <c r="R114" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>5027</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>5/26/2026</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>RIVADAVIA AV. 5012</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>DESPLAZAR COLUMNA TRAMBUS</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J115" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K115" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L115" t="n">
-        <v>1</v>
-      </c>
-      <c r="M115" t="n">
-        <v>-58.436804</v>
-      </c>
-      <c r="N115" t="n">
-        <v>-34.618542</v>
-      </c>
-      <c r="O115" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P115" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q115" t="inlineStr">
-        <is>
-          <t>ALM-F</t>
-        </is>
-      </c>
-      <c r="R115" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 13:05:42)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -8685,7 +8685,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>814109222</t>
+        </is>
+      </c>
       <c r="H97" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8849,7 +8853,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>814109458</t>
+        </is>
+      </c>
       <c r="H99" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8931,7 +8939,11 @@
           <t>Optical Power</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>814109746</t>
+        </is>
+      </c>
       <c r="H100" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-02 15:37:25)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R113"/>
+  <dimension ref="A1:R126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,17 +439,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>798897458</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>798897458</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>801768138</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>801768138</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -699,17 +699,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>799485362</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>799485362</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -785,17 +785,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>802367713</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>802367713</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -867,17 +867,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>803607520</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>803607520</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -953,17 +953,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>803607699</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>803607699</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1039,17 +1039,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>804309801</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>804309801</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804876047</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>804876047</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1211,17 +1211,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>804903810</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>804903810</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1297,17 +1297,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>806926697</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>806926697</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1383,17 +1383,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807044216</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>807044216</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1469,17 +1469,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t xml:space="preserve">ICD30261461 </t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICD30261461 </t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1555,17 +1555,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>807129347</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>807129347</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808150511</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>808150511</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1727,17 +1727,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808615951</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>808615951</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1813,17 +1813,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808615948</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>808615948</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1899,17 +1899,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>03534653</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>03534653</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1985,17 +1985,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809065913</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>809065913</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2071,17 +2071,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>ICD30508311</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2157,17 +2157,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>ICD30593982</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2243,17 +2243,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809309598</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>809309598</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2329,17 +2329,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>ICD30709119</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ICD30709119</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2415,17 +2415,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809837504</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>809837504</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2501,17 +2501,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809972807</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>809972807</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2587,17 +2587,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810015422</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>810015422</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2673,17 +2673,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>ICD31463420</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>ICD31463420</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2759,17 +2759,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2845,17 +2845,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810259135</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>810259135</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2931,17 +2931,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810333113</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>810333113</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3017,17 +3017,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810371027</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>810371027</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3103,17 +3103,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810454541</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>810454541</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3189,17 +3189,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>01230744</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>01230744</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3275,17 +3275,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810526265</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>810526265</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810526272</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>810526272</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3447,17 +3447,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810712730</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>810712730</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3533,17 +3533,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810712887</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>810712887</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3619,17 +3619,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810734112</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>810734112</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3705,17 +3705,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>TLC</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>TLC</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3791,17 +3791,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810804380</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810804380</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3877,17 +3877,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810820553</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>810820553</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3963,17 +3963,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810862736</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>810862736</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4049,17 +4049,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198653</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>811198653</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4135,17 +4135,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198753</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>811198753</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4221,17 +4221,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198692</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>811198692</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4307,17 +4307,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811238719</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>811238719</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4393,17 +4393,17 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811238674</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>811238674</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4479,17 +4479,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811299459</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>811299459</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4565,17 +4565,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811299453</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>811299453</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4651,17 +4651,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811453890</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>811453890</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4737,17 +4737,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454448</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>811454448</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4823,17 +4823,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454435</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>811454435</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4909,17 +4909,17 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811497993</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>811497993</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4995,17 +4995,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626780</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>811626780</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -5081,17 +5081,17 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626771</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>811626771</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5167,17 +5167,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626802</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>811626802</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5253,17 +5253,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626968</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>811626968</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5339,17 +5339,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627028</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>811627028</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5425,17 +5425,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5511,17 +5511,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812503538</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>812503538</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5597,17 +5597,17 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627115</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>811627115</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5683,17 +5683,17 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440072</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>812440072</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5769,17 +5769,17 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440077</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>812440077</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5855,17 +5855,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440563</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>812440563</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5941,17 +5941,17 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440368</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>812440368</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -6027,17 +6027,17 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812439923</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>812439923</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -6113,17 +6113,17 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440314</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>812440314</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -6199,17 +6199,17 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440276</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>812440276</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -6285,17 +6285,17 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812503658</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>812503658</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -6371,17 +6371,17 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -6457,17 +6457,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6539,17 +6539,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107591</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>814107591</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6625,17 +6625,17 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879872</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>812879872</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -6711,17 +6711,17 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879887</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>812879887</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6797,17 +6797,17 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879950</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>812879950</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -6883,17 +6883,17 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046644</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>813046644</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -6969,17 +6969,17 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046882</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>813046882</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -7055,17 +7055,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046942</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>813046942</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -7141,17 +7141,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047032</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>813047032</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -7227,17 +7227,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047548</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>813047548</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -7313,17 +7313,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047562</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>813047562</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -7399,17 +7399,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304908</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>813304908</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -7485,17 +7485,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304933</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>813304933</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -7567,17 +7567,17 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350646</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>813350646</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -7653,17 +7653,17 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350697</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>813350697</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -7735,17 +7735,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352500</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>813352500</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -7821,17 +7821,17 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352503</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>813352503</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7907,17 +7907,17 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813353227</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>813353227</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -7993,17 +7993,17 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631421</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>813631421</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -8079,17 +8079,17 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108554</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>814108554</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -8165,17 +8165,17 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108577</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>814108577</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -8251,17 +8251,17 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108580</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>814108580</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -8337,17 +8337,17 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108583</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>814108583</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -8423,17 +8423,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108590</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>814108590</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -8509,17 +8509,17 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108592</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>814108592</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -8593,17 +8593,17 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
       <c r="H96" t="inlineStr">
         <is>
           <t>DESMONTAR POSTE MADERA</t>
@@ -8677,17 +8677,17 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109222</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>814109222</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -8761,17 +8761,17 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
       <c r="H98" t="inlineStr">
         <is>
           <t xml:space="preserve">DESMONTAR POSTE </t>
@@ -8845,17 +8845,17 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109458</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>814109458</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -8931,17 +8931,17 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109746</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>814109746</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -9017,17 +9017,17 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107932</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>814107932</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -9103,17 +9103,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107988</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>814107988</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -9189,17 +9189,17 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108016</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>814108016</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -9275,17 +9275,17 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108018</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>814108018</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -9359,17 +9359,17 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
       <c r="H105" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9443,17 +9443,17 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108021</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>814108021</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -9529,22 +9529,22 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108059</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>814108059</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>cambiar columna</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -9613,17 +9613,17 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
       <c r="H108" t="inlineStr">
         <is>
           <t>DESMONTAR POSTE</t>
@@ -9695,17 +9695,17 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
       <c r="H109" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9777,17 +9777,17 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
       <c r="H110" t="inlineStr">
         <is>
           <t>DESMONTAR COLUMNA</t>
@@ -9861,15 +9861,19 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111816</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
       <c r="H111" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -9877,7 +9881,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -9939,17 +9943,17 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813649670</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>813649670</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -10025,17 +10029,17 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107858</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>814107858</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -10083,6 +10087,1120 @@
         </is>
       </c>
       <c r="R113" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>-778</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>ARANGUREN, JUAN F., DR. 2429</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>814125561</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>1</v>
+      </c>
+      <c r="M114" t="n">
+        <v>-58.465714</v>
+      </c>
+      <c r="N114" t="n">
+        <v>-34.62319</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>NRA-L</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>-779</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>ARANGUREN, JUAN F., DR. 462</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>814125564</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>base muy corroida</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>1</v>
+      </c>
+      <c r="M115" t="n">
+        <v>-58.437431</v>
+      </c>
+      <c r="N115" t="n">
+        <v>-34.612405</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>ALM-I</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>-780</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ARENGREEN 1478</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>814125576</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>1</v>
+      </c>
+      <c r="M116" t="n">
+        <v>-58.452378</v>
+      </c>
+      <c r="N116" t="n">
+        <v>-34.614705</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>NRA-B</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>-786</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>PERON, EVA AV. 2580</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>814125585</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L117" t="n">
+        <v>1</v>
+      </c>
+      <c r="M117" t="n">
+        <v>-58.456386</v>
+      </c>
+      <c r="N117" t="n">
+        <v>-34.640935</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>PPT-N</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>-792</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>BOGOTA 2356</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L118" t="n">
+        <v>1</v>
+      </c>
+      <c r="M118" t="n">
+        <v>-58.46356</v>
+      </c>
+      <c r="N118" t="n">
+        <v>-34.6251</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>NRA-E</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>-798</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>RAMIREZ, CEFERINO, COMODORO 5496</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L119" t="n">
+        <v>1</v>
+      </c>
+      <c r="M119" t="n">
+        <v>-58.461526</v>
+      </c>
+      <c r="N119" t="n">
+        <v>-34.684686</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>-799</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>CULPINA 541</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>1</v>
+      </c>
+      <c r="M120" t="n">
+        <v>-58.46417</v>
+      </c>
+      <c r="N120" t="n">
+        <v>-34.636302</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>-804</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>MORENO, PERITO AV. 2294</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>814125655</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>base corroida y doblada</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L121" t="n">
+        <v>1</v>
+      </c>
+      <c r="M121" t="n">
+        <v>-58.441867</v>
+      </c>
+      <c r="N121" t="n">
+        <v>-34.650886</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>PPT-A</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>-819</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>RIGLOS 553</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>1</v>
+      </c>
+      <c r="M122" t="n">
+        <v>-58.436277</v>
+      </c>
+      <c r="N122" t="n">
+        <v>-34.625202</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>PCH-B</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>-824</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SENILLOSA 823</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>814125712</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L123" t="n">
+        <v>1</v>
+      </c>
+      <c r="M123" t="n">
+        <v>-58.428429</v>
+      </c>
+      <c r="N123" t="n">
+        <v>-34.626246</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>PCH-B</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>-826</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>TERRERO 318</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>814125722</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>1</v>
+      </c>
+      <c r="M124" t="n">
+        <v>-58.457752</v>
+      </c>
+      <c r="N124" t="n">
+        <v>-34.622812</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>NRA-C</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>-827</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>TRES ARROYOS 1055</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L125" t="n">
+        <v>1</v>
+      </c>
+      <c r="M125" t="n">
+        <v>-58.455033</v>
+      </c>
+      <c r="N125" t="n">
+        <v>-34.606193</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>NRA-I</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>-829</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>VIRASORO, VALENTIN 995</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>814125726</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L126" t="n">
+        <v>1</v>
+      </c>
+      <c r="M126" t="n">
+        <v>-58.443206</v>
+      </c>
+      <c r="N126" t="n">
+        <v>-34.608689</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>ALM-I</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-02 17:11:30)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R126"/>
+  <dimension ref="A1:R125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9509,7 +9509,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">8993 </t>
+          <t>S01401412</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9519,19 +9519,15 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>BERTRES 339</t>
+          <t>LAFUENTE 299</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>814108059</t>
-        </is>
-      </c>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -9544,12 +9540,12 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>cambiar columna</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -9566,10 +9562,10 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.439032</v>
+        <v>-58.46677</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.622296</v>
+        <v>-34.633968</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -9583,7 +9579,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>PCH-K</t>
+          <t>PCH-F</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9595,7 +9591,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>S01401412</t>
+          <t xml:space="preserve">10096 </t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9605,12 +9601,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>LAFUENTE 299</t>
+          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -9626,17 +9622,17 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -9648,10 +9644,10 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.46677</v>
+        <v>-58.460409</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.633968</v>
+        <v>-34.684521</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -9665,7 +9661,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -9677,7 +9673,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">10096 </t>
+          <t xml:space="preserve">10097 </t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9687,12 +9683,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
+          <t>DESCALZI, NICOLAS 5404</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -9708,17 +9704,17 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -9730,10 +9726,10 @@
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.460409</v>
+        <v>-58.463809</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.684521</v>
+        <v>-34.68275</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -9759,7 +9755,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">10097 </t>
+          <t xml:space="preserve">10149 </t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9769,15 +9765,19 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>DESCALZI, NICOLAS 5404</t>
+          <t>ECHEANDIA 3500</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>814111816</t>
+        </is>
+      </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -9790,12 +9790,12 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -9803,33 +9803,29 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K110" t="inlineStr"/>
       <c r="L110" t="n">
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.463809</v>
+        <v>-58.465906</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.68275</v>
+        <v>-34.648743</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9841,27 +9837,27 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">10149 </t>
+          <t>4512</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ECHEANDIA 3500</t>
+          <t>RIVADAVIA AV. 4512</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>814111816</t>
+          <t>813649670</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -9876,7 +9872,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -9889,29 +9885,33 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L111" t="n">
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.465906</v>
+        <v>-58.429509</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.648743</v>
+        <v>-34.615307</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -9923,7 +9923,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>4512</t>
+          <t>5027</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9933,7 +9933,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 4512</t>
+          <t>RIVADAVIA AV. 5012</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>813649670</t>
+          <t>814107858</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -9980,10 +9980,10 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.429509</v>
+        <v>-58.436804</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.615307</v>
+        <v>-34.618542</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -9997,7 +9997,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10009,27 +10009,27 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>5027</t>
+          <t>-778</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 5012</t>
+          <t>ARANGUREN, JUAN F., DR. 2429</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>814107858</t>
+          <t>814125561</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -10066,10 +10066,10 @@
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.436804</v>
+        <v>-58.465714</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.618542</v>
+        <v>-34.62319</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -10083,7 +10083,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10095,7 +10095,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>-778</t>
+          <t>-779</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -10105,17 +10105,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 2429</t>
+          <t>ARANGUREN, JUAN F., DR. 462</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>814125561</t>
+          <t>814125564</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -10130,7 +10130,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base muy corroida</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -10152,14 +10152,14 @@
         <v>1</v>
       </c>
       <c r="M114" t="n">
-        <v>-58.465714</v>
+        <v>-58.437431</v>
       </c>
       <c r="N114" t="n">
-        <v>-34.62319</v>
+        <v>-34.612405</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
@@ -10169,7 +10169,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>ALM-I</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10181,7 +10181,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>-779</t>
+          <t>-780</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -10191,7 +10191,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 462</t>
+          <t>ARENGREEN 1478</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -10201,7 +10201,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>814125564</t>
+          <t>814125576</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -10216,7 +10216,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>base muy corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -10238,14 +10238,14 @@
         <v>1</v>
       </c>
       <c r="M115" t="n">
-        <v>-58.437431</v>
+        <v>-58.452378</v>
       </c>
       <c r="N115" t="n">
-        <v>-34.612405</v>
+        <v>-34.614705</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -10255,7 +10255,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>ALM-I</t>
+          <t>NRA-B</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10267,7 +10267,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>-780</t>
+          <t>-786</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -10277,17 +10277,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ARENGREEN 1478</t>
+          <t>PERON, EVA AV. 2580</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>814125576</t>
+          <t>814125585</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -10324,10 +10324,10 @@
         <v>1</v>
       </c>
       <c r="M116" t="n">
-        <v>-58.452378</v>
+        <v>-58.456386</v>
       </c>
       <c r="N116" t="n">
-        <v>-34.614705</v>
+        <v>-34.640935</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -10341,7 +10341,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>NRA-B</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10353,7 +10353,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>-786</t>
+          <t>-792</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -10363,7 +10363,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>PERON, EVA AV. 2580</t>
+          <t>BOGOTA 2356</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -10373,7 +10373,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>814125585</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -10398,7 +10398,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -10410,10 +10410,10 @@
         <v>1</v>
       </c>
       <c r="M117" t="n">
-        <v>-58.456386</v>
+        <v>-58.46356</v>
       </c>
       <c r="N117" t="n">
-        <v>-34.640935</v>
+        <v>-34.6251</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -10427,7 +10427,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10439,7 +10439,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>-792</t>
+          <t>-798</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -10449,12 +10449,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>BOGOTA 2356</t>
+          <t>RAMIREZ, CEFERINO, COMODORO 5496</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -10484,7 +10484,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -10496,10 +10496,10 @@
         <v>1</v>
       </c>
       <c r="M118" t="n">
-        <v>-58.46356</v>
+        <v>-58.461526</v>
       </c>
       <c r="N118" t="n">
-        <v>-34.6251</v>
+        <v>-34.684686</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -10513,7 +10513,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>NRA-E</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -10525,7 +10525,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>-798</t>
+          <t>-799</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -10535,12 +10535,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>RAMIREZ, CEFERINO, COMODORO 5496</t>
+          <t>CULPINA 541</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -10582,10 +10582,10 @@
         <v>1</v>
       </c>
       <c r="M119" t="n">
-        <v>-58.461526</v>
+        <v>-58.46417</v>
       </c>
       <c r="N119" t="n">
-        <v>-34.684686</v>
+        <v>-34.636302</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -10599,19 +10599,15 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>PAV-U</t>
-        </is>
-      </c>
-      <c r="R119" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>-799</t>
+          <t>-804</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -10621,7 +10617,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>CULPINA 541</t>
+          <t>MORENO, PERITO AV. 2294</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -10631,7 +10627,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125655</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -10646,7 +10642,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base corroida y doblada</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -10656,7 +10652,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -10668,10 +10664,10 @@
         <v>1</v>
       </c>
       <c r="M120" t="n">
-        <v>-58.46417</v>
+        <v>-58.441867</v>
       </c>
       <c r="N120" t="n">
-        <v>-34.636302</v>
+        <v>-34.650886</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -10685,15 +10681,19 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R120" t="inlineStr"/>
+          <t>PPT-A</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>-804</t>
+          <t>-819</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -10703,17 +10703,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>MORENO, PERITO AV. 2294</t>
+          <t>RIGLOS 553</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>814125655</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -10728,7 +10728,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>base corroida y doblada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -10738,7 +10738,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -10750,10 +10750,10 @@
         <v>1</v>
       </c>
       <c r="M121" t="n">
-        <v>-58.441867</v>
+        <v>-58.436277</v>
       </c>
       <c r="N121" t="n">
-        <v>-34.650886</v>
+        <v>-34.625202</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -10767,7 +10767,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>PPT-A</t>
+          <t>PCH-B</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -10779,7 +10779,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>-819</t>
+          <t>-824</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -10789,7 +10789,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>RIGLOS 553</t>
+          <t>SENILLOSA 823</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125712</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -10836,10 +10836,10 @@
         <v>1</v>
       </c>
       <c r="M122" t="n">
-        <v>-58.436277</v>
+        <v>-58.428429</v>
       </c>
       <c r="N122" t="n">
-        <v>-34.625202</v>
+        <v>-34.626246</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -10865,7 +10865,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>-824</t>
+          <t>-826</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -10875,17 +10875,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>SENILLOSA 823</t>
+          <t>TERRERO 318</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>814125712</t>
+          <t>814125722</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -10922,10 +10922,10 @@
         <v>1</v>
       </c>
       <c r="M123" t="n">
-        <v>-58.428429</v>
+        <v>-58.457752</v>
       </c>
       <c r="N123" t="n">
-        <v>-34.626246</v>
+        <v>-34.622812</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -10939,7 +10939,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>PCH-B</t>
+          <t>NRA-C</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -10951,7 +10951,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>-826</t>
+          <t>-827</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -10961,17 +10961,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>TERRERO 318</t>
+          <t>TRES ARROYOS 1055</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>814125722</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -11008,24 +11008,24 @@
         <v>1</v>
       </c>
       <c r="M124" t="n">
-        <v>-58.457752</v>
+        <v>-58.455033</v>
       </c>
       <c r="N124" t="n">
-        <v>-34.622812</v>
+        <v>-34.606193</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>NRA-C</t>
+          <t>NRA-I</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11037,7 +11037,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>-827</t>
+          <t>-829</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -11047,7 +11047,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>TRES ARROYOS 1055</t>
+          <t>VIRASORO, VALENTIN 995</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -11057,7 +11057,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125726</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -11094,113 +11094,27 @@
         <v>1</v>
       </c>
       <c r="M125" t="n">
-        <v>-58.455033</v>
+        <v>-58.443206</v>
       </c>
       <c r="N125" t="n">
-        <v>-34.606193</v>
+        <v>-34.608689</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>NRA-I</t>
+          <t>ALM-I</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>-829</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>VIRASORO, VALENTIN 995</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>814125726</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L126" t="n">
-        <v>1</v>
-      </c>
-      <c r="M126" t="n">
-        <v>-58.443206</v>
-      </c>
-      <c r="N126" t="n">
-        <v>-34.608689</v>
-      </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P126" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>ALM-I</t>
-        </is>
-      </c>
-      <c r="R126" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-03 11:57:58)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -5425,7 +5425,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Pendiente ADM OT GxC</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -6361,7 +6361,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicolás Descalzi 5582 </t>
+          <t>DESCALZI, NICOLAS 5582</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>Pendiente ADM OT GxC</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-08 12:33:48)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R120"/>
+  <dimension ref="A1:R118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7461,17 +7461,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>S00305777</t>
+          <t>S00061238</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2353</t>
+          <t>TERRADA 440</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7486,7 +7486,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>813631421</t>
+          <t>814108554</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -7518,10 +7518,10 @@
         <v>1</v>
       </c>
       <c r="M83" t="n">
-        <v>-58.46138</v>
+        <v>-58.469993</v>
       </c>
       <c r="N83" t="n">
-        <v>-34.629774</v>
+        <v>-34.626657</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -7535,7 +7535,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>S00061238</t>
+          <t>S00434076</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>TERRADA 440</t>
+          <t>SENILLOSA 1113</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>814108554</t>
+          <t>814108577</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -7604,10 +7604,10 @@
         <v>1</v>
       </c>
       <c r="M84" t="n">
-        <v>-58.469993</v>
+        <v>-58.427622</v>
       </c>
       <c r="N84" t="n">
-        <v>-34.626657</v>
+        <v>-34.629853</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>PPT-P</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -7633,7 +7633,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>S00434076</t>
+          <t>S00430171</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7643,7 +7643,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>SENILLOSA 1113</t>
+          <t>VARELA AV. 760</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>814108577</t>
+          <t>814108580</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -7690,10 +7690,10 @@
         <v>1</v>
       </c>
       <c r="M85" t="n">
-        <v>-58.427622</v>
+        <v>-58.4599</v>
       </c>
       <c r="N85" t="n">
-        <v>-34.629853</v>
+        <v>-34.638193</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -7707,7 +7707,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>PPT-P</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7719,7 +7719,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>S00430171</t>
+          <t>S00363093</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>VARELA AV. 760</t>
+          <t>BACACAY 665</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>814108580</t>
+          <t>814108583</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -7776,14 +7776,14 @@
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>-58.4599</v>
+        <v>-58.439489</v>
       </c>
       <c r="N86" t="n">
-        <v>-34.638193</v>
+        <v>-34.616916</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -7793,7 +7793,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -7805,7 +7805,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>S00363093</t>
+          <t>S00457605</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>BACACAY 665</t>
+          <t>FALCON, RAMON L.,CNEL. 2363</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>814108583</t>
+          <t>814108590</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -7862,14 +7862,14 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.439489</v>
+        <v>-58.46164</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.616916</v>
+        <v>-34.629853</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -7879,7 +7879,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7891,7 +7891,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>S00457605</t>
+          <t>S00459651</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2363</t>
+          <t>CULPINA 89</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>814108590</t>
+          <t>814108592</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -7948,10 +7948,10 @@
         <v>1</v>
       </c>
       <c r="M88" t="n">
-        <v>-58.46164</v>
+        <v>-58.466433</v>
       </c>
       <c r="N88" t="n">
-        <v>-34.629853</v>
+        <v>-34.631185</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -7977,7 +7977,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>S00459651</t>
+          <t xml:space="preserve">8557 </t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -7987,12 +7987,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CULPINA 89</t>
+          <t>JANER, ANA MARIA 3424</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -8000,11 +8000,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>814108592</t>
-        </is>
-      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -8012,12 +8008,12 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE MADERA</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -8034,10 +8030,10 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.466433</v>
+        <v>-58.450189</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.631185</v>
+        <v>-34.659997</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -8051,7 +8047,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PPT-I</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8063,7 +8059,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">8557 </t>
+          <t xml:space="preserve">900009974510 </t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -8073,12 +8069,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>JANER, ANA MARIA 3424</t>
+          <t>FALCON, RAMON L.,CNEL. 2819</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -8086,7 +8082,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>814109222</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -8094,12 +8094,12 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE MADERA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -8116,10 +8116,10 @@
         <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>-58.450189</v>
+        <v>-58.467888</v>
       </c>
       <c r="N90" t="n">
-        <v>-34.659997</v>
+        <v>-34.631753</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -8133,7 +8133,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>PPT-I</t>
+          <t>PCH-H</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8145,7 +8145,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009974510 </t>
+          <t xml:space="preserve">9206 </t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2819</t>
+          <t>BONORINO, ESTEBAN, CNEL. AV. 2945</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8168,11 +8168,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>814109222</t>
-        </is>
-      </c>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -8180,12 +8176,12 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t xml:space="preserve">DESMONTAR POSTE </t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -8202,14 +8198,14 @@
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>-58.467888</v>
+        <v>-58.431721</v>
       </c>
       <c r="N91" t="n">
-        <v>-34.631753</v>
+        <v>-34.655142</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -8219,7 +8215,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>PCH-H</t>
+          <t>PPT-J</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -8231,7 +8227,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">9206 </t>
+          <t xml:space="preserve">9209 </t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -8241,7 +8237,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>BONORINO, ESTEBAN, CNEL. AV. 2945</t>
+          <t>ARANGUREN, JUAN F., DR. 2429</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8254,7 +8250,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>814109458</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -8262,12 +8262,12 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t xml:space="preserve">DESMONTAR POSTE </t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -8284,14 +8284,14 @@
         <v>1</v>
       </c>
       <c r="M92" t="n">
-        <v>-58.431721</v>
+        <v>-58.465714</v>
       </c>
       <c r="N92" t="n">
-        <v>-34.655142</v>
+        <v>-34.62319</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>PPT-J</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8313,7 +8313,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">9209 </t>
+          <t xml:space="preserve">9921 </t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -8323,7 +8323,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 2429</t>
+          <t>AVELLANEDA AV. 1881</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8338,7 +8338,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>814109458</t>
+          <t>814109746</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -8370,10 +8370,10 @@
         <v>1</v>
       </c>
       <c r="M93" t="n">
-        <v>-58.465714</v>
+        <v>-58.457457</v>
       </c>
       <c r="N93" t="n">
-        <v>-34.62319</v>
+        <v>-34.621606</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -8387,7 +8387,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>NRA-C</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8399,17 +8399,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">9921 </t>
+          <t>S00535834</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>AVELLANEDA AV. 1881</t>
+          <t>FALCON, RAMON L.,CNEL. 2355</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8424,7 +8424,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>814109746</t>
+          <t>814107932</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -8456,10 +8456,10 @@
         <v>1</v>
       </c>
       <c r="M94" t="n">
-        <v>-58.457457</v>
+        <v>-58.461432</v>
       </c>
       <c r="N94" t="n">
-        <v>-34.621606</v>
+        <v>-34.62979</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>NRA-C</t>
+          <t>PCH-J</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8485,7 +8485,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>S00535834</t>
+          <t>S00535884</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2355</t>
+          <t>FALCON, RAMON L.,CNEL. 2327</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8510,7 +8510,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>814107932</t>
+          <t>814107988</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -8542,10 +8542,10 @@
         <v>1</v>
       </c>
       <c r="M95" t="n">
-        <v>-58.461432</v>
+        <v>-58.46114</v>
       </c>
       <c r="N95" t="n">
-        <v>-34.62979</v>
+        <v>-34.629702</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -8571,7 +8571,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>S00535884</t>
+          <t xml:space="preserve">8884 </t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -8581,7 +8581,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 2327</t>
+          <t>PRIMERA JUNTA 2899</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8596,7 +8596,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>814107988</t>
+          <t>814108016</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -8628,10 +8628,10 @@
         <v>1</v>
       </c>
       <c r="M96" t="n">
-        <v>-58.46114</v>
+        <v>-58.46026</v>
       </c>
       <c r="N96" t="n">
-        <v>-34.629702</v>
+        <v>-34.640706</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -8645,7 +8645,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>PCH-J</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8657,7 +8657,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">8884 </t>
+          <t xml:space="preserve">8889 </t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -8667,12 +8667,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>PRIMERA JUNTA 2899</t>
+          <t>ARAOZ ALFARO, GREGORIO, DR 270</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>814108016</t>
+          <t>814108018</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -8714,14 +8714,14 @@
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>-58.46026</v>
+        <v>-58.434739</v>
       </c>
       <c r="N97" t="n">
-        <v>-34.640706</v>
+        <v>-34.615027</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>ALM-H</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8743,7 +8743,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">8889 </t>
+          <t xml:space="preserve">8908 </t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -8753,7 +8753,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ARAOZ ALFARO, GREGORIO, DR 270</t>
+          <t>RIGLOS 549</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8766,11 +8766,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>814108018</t>
-        </is>
-      </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -8788,7 +8784,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -8800,14 +8796,14 @@
         <v>1</v>
       </c>
       <c r="M98" t="n">
-        <v>-58.434739</v>
+        <v>-58.436278</v>
       </c>
       <c r="N98" t="n">
-        <v>-34.615027</v>
+        <v>-34.625163</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -8817,7 +8813,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>ALM-H</t>
+          <t>PCH-B</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -8829,7 +8825,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">8908 </t>
+          <t xml:space="preserve">8934 </t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8839,12 +8835,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>RIGLOS 549</t>
+          <t>GRANADEROS 482</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -8852,7 +8848,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>814108021</t>
+        </is>
+      </c>
       <c r="G99" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -8870,7 +8870,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -8882,10 +8882,10 @@
         <v>1</v>
       </c>
       <c r="M99" t="n">
-        <v>-58.436278</v>
+        <v>-58.461709</v>
       </c>
       <c r="N99" t="n">
-        <v>-34.625163</v>
+        <v>-34.62211</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -8899,7 +8899,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>PCH-B</t>
+          <t>NRA-D</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8911,7 +8911,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">8934 </t>
+          <t xml:space="preserve">10096 </t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8921,12 +8921,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>GRANADEROS 482</t>
+          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -8934,11 +8934,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>814108021</t>
-        </is>
-      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -8956,7 +8952,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -8968,10 +8964,10 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>-58.461709</v>
+        <v>-58.460409</v>
       </c>
       <c r="N100" t="n">
-        <v>-34.62211</v>
+        <v>-34.684521</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -8985,7 +8981,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>NRA-D</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -8997,7 +8993,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>S01401412</t>
+          <t xml:space="preserve">10097 </t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -9007,12 +9003,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LAFUENTE 299</t>
+          <t>DESCALZI, NICOLAS 5404</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -9028,7 +9024,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -9050,10 +9046,10 @@
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>-58.46677</v>
+        <v>-58.463809</v>
       </c>
       <c r="N101" t="n">
-        <v>-34.633968</v>
+        <v>-34.68275</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -9067,7 +9063,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>PCH-F</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9079,7 +9075,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">10096 </t>
+          <t xml:space="preserve">10149 </t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -9089,12 +9085,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
+          <t>ECHEANDIA 3500</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -9102,7 +9098,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>814111816</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -9110,7 +9110,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -9120,36 +9120,32 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
-        </is>
-      </c>
-      <c r="K102" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr"/>
       <c r="L102" t="n">
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>-58.460409</v>
+        <v>-58.465906</v>
       </c>
       <c r="N102" t="n">
-        <v>-34.684521</v>
+        <v>-34.648743</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9161,22 +9157,22 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">10097 </t>
+          <t>4512</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>DESCALZI, NICOLAS 5404</t>
+          <t>RIVADAVIA AV. 4512</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -9184,7 +9180,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>813649670</t>
+        </is>
+      </c>
       <c r="G103" t="inlineStr">
         <is>
           <t>Optical Power</t>
@@ -9192,12 +9192,12 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -9214,10 +9214,10 @@
         <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>-58.463809</v>
+        <v>-58.429509</v>
       </c>
       <c r="N103" t="n">
-        <v>-34.68275</v>
+        <v>-34.615307</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>ALM-J</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9243,22 +9243,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">10149 </t>
+          <t>5027</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ECHEANDIA 3500</t>
+          <t>RIVADAVIA AV. 5012</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -9268,7 +9268,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>814111816</t>
+          <t>814107858</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -9291,29 +9291,33 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L104" t="n">
         <v>1</v>
       </c>
       <c r="M104" t="n">
-        <v>-58.465906</v>
+        <v>-58.436804</v>
       </c>
       <c r="N104" t="n">
-        <v>-34.648743</v>
+        <v>-34.618542</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9325,22 +9329,22 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>4512</t>
+          <t>-778</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 4512</t>
+          <t>ARANGUREN, JUAN F., DR. 2429</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -9350,7 +9354,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>813649670</t>
+          <t>814125561</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -9360,7 +9364,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>REALIZAR DESPLAZAMIENTO TRAMBUS</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -9382,10 +9386,10 @@
         <v>1</v>
       </c>
       <c r="M105" t="n">
-        <v>-58.429509</v>
+        <v>-58.465714</v>
       </c>
       <c r="N105" t="n">
-        <v>-34.615307</v>
+        <v>-34.62319</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -9399,7 +9403,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>ALM-J</t>
+          <t>NRA-L</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9411,17 +9415,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>5027</t>
+          <t>-779</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 5012</t>
+          <t>ARANGUREN, JUAN F., DR. 462</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9436,7 +9440,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>814107858</t>
+          <t>814125564</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -9446,7 +9450,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base muy corroida</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -9468,14 +9472,14 @@
         <v>1</v>
       </c>
       <c r="M106" t="n">
-        <v>-58.436804</v>
+        <v>-58.437431</v>
       </c>
       <c r="N106" t="n">
-        <v>-34.618542</v>
+        <v>-34.612405</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
@@ -9485,7 +9489,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>ALM-I</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9497,7 +9501,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>-778</t>
+          <t>-780</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9507,12 +9511,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 2429</t>
+          <t>ARENGREEN 1478</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -9522,7 +9526,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>814125561</t>
+          <t>814125576</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -9554,10 +9558,10 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.465714</v>
+        <v>-58.452378</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.62319</v>
+        <v>-34.614705</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -9571,7 +9575,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>NRA-L</t>
+          <t>NRA-B</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9583,7 +9587,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>-779</t>
+          <t>-786</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9593,12 +9597,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 462</t>
+          <t>PERON, EVA AV. 2580</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -9608,7 +9612,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>814125564</t>
+          <t>814125585</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -9618,7 +9622,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>base muy corroida</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -9640,14 +9644,14 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.437431</v>
+        <v>-58.456386</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.612405</v>
+        <v>-34.640935</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
@@ -9657,7 +9661,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>ALM-I</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -9669,7 +9673,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>-780</t>
+          <t>-792</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9679,12 +9683,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ARENGREEN 1478</t>
+          <t>BOGOTA 2356</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -9694,7 +9698,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>814125576</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -9714,7 +9718,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -9726,10 +9730,10 @@
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.452378</v>
+        <v>-58.46356</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.614705</v>
+        <v>-34.6251</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -9743,7 +9747,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>NRA-B</t>
+          <t>NRA-E</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -9755,7 +9759,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>-786</t>
+          <t>-798</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9765,12 +9769,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>PERON, EVA AV. 2580</t>
+          <t>RAMIREZ, CEFERINO, COMODORO 5496</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -9780,7 +9784,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>814125585</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -9812,10 +9816,10 @@
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.456386</v>
+        <v>-58.461526</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.640935</v>
+        <v>-34.684686</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -9829,7 +9833,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9841,7 +9845,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>-792</t>
+          <t>-799</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9851,7 +9855,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>BOGOTA 2356</t>
+          <t>CULPINA 541</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9898,10 +9902,10 @@
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.46356</v>
+        <v>-58.46417</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.6251</v>
+        <v>-34.636302</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -9915,19 +9919,15 @@
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>NRA-E</t>
-        </is>
-      </c>
-      <c r="R111" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-N</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>-798</t>
+          <t>-804</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9937,12 +9937,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>RAMIREZ, CEFERINO, COMODORO 5496</t>
+          <t>MORENO, PERITO AV. 2294</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -9952,7 +9952,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125655</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base corroida y doblada</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -9984,10 +9984,10 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.461526</v>
+        <v>-58.441867</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.684686</v>
+        <v>-34.650886</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -10001,7 +10001,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PPT-A</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10013,7 +10013,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>-799</t>
+          <t>-819</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -10023,12 +10023,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>CULPINA 541</t>
+          <t>RIGLOS 553</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -10070,10 +10070,10 @@
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.46417</v>
+        <v>-58.436277</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.636302</v>
+        <v>-34.625202</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -10087,15 +10087,19 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>PCH-N</t>
-        </is>
-      </c>
-      <c r="R113" t="inlineStr"/>
+          <t>PCH-B</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>-804</t>
+          <t>-824</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -10105,12 +10109,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>MORENO, PERITO AV. 2294</t>
+          <t>SENILLOSA 823</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -10120,7 +10124,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>814125655</t>
+          <t>814125712</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -10130,7 +10134,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>base corroida y doblada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -10152,10 +10156,10 @@
         <v>1</v>
       </c>
       <c r="M114" t="n">
-        <v>-58.441867</v>
+        <v>-58.428429</v>
       </c>
       <c r="N114" t="n">
-        <v>-34.650886</v>
+        <v>-34.626246</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -10169,7 +10173,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>PPT-A</t>
+          <t>PCH-B</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10181,7 +10185,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>-819</t>
+          <t>-826</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -10191,12 +10195,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>RIGLOS 553</t>
+          <t>TERRERO 318</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -10206,7 +10210,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125722</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -10226,7 +10230,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -10238,10 +10242,10 @@
         <v>1</v>
       </c>
       <c r="M115" t="n">
-        <v>-58.436277</v>
+        <v>-58.457752</v>
       </c>
       <c r="N115" t="n">
-        <v>-34.625202</v>
+        <v>-34.622812</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -10255,7 +10259,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>PCH-B</t>
+          <t>NRA-C</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10267,7 +10271,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>-824</t>
+          <t>-827</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -10277,7 +10281,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>SENILLOSA 823</t>
+          <t>TRES ARROYOS 1055</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -10292,7 +10296,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>814125712</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -10312,7 +10316,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -10324,24 +10328,24 @@
         <v>1</v>
       </c>
       <c r="M116" t="n">
-        <v>-58.428429</v>
+        <v>-58.455033</v>
       </c>
       <c r="N116" t="n">
-        <v>-34.626246</v>
+        <v>-34.606193</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>PCH-B</t>
+          <t>NRA-I</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10353,7 +10357,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>-826</t>
+          <t>-829</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -10363,12 +10367,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>TERRERO 318</t>
+          <t>VIRASORO, VALENTIN 995</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -10378,7 +10382,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>814125722</t>
+          <t>814125726</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -10410,14 +10414,14 @@
         <v>1</v>
       </c>
       <c r="M117" t="n">
-        <v>-58.457752</v>
+        <v>-58.443206</v>
       </c>
       <c r="N117" t="n">
-        <v>-34.622812</v>
+        <v>-34.608689</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -10427,7 +10431,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>NRA-C</t>
+          <t>ALM-I</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10439,22 +10443,22 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>-827</t>
+          <t>1406PN</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>6/2/2026</t>
+          <t>6/5/2026</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>TRES ARROYOS 1055</t>
+          <t>CASTAÑARES 1406</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -10464,7 +10468,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814231011</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -10474,7 +10478,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -10484,7 +10488,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -10493,202 +10497,30 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M118" t="n">
-        <v>-58.455033</v>
+        <v>-58.438075</v>
       </c>
       <c r="N118" t="n">
-        <v>-34.606193</v>
+        <v>-34.637952</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>NRA-I</t>
+          <t>PPT-S</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>-829</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>VIRASORO, VALENTIN 995</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>814125726</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>base corroida</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J119" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L119" t="n">
-        <v>1</v>
-      </c>
-      <c r="M119" t="n">
-        <v>-58.443206</v>
-      </c>
-      <c r="N119" t="n">
-        <v>-34.608689</v>
-      </c>
-      <c r="O119" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P119" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q119" t="inlineStr">
-        <is>
-          <t>ALM-I</t>
-        </is>
-      </c>
-      <c r="R119" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>1406PN</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>6/5/2026</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>CASTAÑARES 1406</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>814231011</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L120" t="n">
-        <v>0</v>
-      </c>
-      <c r="M120" t="n">
-        <v>-58.438075</v>
-      </c>
-      <c r="N120" t="n">
-        <v>-34.637952</v>
-      </c>
-      <c r="O120" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P120" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q120" t="inlineStr">
-        <is>
-          <t>PPT-S</t>
-        </is>
-      </c>
-      <c r="R120" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-10 15:52:50)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R105"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9408,6 +9408,88 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>0011111</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>6/10/2026</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ALVAREZ THOMAS AV 3190</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L106" t="n">
+        <v>1</v>
+      </c>
+      <c r="M106" t="n">
+        <v>-58.483183</v>
+      </c>
+      <c r="N106" t="n">
+        <v>-34.571653</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>ATH-E</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-11 11:02:51)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R106"/>
+  <dimension ref="A1:R108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9490,6 +9490,178 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>814443578</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>6/11/2026</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>AV LA PLATA 510</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>814443578</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA TRAMBUS</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" t="n">
+        <v>-58.427928</v>
+      </c>
+      <c r="N107" t="n">
+        <v>-34.620873</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>ALM-B</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>814443589</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>6/11/2026</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>AV LA PLATA 1105</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>814443589</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA TRAMBUS</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" t="n">
+        <v>-58.426519</v>
+      </c>
+      <c r="N108" t="n">
+        <v>-34.628511</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>PPT-P</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>